<commit_message>
Connect product dimensions to shipping quotes
</commit_message>
<xml_diff>
--- a/public/templates/reach-projector-product-import.xlsx
+++ b/public/templates/reach-projector-product-import.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R4fb2e531aad949a5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Specifications" sheetId="2" r:id="R0c68aa6d18a04313"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="3" r:id="R33faa2e2ceb14b6b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R4db6ecbf6ad04fb2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Specifications" sheetId="2" r:id="R8d33d1b4d36d4ea3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="3" r:id="R88b8b34c0c2d495a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -455,11 +455,15 @@
     <x:col min="20" max="20" width="18" hidden="0" customWidth="1"/>
     <x:col min="21" max="21" width="18" hidden="0" customWidth="1"/>
     <x:col min="22" max="22" width="18" hidden="0" customWidth="1"/>
-    <x:col min="23" max="23" width="42" hidden="0" customWidth="1"/>
-    <x:col min="24" max="24" width="42" hidden="0" customWidth="1"/>
-    <x:col min="25" max="25" width="36" hidden="0" customWidth="1"/>
-    <x:col min="26" max="26" width="36" hidden="0" customWidth="1"/>
-    <x:col min="27" max="27" width="18" hidden="0" customWidth="1"/>
+    <x:col min="23" max="23" width="18" hidden="0" customWidth="1"/>
+    <x:col min="24" max="24" width="18" hidden="0" customWidth="1"/>
+    <x:col min="25" max="25" width="18" hidden="0" customWidth="1"/>
+    <x:col min="26" max="26" width="18" hidden="0" customWidth="1"/>
+    <x:col min="27" max="27" width="42" hidden="0" customWidth="1"/>
+    <x:col min="28" max="28" width="42" hidden="0" customWidth="1"/>
+    <x:col min="29" max="29" width="36" hidden="0" customWidth="1"/>
+    <x:col min="30" max="30" width="36" hidden="0" customWidth="1"/>
+    <x:col min="31" max="31" width="18" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
@@ -518,30 +522,42 @@
         <x:v>Country of Origin</x:v>
       </x:c>
       <x:c r="S1" s="13" t="str">
-        <x:v>Product Dimensions</x:v>
+        <x:v>Product Length (cm)</x:v>
       </x:c>
       <x:c r="T1" s="13" t="str">
-        <x:v>Package Dimensions</x:v>
+        <x:v>Product Width (cm)</x:v>
       </x:c>
       <x:c r="U1" s="13" t="str">
+        <x:v>Product Height (cm)</x:v>
+      </x:c>
+      <x:c r="V1" s="13" t="str">
+        <x:v>Package Length (cm)</x:v>
+      </x:c>
+      <x:c r="W1" s="13" t="str">
+        <x:v>Package Width (cm)</x:v>
+      </x:c>
+      <x:c r="X1" s="13" t="str">
+        <x:v>Package Height (cm)</x:v>
+      </x:c>
+      <x:c r="Y1" s="13" t="str">
         <x:v>Net Weight (kg)</x:v>
       </x:c>
-      <x:c r="V1" s="13" t="str">
+      <x:c r="Z1" s="13" t="str">
         <x:v>Gross Weight (kg)</x:v>
       </x:c>
-      <x:c r="W1" s="13" t="str">
+      <x:c r="AA1" s="13" t="str">
         <x:v>Short Description</x:v>
       </x:c>
-      <x:c r="X1" s="13" t="str">
+      <x:c r="AB1" s="13" t="str">
         <x:v>Full Description</x:v>
       </x:c>
-      <x:c r="Y1" s="13" t="str">
+      <x:c r="AC1" s="13" t="str">
         <x:v>SEO Title</x:v>
       </x:c>
-      <x:c r="Z1" s="13" t="str">
+      <x:c r="AD1" s="13" t="str">
         <x:v>Meta Description</x:v>
       </x:c>
-      <x:c r="AA1" s="13" t="str">
+      <x:c r="AE1" s="13" t="str">
         <x:v>Product Status</x:v>
       </x:c>
     </x:row>
@@ -600,31 +616,43 @@
       <x:c r="R2" s="14" t="str">
         <x:v>China</x:v>
       </x:c>
-      <x:c r="S2" s="14" t="str">
-        <x:v>250 x 200 x 100 mm</x:v>
-      </x:c>
-      <x:c r="T2" s="14" t="str">
-        <x:v>350 x 300 x 200 mm</x:v>
+      <x:c r="S2" s="17" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="T2" s="17" t="n">
+        <x:v>20</x:v>
       </x:c>
       <x:c r="U2" s="17" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="V2" s="17" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="W2" s="17" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="X2" s="17" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="Y2" s="17" t="n">
         <x:v>3.2</x:v>
       </x:c>
-      <x:c r="V2" s="17" t="n">
+      <x:c r="Z2" s="17" t="n">
         <x:v>4.5</x:v>
       </x:c>
-      <x:c r="W2" s="14" t="str">
+      <x:c r="AA2" s="14" t="str">
         <x:v>Replace this example with verified product facts.</x:v>
       </x:c>
-      <x:c r="X2" s="14" t="str">
+      <x:c r="AB2" s="14" t="str">
         <x:v>Delete this row before importing.</x:v>
       </x:c>
-      <x:c r="Y2" s="14" t="str">
+      <x:c r="AC2" s="14" t="str">
         <x:v>Example Projector | Reach Projector</x:v>
       </x:c>
-      <x:c r="Z2" s="14" t="str">
+      <x:c r="AD2" s="14" t="str">
         <x:v>Replace with a factual product description.</x:v>
       </x:c>
-      <x:c r="AA2" s="14" t="str">
+      <x:c r="AE2" s="14" t="str">
         <x:v>draft</x:v>
       </x:c>
     </x:row>
@@ -647,15 +675,19 @@
       <x:c r="P3" s="18"/>
       <x:c r="Q3" s="18"/>
       <x:c r="R3" s="18"/>
-      <x:c r="S3" s="18"/>
-      <x:c r="T3" s="18"/>
+      <x:c r="S3" s="21"/>
+      <x:c r="T3" s="21"/>
       <x:c r="U3" s="21"/>
       <x:c r="V3" s="21"/>
-      <x:c r="W3" s="18"/>
-      <x:c r="X3" s="18"/>
-      <x:c r="Y3" s="18"/>
-      <x:c r="Z3" s="18"/>
+      <x:c r="W3" s="21"/>
+      <x:c r="X3" s="21"/>
+      <x:c r="Y3" s="21"/>
+      <x:c r="Z3" s="21"/>
       <x:c r="AA3" s="18"/>
+      <x:c r="AB3" s="18"/>
+      <x:c r="AC3" s="18"/>
+      <x:c r="AD3" s="18"/>
+      <x:c r="AE3" s="18"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="18"/>
@@ -676,15 +708,19 @@
       <x:c r="P4" s="18"/>
       <x:c r="Q4" s="18"/>
       <x:c r="R4" s="18"/>
-      <x:c r="S4" s="18"/>
-      <x:c r="T4" s="18"/>
+      <x:c r="S4" s="21"/>
+      <x:c r="T4" s="21"/>
       <x:c r="U4" s="21"/>
       <x:c r="V4" s="21"/>
-      <x:c r="W4" s="18"/>
-      <x:c r="X4" s="18"/>
-      <x:c r="Y4" s="18"/>
-      <x:c r="Z4" s="18"/>
+      <x:c r="W4" s="21"/>
+      <x:c r="X4" s="21"/>
+      <x:c r="Y4" s="21"/>
+      <x:c r="Z4" s="21"/>
       <x:c r="AA4" s="18"/>
+      <x:c r="AB4" s="18"/>
+      <x:c r="AC4" s="18"/>
+      <x:c r="AD4" s="18"/>
+      <x:c r="AE4" s="18"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="18"/>
@@ -705,15 +741,19 @@
       <x:c r="P5" s="18"/>
       <x:c r="Q5" s="18"/>
       <x:c r="R5" s="18"/>
-      <x:c r="S5" s="18"/>
-      <x:c r="T5" s="18"/>
+      <x:c r="S5" s="21"/>
+      <x:c r="T5" s="21"/>
       <x:c r="U5" s="21"/>
       <x:c r="V5" s="21"/>
-      <x:c r="W5" s="18"/>
-      <x:c r="X5" s="18"/>
-      <x:c r="Y5" s="18"/>
-      <x:c r="Z5" s="18"/>
+      <x:c r="W5" s="21"/>
+      <x:c r="X5" s="21"/>
+      <x:c r="Y5" s="21"/>
+      <x:c r="Z5" s="21"/>
       <x:c r="AA5" s="18"/>
+      <x:c r="AB5" s="18"/>
+      <x:c r="AC5" s="18"/>
+      <x:c r="AD5" s="18"/>
+      <x:c r="AE5" s="18"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="18"/>
@@ -734,15 +774,19 @@
       <x:c r="P6" s="18"/>
       <x:c r="Q6" s="18"/>
       <x:c r="R6" s="18"/>
-      <x:c r="S6" s="18"/>
-      <x:c r="T6" s="18"/>
+      <x:c r="S6" s="21"/>
+      <x:c r="T6" s="21"/>
       <x:c r="U6" s="21"/>
       <x:c r="V6" s="21"/>
-      <x:c r="W6" s="18"/>
-      <x:c r="X6" s="18"/>
-      <x:c r="Y6" s="18"/>
-      <x:c r="Z6" s="18"/>
+      <x:c r="W6" s="21"/>
+      <x:c r="X6" s="21"/>
+      <x:c r="Y6" s="21"/>
+      <x:c r="Z6" s="21"/>
       <x:c r="AA6" s="18"/>
+      <x:c r="AB6" s="18"/>
+      <x:c r="AC6" s="18"/>
+      <x:c r="AD6" s="18"/>
+      <x:c r="AE6" s="18"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="18"/>
@@ -763,15 +807,19 @@
       <x:c r="P7" s="18"/>
       <x:c r="Q7" s="18"/>
       <x:c r="R7" s="18"/>
-      <x:c r="S7" s="18"/>
-      <x:c r="T7" s="18"/>
+      <x:c r="S7" s="21"/>
+      <x:c r="T7" s="21"/>
       <x:c r="U7" s="21"/>
       <x:c r="V7" s="21"/>
-      <x:c r="W7" s="18"/>
-      <x:c r="X7" s="18"/>
-      <x:c r="Y7" s="18"/>
-      <x:c r="Z7" s="18"/>
+      <x:c r="W7" s="21"/>
+      <x:c r="X7" s="21"/>
+      <x:c r="Y7" s="21"/>
+      <x:c r="Z7" s="21"/>
       <x:c r="AA7" s="18"/>
+      <x:c r="AB7" s="18"/>
+      <x:c r="AC7" s="18"/>
+      <x:c r="AD7" s="18"/>
+      <x:c r="AE7" s="18"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="18"/>
@@ -792,15 +840,19 @@
       <x:c r="P8" s="18"/>
       <x:c r="Q8" s="18"/>
       <x:c r="R8" s="18"/>
-      <x:c r="S8" s="18"/>
-      <x:c r="T8" s="18"/>
+      <x:c r="S8" s="21"/>
+      <x:c r="T8" s="21"/>
       <x:c r="U8" s="21"/>
       <x:c r="V8" s="21"/>
-      <x:c r="W8" s="18"/>
-      <x:c r="X8" s="18"/>
-      <x:c r="Y8" s="18"/>
-      <x:c r="Z8" s="18"/>
+      <x:c r="W8" s="21"/>
+      <x:c r="X8" s="21"/>
+      <x:c r="Y8" s="21"/>
+      <x:c r="Z8" s="21"/>
       <x:c r="AA8" s="18"/>
+      <x:c r="AB8" s="18"/>
+      <x:c r="AC8" s="18"/>
+      <x:c r="AD8" s="18"/>
+      <x:c r="AE8" s="18"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="18"/>
@@ -821,15 +873,19 @@
       <x:c r="P9" s="18"/>
       <x:c r="Q9" s="18"/>
       <x:c r="R9" s="18"/>
-      <x:c r="S9" s="18"/>
-      <x:c r="T9" s="18"/>
+      <x:c r="S9" s="21"/>
+      <x:c r="T9" s="21"/>
       <x:c r="U9" s="21"/>
       <x:c r="V9" s="21"/>
-      <x:c r="W9" s="18"/>
-      <x:c r="X9" s="18"/>
-      <x:c r="Y9" s="18"/>
-      <x:c r="Z9" s="18"/>
+      <x:c r="W9" s="21"/>
+      <x:c r="X9" s="21"/>
+      <x:c r="Y9" s="21"/>
+      <x:c r="Z9" s="21"/>
       <x:c r="AA9" s="18"/>
+      <x:c r="AB9" s="18"/>
+      <x:c r="AC9" s="18"/>
+      <x:c r="AD9" s="18"/>
+      <x:c r="AE9" s="18"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="18"/>
@@ -850,15 +906,19 @@
       <x:c r="P10" s="18"/>
       <x:c r="Q10" s="18"/>
       <x:c r="R10" s="18"/>
-      <x:c r="S10" s="18"/>
-      <x:c r="T10" s="18"/>
+      <x:c r="S10" s="21"/>
+      <x:c r="T10" s="21"/>
       <x:c r="U10" s="21"/>
       <x:c r="V10" s="21"/>
-      <x:c r="W10" s="18"/>
-      <x:c r="X10" s="18"/>
-      <x:c r="Y10" s="18"/>
-      <x:c r="Z10" s="18"/>
+      <x:c r="W10" s="21"/>
+      <x:c r="X10" s="21"/>
+      <x:c r="Y10" s="21"/>
+      <x:c r="Z10" s="21"/>
       <x:c r="AA10" s="18"/>
+      <x:c r="AB10" s="18"/>
+      <x:c r="AC10" s="18"/>
+      <x:c r="AD10" s="18"/>
+      <x:c r="AE10" s="18"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="18"/>
@@ -879,15 +939,19 @@
       <x:c r="P11" s="18"/>
       <x:c r="Q11" s="18"/>
       <x:c r="R11" s="18"/>
-      <x:c r="S11" s="18"/>
-      <x:c r="T11" s="18"/>
+      <x:c r="S11" s="21"/>
+      <x:c r="T11" s="21"/>
       <x:c r="U11" s="21"/>
       <x:c r="V11" s="21"/>
-      <x:c r="W11" s="18"/>
-      <x:c r="X11" s="18"/>
-      <x:c r="Y11" s="18"/>
-      <x:c r="Z11" s="18"/>
+      <x:c r="W11" s="21"/>
+      <x:c r="X11" s="21"/>
+      <x:c r="Y11" s="21"/>
+      <x:c r="Z11" s="21"/>
       <x:c r="AA11" s="18"/>
+      <x:c r="AB11" s="18"/>
+      <x:c r="AC11" s="18"/>
+      <x:c r="AD11" s="18"/>
+      <x:c r="AE11" s="18"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="18"/>
@@ -908,15 +972,19 @@
       <x:c r="P12" s="18"/>
       <x:c r="Q12" s="18"/>
       <x:c r="R12" s="18"/>
-      <x:c r="S12" s="18"/>
-      <x:c r="T12" s="18"/>
+      <x:c r="S12" s="21"/>
+      <x:c r="T12" s="21"/>
       <x:c r="U12" s="21"/>
       <x:c r="V12" s="21"/>
-      <x:c r="W12" s="18"/>
-      <x:c r="X12" s="18"/>
-      <x:c r="Y12" s="18"/>
-      <x:c r="Z12" s="18"/>
+      <x:c r="W12" s="21"/>
+      <x:c r="X12" s="21"/>
+      <x:c r="Y12" s="21"/>
+      <x:c r="Z12" s="21"/>
       <x:c r="AA12" s="18"/>
+      <x:c r="AB12" s="18"/>
+      <x:c r="AC12" s="18"/>
+      <x:c r="AD12" s="18"/>
+      <x:c r="AE12" s="18"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="18"/>
@@ -937,15 +1005,19 @@
       <x:c r="P13" s="18"/>
       <x:c r="Q13" s="18"/>
       <x:c r="R13" s="18"/>
-      <x:c r="S13" s="18"/>
-      <x:c r="T13" s="18"/>
+      <x:c r="S13" s="21"/>
+      <x:c r="T13" s="21"/>
       <x:c r="U13" s="21"/>
       <x:c r="V13" s="21"/>
-      <x:c r="W13" s="18"/>
-      <x:c r="X13" s="18"/>
-      <x:c r="Y13" s="18"/>
-      <x:c r="Z13" s="18"/>
+      <x:c r="W13" s="21"/>
+      <x:c r="X13" s="21"/>
+      <x:c r="Y13" s="21"/>
+      <x:c r="Z13" s="21"/>
       <x:c r="AA13" s="18"/>
+      <x:c r="AB13" s="18"/>
+      <x:c r="AC13" s="18"/>
+      <x:c r="AD13" s="18"/>
+      <x:c r="AE13" s="18"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="18"/>
@@ -966,15 +1038,19 @@
       <x:c r="P14" s="18"/>
       <x:c r="Q14" s="18"/>
       <x:c r="R14" s="18"/>
-      <x:c r="S14" s="18"/>
-      <x:c r="T14" s="18"/>
+      <x:c r="S14" s="21"/>
+      <x:c r="T14" s="21"/>
       <x:c r="U14" s="21"/>
       <x:c r="V14" s="21"/>
-      <x:c r="W14" s="18"/>
-      <x:c r="X14" s="18"/>
-      <x:c r="Y14" s="18"/>
-      <x:c r="Z14" s="18"/>
+      <x:c r="W14" s="21"/>
+      <x:c r="X14" s="21"/>
+      <x:c r="Y14" s="21"/>
+      <x:c r="Z14" s="21"/>
       <x:c r="AA14" s="18"/>
+      <x:c r="AB14" s="18"/>
+      <x:c r="AC14" s="18"/>
+      <x:c r="AD14" s="18"/>
+      <x:c r="AE14" s="18"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="18"/>
@@ -995,15 +1071,19 @@
       <x:c r="P15" s="18"/>
       <x:c r="Q15" s="18"/>
       <x:c r="R15" s="18"/>
-      <x:c r="S15" s="18"/>
-      <x:c r="T15" s="18"/>
+      <x:c r="S15" s="21"/>
+      <x:c r="T15" s="21"/>
       <x:c r="U15" s="21"/>
       <x:c r="V15" s="21"/>
-      <x:c r="W15" s="18"/>
-      <x:c r="X15" s="18"/>
-      <x:c r="Y15" s="18"/>
-      <x:c r="Z15" s="18"/>
+      <x:c r="W15" s="21"/>
+      <x:c r="X15" s="21"/>
+      <x:c r="Y15" s="21"/>
+      <x:c r="Z15" s="21"/>
       <x:c r="AA15" s="18"/>
+      <x:c r="AB15" s="18"/>
+      <x:c r="AC15" s="18"/>
+      <x:c r="AD15" s="18"/>
+      <x:c r="AE15" s="18"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="18"/>
@@ -1024,15 +1104,19 @@
       <x:c r="P16" s="18"/>
       <x:c r="Q16" s="18"/>
       <x:c r="R16" s="18"/>
-      <x:c r="S16" s="18"/>
-      <x:c r="T16" s="18"/>
+      <x:c r="S16" s="21"/>
+      <x:c r="T16" s="21"/>
       <x:c r="U16" s="21"/>
       <x:c r="V16" s="21"/>
-      <x:c r="W16" s="18"/>
-      <x:c r="X16" s="18"/>
-      <x:c r="Y16" s="18"/>
-      <x:c r="Z16" s="18"/>
+      <x:c r="W16" s="21"/>
+      <x:c r="X16" s="21"/>
+      <x:c r="Y16" s="21"/>
+      <x:c r="Z16" s="21"/>
       <x:c r="AA16" s="18"/>
+      <x:c r="AB16" s="18"/>
+      <x:c r="AC16" s="18"/>
+      <x:c r="AD16" s="18"/>
+      <x:c r="AE16" s="18"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="18"/>
@@ -1053,15 +1137,19 @@
       <x:c r="P17" s="18"/>
       <x:c r="Q17" s="18"/>
       <x:c r="R17" s="18"/>
-      <x:c r="S17" s="18"/>
-      <x:c r="T17" s="18"/>
+      <x:c r="S17" s="21"/>
+      <x:c r="T17" s="21"/>
       <x:c r="U17" s="21"/>
       <x:c r="V17" s="21"/>
-      <x:c r="W17" s="18"/>
-      <x:c r="X17" s="18"/>
-      <x:c r="Y17" s="18"/>
-      <x:c r="Z17" s="18"/>
+      <x:c r="W17" s="21"/>
+      <x:c r="X17" s="21"/>
+      <x:c r="Y17" s="21"/>
+      <x:c r="Z17" s="21"/>
       <x:c r="AA17" s="18"/>
+      <x:c r="AB17" s="18"/>
+      <x:c r="AC17" s="18"/>
+      <x:c r="AD17" s="18"/>
+      <x:c r="AE17" s="18"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="18"/>
@@ -1082,15 +1170,19 @@
       <x:c r="P18" s="18"/>
       <x:c r="Q18" s="18"/>
       <x:c r="R18" s="18"/>
-      <x:c r="S18" s="18"/>
-      <x:c r="T18" s="18"/>
+      <x:c r="S18" s="21"/>
+      <x:c r="T18" s="21"/>
       <x:c r="U18" s="21"/>
       <x:c r="V18" s="21"/>
-      <x:c r="W18" s="18"/>
-      <x:c r="X18" s="18"/>
-      <x:c r="Y18" s="18"/>
-      <x:c r="Z18" s="18"/>
+      <x:c r="W18" s="21"/>
+      <x:c r="X18" s="21"/>
+      <x:c r="Y18" s="21"/>
+      <x:c r="Z18" s="21"/>
       <x:c r="AA18" s="18"/>
+      <x:c r="AB18" s="18"/>
+      <x:c r="AC18" s="18"/>
+      <x:c r="AD18" s="18"/>
+      <x:c r="AE18" s="18"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="18"/>
@@ -1111,15 +1203,19 @@
       <x:c r="P19" s="18"/>
       <x:c r="Q19" s="18"/>
       <x:c r="R19" s="18"/>
-      <x:c r="S19" s="18"/>
-      <x:c r="T19" s="18"/>
+      <x:c r="S19" s="21"/>
+      <x:c r="T19" s="21"/>
       <x:c r="U19" s="21"/>
       <x:c r="V19" s="21"/>
-      <x:c r="W19" s="18"/>
-      <x:c r="X19" s="18"/>
-      <x:c r="Y19" s="18"/>
-      <x:c r="Z19" s="18"/>
+      <x:c r="W19" s="21"/>
+      <x:c r="X19" s="21"/>
+      <x:c r="Y19" s="21"/>
+      <x:c r="Z19" s="21"/>
       <x:c r="AA19" s="18"/>
+      <x:c r="AB19" s="18"/>
+      <x:c r="AC19" s="18"/>
+      <x:c r="AD19" s="18"/>
+      <x:c r="AE19" s="18"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="18"/>
@@ -1140,15 +1236,19 @@
       <x:c r="P20" s="18"/>
       <x:c r="Q20" s="18"/>
       <x:c r="R20" s="18"/>
-      <x:c r="S20" s="18"/>
-      <x:c r="T20" s="18"/>
+      <x:c r="S20" s="21"/>
+      <x:c r="T20" s="21"/>
       <x:c r="U20" s="21"/>
       <x:c r="V20" s="21"/>
-      <x:c r="W20" s="18"/>
-      <x:c r="X20" s="18"/>
-      <x:c r="Y20" s="18"/>
-      <x:c r="Z20" s="18"/>
+      <x:c r="W20" s="21"/>
+      <x:c r="X20" s="21"/>
+      <x:c r="Y20" s="21"/>
+      <x:c r="Z20" s="21"/>
       <x:c r="AA20" s="18"/>
+      <x:c r="AB20" s="18"/>
+      <x:c r="AC20" s="18"/>
+      <x:c r="AD20" s="18"/>
+      <x:c r="AE20" s="18"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="18"/>
@@ -1169,15 +1269,19 @@
       <x:c r="P21" s="18"/>
       <x:c r="Q21" s="18"/>
       <x:c r="R21" s="18"/>
-      <x:c r="S21" s="18"/>
-      <x:c r="T21" s="18"/>
+      <x:c r="S21" s="21"/>
+      <x:c r="T21" s="21"/>
       <x:c r="U21" s="21"/>
       <x:c r="V21" s="21"/>
-      <x:c r="W21" s="18"/>
-      <x:c r="X21" s="18"/>
-      <x:c r="Y21" s="18"/>
-      <x:c r="Z21" s="18"/>
+      <x:c r="W21" s="21"/>
+      <x:c r="X21" s="21"/>
+      <x:c r="Y21" s="21"/>
+      <x:c r="Z21" s="21"/>
       <x:c r="AA21" s="18"/>
+      <x:c r="AB21" s="18"/>
+      <x:c r="AC21" s="18"/>
+      <x:c r="AD21" s="18"/>
+      <x:c r="AE21" s="18"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="18"/>
@@ -1198,15 +1302,19 @@
       <x:c r="P22" s="18"/>
       <x:c r="Q22" s="18"/>
       <x:c r="R22" s="18"/>
-      <x:c r="S22" s="18"/>
-      <x:c r="T22" s="18"/>
+      <x:c r="S22" s="21"/>
+      <x:c r="T22" s="21"/>
       <x:c r="U22" s="21"/>
       <x:c r="V22" s="21"/>
-      <x:c r="W22" s="18"/>
-      <x:c r="X22" s="18"/>
-      <x:c r="Y22" s="18"/>
-      <x:c r="Z22" s="18"/>
+      <x:c r="W22" s="21"/>
+      <x:c r="X22" s="21"/>
+      <x:c r="Y22" s="21"/>
+      <x:c r="Z22" s="21"/>
       <x:c r="AA22" s="18"/>
+      <x:c r="AB22" s="18"/>
+      <x:c r="AC22" s="18"/>
+      <x:c r="AD22" s="18"/>
+      <x:c r="AE22" s="18"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="18"/>
@@ -1227,15 +1335,19 @@
       <x:c r="P23" s="18"/>
       <x:c r="Q23" s="18"/>
       <x:c r="R23" s="18"/>
-      <x:c r="S23" s="18"/>
-      <x:c r="T23" s="18"/>
+      <x:c r="S23" s="21"/>
+      <x:c r="T23" s="21"/>
       <x:c r="U23" s="21"/>
       <x:c r="V23" s="21"/>
-      <x:c r="W23" s="18"/>
-      <x:c r="X23" s="18"/>
-      <x:c r="Y23" s="18"/>
-      <x:c r="Z23" s="18"/>
+      <x:c r="W23" s="21"/>
+      <x:c r="X23" s="21"/>
+      <x:c r="Y23" s="21"/>
+      <x:c r="Z23" s="21"/>
       <x:c r="AA23" s="18"/>
+      <x:c r="AB23" s="18"/>
+      <x:c r="AC23" s="18"/>
+      <x:c r="AD23" s="18"/>
+      <x:c r="AE23" s="18"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="18"/>
@@ -1256,15 +1368,19 @@
       <x:c r="P24" s="18"/>
       <x:c r="Q24" s="18"/>
       <x:c r="R24" s="18"/>
-      <x:c r="S24" s="18"/>
-      <x:c r="T24" s="18"/>
+      <x:c r="S24" s="21"/>
+      <x:c r="T24" s="21"/>
       <x:c r="U24" s="21"/>
       <x:c r="V24" s="21"/>
-      <x:c r="W24" s="18"/>
-      <x:c r="X24" s="18"/>
-      <x:c r="Y24" s="18"/>
-      <x:c r="Z24" s="18"/>
+      <x:c r="W24" s="21"/>
+      <x:c r="X24" s="21"/>
+      <x:c r="Y24" s="21"/>
+      <x:c r="Z24" s="21"/>
       <x:c r="AA24" s="18"/>
+      <x:c r="AB24" s="18"/>
+      <x:c r="AC24" s="18"/>
+      <x:c r="AD24" s="18"/>
+      <x:c r="AE24" s="18"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="18"/>
@@ -1285,15 +1401,19 @@
       <x:c r="P25" s="18"/>
       <x:c r="Q25" s="18"/>
       <x:c r="R25" s="18"/>
-      <x:c r="S25" s="18"/>
-      <x:c r="T25" s="18"/>
+      <x:c r="S25" s="21"/>
+      <x:c r="T25" s="21"/>
       <x:c r="U25" s="21"/>
       <x:c r="V25" s="21"/>
-      <x:c r="W25" s="18"/>
-      <x:c r="X25" s="18"/>
-      <x:c r="Y25" s="18"/>
-      <x:c r="Z25" s="18"/>
+      <x:c r="W25" s="21"/>
+      <x:c r="X25" s="21"/>
+      <x:c r="Y25" s="21"/>
+      <x:c r="Z25" s="21"/>
       <x:c r="AA25" s="18"/>
+      <x:c r="AB25" s="18"/>
+      <x:c r="AC25" s="18"/>
+      <x:c r="AD25" s="18"/>
+      <x:c r="AE25" s="18"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="18"/>
@@ -1314,15 +1434,19 @@
       <x:c r="P26" s="18"/>
       <x:c r="Q26" s="18"/>
       <x:c r="R26" s="18"/>
-      <x:c r="S26" s="18"/>
-      <x:c r="T26" s="18"/>
+      <x:c r="S26" s="21"/>
+      <x:c r="T26" s="21"/>
       <x:c r="U26" s="21"/>
       <x:c r="V26" s="21"/>
-      <x:c r="W26" s="18"/>
-      <x:c r="X26" s="18"/>
-      <x:c r="Y26" s="18"/>
-      <x:c r="Z26" s="18"/>
+      <x:c r="W26" s="21"/>
+      <x:c r="X26" s="21"/>
+      <x:c r="Y26" s="21"/>
+      <x:c r="Z26" s="21"/>
       <x:c r="AA26" s="18"/>
+      <x:c r="AB26" s="18"/>
+      <x:c r="AC26" s="18"/>
+      <x:c r="AD26" s="18"/>
+      <x:c r="AE26" s="18"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="18"/>
@@ -1343,15 +1467,19 @@
       <x:c r="P27" s="18"/>
       <x:c r="Q27" s="18"/>
       <x:c r="R27" s="18"/>
-      <x:c r="S27" s="18"/>
-      <x:c r="T27" s="18"/>
+      <x:c r="S27" s="21"/>
+      <x:c r="T27" s="21"/>
       <x:c r="U27" s="21"/>
       <x:c r="V27" s="21"/>
-      <x:c r="W27" s="18"/>
-      <x:c r="X27" s="18"/>
-      <x:c r="Y27" s="18"/>
-      <x:c r="Z27" s="18"/>
+      <x:c r="W27" s="21"/>
+      <x:c r="X27" s="21"/>
+      <x:c r="Y27" s="21"/>
+      <x:c r="Z27" s="21"/>
       <x:c r="AA27" s="18"/>
+      <x:c r="AB27" s="18"/>
+      <x:c r="AC27" s="18"/>
+      <x:c r="AD27" s="18"/>
+      <x:c r="AE27" s="18"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="18"/>
@@ -1372,15 +1500,19 @@
       <x:c r="P28" s="18"/>
       <x:c r="Q28" s="18"/>
       <x:c r="R28" s="18"/>
-      <x:c r="S28" s="18"/>
-      <x:c r="T28" s="18"/>
+      <x:c r="S28" s="21"/>
+      <x:c r="T28" s="21"/>
       <x:c r="U28" s="21"/>
       <x:c r="V28" s="21"/>
-      <x:c r="W28" s="18"/>
-      <x:c r="X28" s="18"/>
-      <x:c r="Y28" s="18"/>
-      <x:c r="Z28" s="18"/>
+      <x:c r="W28" s="21"/>
+      <x:c r="X28" s="21"/>
+      <x:c r="Y28" s="21"/>
+      <x:c r="Z28" s="21"/>
       <x:c r="AA28" s="18"/>
+      <x:c r="AB28" s="18"/>
+      <x:c r="AC28" s="18"/>
+      <x:c r="AD28" s="18"/>
+      <x:c r="AE28" s="18"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="18"/>
@@ -1401,15 +1533,19 @@
       <x:c r="P29" s="18"/>
       <x:c r="Q29" s="18"/>
       <x:c r="R29" s="18"/>
-      <x:c r="S29" s="18"/>
-      <x:c r="T29" s="18"/>
+      <x:c r="S29" s="21"/>
+      <x:c r="T29" s="21"/>
       <x:c r="U29" s="21"/>
       <x:c r="V29" s="21"/>
-      <x:c r="W29" s="18"/>
-      <x:c r="X29" s="18"/>
-      <x:c r="Y29" s="18"/>
-      <x:c r="Z29" s="18"/>
+      <x:c r="W29" s="21"/>
+      <x:c r="X29" s="21"/>
+      <x:c r="Y29" s="21"/>
+      <x:c r="Z29" s="21"/>
       <x:c r="AA29" s="18"/>
+      <x:c r="AB29" s="18"/>
+      <x:c r="AC29" s="18"/>
+      <x:c r="AD29" s="18"/>
+      <x:c r="AE29" s="18"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="18"/>
@@ -1430,15 +1566,19 @@
       <x:c r="P30" s="18"/>
       <x:c r="Q30" s="18"/>
       <x:c r="R30" s="18"/>
-      <x:c r="S30" s="18"/>
-      <x:c r="T30" s="18"/>
+      <x:c r="S30" s="21"/>
+      <x:c r="T30" s="21"/>
       <x:c r="U30" s="21"/>
       <x:c r="V30" s="21"/>
-      <x:c r="W30" s="18"/>
-      <x:c r="X30" s="18"/>
-      <x:c r="Y30" s="18"/>
-      <x:c r="Z30" s="18"/>
+      <x:c r="W30" s="21"/>
+      <x:c r="X30" s="21"/>
+      <x:c r="Y30" s="21"/>
+      <x:c r="Z30" s="21"/>
       <x:c r="AA30" s="18"/>
+      <x:c r="AB30" s="18"/>
+      <x:c r="AC30" s="18"/>
+      <x:c r="AD30" s="18"/>
+      <x:c r="AE30" s="18"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="18"/>
@@ -1459,15 +1599,19 @@
       <x:c r="P31" s="18"/>
       <x:c r="Q31" s="18"/>
       <x:c r="R31" s="18"/>
-      <x:c r="S31" s="18"/>
-      <x:c r="T31" s="18"/>
+      <x:c r="S31" s="21"/>
+      <x:c r="T31" s="21"/>
       <x:c r="U31" s="21"/>
       <x:c r="V31" s="21"/>
-      <x:c r="W31" s="18"/>
-      <x:c r="X31" s="18"/>
-      <x:c r="Y31" s="18"/>
-      <x:c r="Z31" s="18"/>
+      <x:c r="W31" s="21"/>
+      <x:c r="X31" s="21"/>
+      <x:c r="Y31" s="21"/>
+      <x:c r="Z31" s="21"/>
       <x:c r="AA31" s="18"/>
+      <x:c r="AB31" s="18"/>
+      <x:c r="AC31" s="18"/>
+      <x:c r="AD31" s="18"/>
+      <x:c r="AE31" s="18"/>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="18"/>
@@ -1488,15 +1632,19 @@
       <x:c r="P32" s="18"/>
       <x:c r="Q32" s="18"/>
       <x:c r="R32" s="18"/>
-      <x:c r="S32" s="18"/>
-      <x:c r="T32" s="18"/>
+      <x:c r="S32" s="21"/>
+      <x:c r="T32" s="21"/>
       <x:c r="U32" s="21"/>
       <x:c r="V32" s="21"/>
-      <x:c r="W32" s="18"/>
-      <x:c r="X32" s="18"/>
-      <x:c r="Y32" s="18"/>
-      <x:c r="Z32" s="18"/>
+      <x:c r="W32" s="21"/>
+      <x:c r="X32" s="21"/>
+      <x:c r="Y32" s="21"/>
+      <x:c r="Z32" s="21"/>
       <x:c r="AA32" s="18"/>
+      <x:c r="AB32" s="18"/>
+      <x:c r="AC32" s="18"/>
+      <x:c r="AD32" s="18"/>
+      <x:c r="AE32" s="18"/>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="18"/>
@@ -1517,15 +1665,19 @@
       <x:c r="P33" s="18"/>
       <x:c r="Q33" s="18"/>
       <x:c r="R33" s="18"/>
-      <x:c r="S33" s="18"/>
-      <x:c r="T33" s="18"/>
+      <x:c r="S33" s="21"/>
+      <x:c r="T33" s="21"/>
       <x:c r="U33" s="21"/>
       <x:c r="V33" s="21"/>
-      <x:c r="W33" s="18"/>
-      <x:c r="X33" s="18"/>
-      <x:c r="Y33" s="18"/>
-      <x:c r="Z33" s="18"/>
+      <x:c r="W33" s="21"/>
+      <x:c r="X33" s="21"/>
+      <x:c r="Y33" s="21"/>
+      <x:c r="Z33" s="21"/>
       <x:c r="AA33" s="18"/>
+      <x:c r="AB33" s="18"/>
+      <x:c r="AC33" s="18"/>
+      <x:c r="AD33" s="18"/>
+      <x:c r="AE33" s="18"/>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="18"/>
@@ -1546,15 +1698,19 @@
       <x:c r="P34" s="18"/>
       <x:c r="Q34" s="18"/>
       <x:c r="R34" s="18"/>
-      <x:c r="S34" s="18"/>
-      <x:c r="T34" s="18"/>
+      <x:c r="S34" s="21"/>
+      <x:c r="T34" s="21"/>
       <x:c r="U34" s="21"/>
       <x:c r="V34" s="21"/>
-      <x:c r="W34" s="18"/>
-      <x:c r="X34" s="18"/>
-      <x:c r="Y34" s="18"/>
-      <x:c r="Z34" s="18"/>
+      <x:c r="W34" s="21"/>
+      <x:c r="X34" s="21"/>
+      <x:c r="Y34" s="21"/>
+      <x:c r="Z34" s="21"/>
       <x:c r="AA34" s="18"/>
+      <x:c r="AB34" s="18"/>
+      <x:c r="AC34" s="18"/>
+      <x:c r="AD34" s="18"/>
+      <x:c r="AE34" s="18"/>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="18"/>
@@ -1575,15 +1731,19 @@
       <x:c r="P35" s="18"/>
       <x:c r="Q35" s="18"/>
       <x:c r="R35" s="18"/>
-      <x:c r="S35" s="18"/>
-      <x:c r="T35" s="18"/>
+      <x:c r="S35" s="21"/>
+      <x:c r="T35" s="21"/>
       <x:c r="U35" s="21"/>
       <x:c r="V35" s="21"/>
-      <x:c r="W35" s="18"/>
-      <x:c r="X35" s="18"/>
-      <x:c r="Y35" s="18"/>
-      <x:c r="Z35" s="18"/>
+      <x:c r="W35" s="21"/>
+      <x:c r="X35" s="21"/>
+      <x:c r="Y35" s="21"/>
+      <x:c r="Z35" s="21"/>
       <x:c r="AA35" s="18"/>
+      <x:c r="AB35" s="18"/>
+      <x:c r="AC35" s="18"/>
+      <x:c r="AD35" s="18"/>
+      <x:c r="AE35" s="18"/>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="18"/>
@@ -1604,15 +1764,19 @@
       <x:c r="P36" s="18"/>
       <x:c r="Q36" s="18"/>
       <x:c r="R36" s="18"/>
-      <x:c r="S36" s="18"/>
-      <x:c r="T36" s="18"/>
+      <x:c r="S36" s="21"/>
+      <x:c r="T36" s="21"/>
       <x:c r="U36" s="21"/>
       <x:c r="V36" s="21"/>
-      <x:c r="W36" s="18"/>
-      <x:c r="X36" s="18"/>
-      <x:c r="Y36" s="18"/>
-      <x:c r="Z36" s="18"/>
+      <x:c r="W36" s="21"/>
+      <x:c r="X36" s="21"/>
+      <x:c r="Y36" s="21"/>
+      <x:c r="Z36" s="21"/>
       <x:c r="AA36" s="18"/>
+      <x:c r="AB36" s="18"/>
+      <x:c r="AC36" s="18"/>
+      <x:c r="AD36" s="18"/>
+      <x:c r="AE36" s="18"/>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="18"/>
@@ -1633,15 +1797,19 @@
       <x:c r="P37" s="18"/>
       <x:c r="Q37" s="18"/>
       <x:c r="R37" s="18"/>
-      <x:c r="S37" s="18"/>
-      <x:c r="T37" s="18"/>
+      <x:c r="S37" s="21"/>
+      <x:c r="T37" s="21"/>
       <x:c r="U37" s="21"/>
       <x:c r="V37" s="21"/>
-      <x:c r="W37" s="18"/>
-      <x:c r="X37" s="18"/>
-      <x:c r="Y37" s="18"/>
-      <x:c r="Z37" s="18"/>
+      <x:c r="W37" s="21"/>
+      <x:c r="X37" s="21"/>
+      <x:c r="Y37" s="21"/>
+      <x:c r="Z37" s="21"/>
       <x:c r="AA37" s="18"/>
+      <x:c r="AB37" s="18"/>
+      <x:c r="AC37" s="18"/>
+      <x:c r="AD37" s="18"/>
+      <x:c r="AE37" s="18"/>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="18"/>
@@ -1662,15 +1830,19 @@
       <x:c r="P38" s="18"/>
       <x:c r="Q38" s="18"/>
       <x:c r="R38" s="18"/>
-      <x:c r="S38" s="18"/>
-      <x:c r="T38" s="18"/>
+      <x:c r="S38" s="21"/>
+      <x:c r="T38" s="21"/>
       <x:c r="U38" s="21"/>
       <x:c r="V38" s="21"/>
-      <x:c r="W38" s="18"/>
-      <x:c r="X38" s="18"/>
-      <x:c r="Y38" s="18"/>
-      <x:c r="Z38" s="18"/>
+      <x:c r="W38" s="21"/>
+      <x:c r="X38" s="21"/>
+      <x:c r="Y38" s="21"/>
+      <x:c r="Z38" s="21"/>
       <x:c r="AA38" s="18"/>
+      <x:c r="AB38" s="18"/>
+      <x:c r="AC38" s="18"/>
+      <x:c r="AD38" s="18"/>
+      <x:c r="AE38" s="18"/>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="18"/>
@@ -1691,15 +1863,19 @@
       <x:c r="P39" s="18"/>
       <x:c r="Q39" s="18"/>
       <x:c r="R39" s="18"/>
-      <x:c r="S39" s="18"/>
-      <x:c r="T39" s="18"/>
+      <x:c r="S39" s="21"/>
+      <x:c r="T39" s="21"/>
       <x:c r="U39" s="21"/>
       <x:c r="V39" s="21"/>
-      <x:c r="W39" s="18"/>
-      <x:c r="X39" s="18"/>
-      <x:c r="Y39" s="18"/>
-      <x:c r="Z39" s="18"/>
+      <x:c r="W39" s="21"/>
+      <x:c r="X39" s="21"/>
+      <x:c r="Y39" s="21"/>
+      <x:c r="Z39" s="21"/>
       <x:c r="AA39" s="18"/>
+      <x:c r="AB39" s="18"/>
+      <x:c r="AC39" s="18"/>
+      <x:c r="AD39" s="18"/>
+      <x:c r="AE39" s="18"/>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="18"/>
@@ -1720,15 +1896,19 @@
       <x:c r="P40" s="18"/>
       <x:c r="Q40" s="18"/>
       <x:c r="R40" s="18"/>
-      <x:c r="S40" s="18"/>
-      <x:c r="T40" s="18"/>
+      <x:c r="S40" s="21"/>
+      <x:c r="T40" s="21"/>
       <x:c r="U40" s="21"/>
       <x:c r="V40" s="21"/>
-      <x:c r="W40" s="18"/>
-      <x:c r="X40" s="18"/>
-      <x:c r="Y40" s="18"/>
-      <x:c r="Z40" s="18"/>
+      <x:c r="W40" s="21"/>
+      <x:c r="X40" s="21"/>
+      <x:c r="Y40" s="21"/>
+      <x:c r="Z40" s="21"/>
       <x:c r="AA40" s="18"/>
+      <x:c r="AB40" s="18"/>
+      <x:c r="AC40" s="18"/>
+      <x:c r="AD40" s="18"/>
+      <x:c r="AE40" s="18"/>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="18"/>
@@ -1749,15 +1929,19 @@
       <x:c r="P41" s="18"/>
       <x:c r="Q41" s="18"/>
       <x:c r="R41" s="18"/>
-      <x:c r="S41" s="18"/>
-      <x:c r="T41" s="18"/>
+      <x:c r="S41" s="21"/>
+      <x:c r="T41" s="21"/>
       <x:c r="U41" s="21"/>
       <x:c r="V41" s="21"/>
-      <x:c r="W41" s="18"/>
-      <x:c r="X41" s="18"/>
-      <x:c r="Y41" s="18"/>
-      <x:c r="Z41" s="18"/>
+      <x:c r="W41" s="21"/>
+      <x:c r="X41" s="21"/>
+      <x:c r="Y41" s="21"/>
+      <x:c r="Z41" s="21"/>
       <x:c r="AA41" s="18"/>
+      <x:c r="AB41" s="18"/>
+      <x:c r="AC41" s="18"/>
+      <x:c r="AD41" s="18"/>
+      <x:c r="AE41" s="18"/>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="18"/>
@@ -1778,15 +1962,19 @@
       <x:c r="P42" s="18"/>
       <x:c r="Q42" s="18"/>
       <x:c r="R42" s="18"/>
-      <x:c r="S42" s="18"/>
-      <x:c r="T42" s="18"/>
+      <x:c r="S42" s="21"/>
+      <x:c r="T42" s="21"/>
       <x:c r="U42" s="21"/>
       <x:c r="V42" s="21"/>
-      <x:c r="W42" s="18"/>
-      <x:c r="X42" s="18"/>
-      <x:c r="Y42" s="18"/>
-      <x:c r="Z42" s="18"/>
+      <x:c r="W42" s="21"/>
+      <x:c r="X42" s="21"/>
+      <x:c r="Y42" s="21"/>
+      <x:c r="Z42" s="21"/>
       <x:c r="AA42" s="18"/>
+      <x:c r="AB42" s="18"/>
+      <x:c r="AC42" s="18"/>
+      <x:c r="AD42" s="18"/>
+      <x:c r="AE42" s="18"/>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="18"/>
@@ -1807,15 +1995,19 @@
       <x:c r="P43" s="18"/>
       <x:c r="Q43" s="18"/>
       <x:c r="R43" s="18"/>
-      <x:c r="S43" s="18"/>
-      <x:c r="T43" s="18"/>
+      <x:c r="S43" s="21"/>
+      <x:c r="T43" s="21"/>
       <x:c r="U43" s="21"/>
       <x:c r="V43" s="21"/>
-      <x:c r="W43" s="18"/>
-      <x:c r="X43" s="18"/>
-      <x:c r="Y43" s="18"/>
-      <x:c r="Z43" s="18"/>
+      <x:c r="W43" s="21"/>
+      <x:c r="X43" s="21"/>
+      <x:c r="Y43" s="21"/>
+      <x:c r="Z43" s="21"/>
       <x:c r="AA43" s="18"/>
+      <x:c r="AB43" s="18"/>
+      <x:c r="AC43" s="18"/>
+      <x:c r="AD43" s="18"/>
+      <x:c r="AE43" s="18"/>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="18"/>
@@ -1836,15 +2028,19 @@
       <x:c r="P44" s="18"/>
       <x:c r="Q44" s="18"/>
       <x:c r="R44" s="18"/>
-      <x:c r="S44" s="18"/>
-      <x:c r="T44" s="18"/>
+      <x:c r="S44" s="21"/>
+      <x:c r="T44" s="21"/>
       <x:c r="U44" s="21"/>
       <x:c r="V44" s="21"/>
-      <x:c r="W44" s="18"/>
-      <x:c r="X44" s="18"/>
-      <x:c r="Y44" s="18"/>
-      <x:c r="Z44" s="18"/>
+      <x:c r="W44" s="21"/>
+      <x:c r="X44" s="21"/>
+      <x:c r="Y44" s="21"/>
+      <x:c r="Z44" s="21"/>
       <x:c r="AA44" s="18"/>
+      <x:c r="AB44" s="18"/>
+      <x:c r="AC44" s="18"/>
+      <x:c r="AD44" s="18"/>
+      <x:c r="AE44" s="18"/>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="18"/>
@@ -1865,15 +2061,19 @@
       <x:c r="P45" s="18"/>
       <x:c r="Q45" s="18"/>
       <x:c r="R45" s="18"/>
-      <x:c r="S45" s="18"/>
-      <x:c r="T45" s="18"/>
+      <x:c r="S45" s="21"/>
+      <x:c r="T45" s="21"/>
       <x:c r="U45" s="21"/>
       <x:c r="V45" s="21"/>
-      <x:c r="W45" s="18"/>
-      <x:c r="X45" s="18"/>
-      <x:c r="Y45" s="18"/>
-      <x:c r="Z45" s="18"/>
+      <x:c r="W45" s="21"/>
+      <x:c r="X45" s="21"/>
+      <x:c r="Y45" s="21"/>
+      <x:c r="Z45" s="21"/>
       <x:c r="AA45" s="18"/>
+      <x:c r="AB45" s="18"/>
+      <x:c r="AC45" s="18"/>
+      <x:c r="AD45" s="18"/>
+      <x:c r="AE45" s="18"/>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="18"/>
@@ -1894,15 +2094,19 @@
       <x:c r="P46" s="18"/>
       <x:c r="Q46" s="18"/>
       <x:c r="R46" s="18"/>
-      <x:c r="S46" s="18"/>
-      <x:c r="T46" s="18"/>
+      <x:c r="S46" s="21"/>
+      <x:c r="T46" s="21"/>
       <x:c r="U46" s="21"/>
       <x:c r="V46" s="21"/>
-      <x:c r="W46" s="18"/>
-      <x:c r="X46" s="18"/>
-      <x:c r="Y46" s="18"/>
-      <x:c r="Z46" s="18"/>
+      <x:c r="W46" s="21"/>
+      <x:c r="X46" s="21"/>
+      <x:c r="Y46" s="21"/>
+      <x:c r="Z46" s="21"/>
       <x:c r="AA46" s="18"/>
+      <x:c r="AB46" s="18"/>
+      <x:c r="AC46" s="18"/>
+      <x:c r="AD46" s="18"/>
+      <x:c r="AE46" s="18"/>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="18"/>
@@ -1923,15 +2127,19 @@
       <x:c r="P47" s="18"/>
       <x:c r="Q47" s="18"/>
       <x:c r="R47" s="18"/>
-      <x:c r="S47" s="18"/>
-      <x:c r="T47" s="18"/>
+      <x:c r="S47" s="21"/>
+      <x:c r="T47" s="21"/>
       <x:c r="U47" s="21"/>
       <x:c r="V47" s="21"/>
-      <x:c r="W47" s="18"/>
-      <x:c r="X47" s="18"/>
-      <x:c r="Y47" s="18"/>
-      <x:c r="Z47" s="18"/>
+      <x:c r="W47" s="21"/>
+      <x:c r="X47" s="21"/>
+      <x:c r="Y47" s="21"/>
+      <x:c r="Z47" s="21"/>
       <x:c r="AA47" s="18"/>
+      <x:c r="AB47" s="18"/>
+      <x:c r="AC47" s="18"/>
+      <x:c r="AD47" s="18"/>
+      <x:c r="AE47" s="18"/>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="18"/>
@@ -1952,15 +2160,19 @@
       <x:c r="P48" s="18"/>
       <x:c r="Q48" s="18"/>
       <x:c r="R48" s="18"/>
-      <x:c r="S48" s="18"/>
-      <x:c r="T48" s="18"/>
+      <x:c r="S48" s="21"/>
+      <x:c r="T48" s="21"/>
       <x:c r="U48" s="21"/>
       <x:c r="V48" s="21"/>
-      <x:c r="W48" s="18"/>
-      <x:c r="X48" s="18"/>
-      <x:c r="Y48" s="18"/>
-      <x:c r="Z48" s="18"/>
+      <x:c r="W48" s="21"/>
+      <x:c r="X48" s="21"/>
+      <x:c r="Y48" s="21"/>
+      <x:c r="Z48" s="21"/>
       <x:c r="AA48" s="18"/>
+      <x:c r="AB48" s="18"/>
+      <x:c r="AC48" s="18"/>
+      <x:c r="AD48" s="18"/>
+      <x:c r="AE48" s="18"/>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="18"/>
@@ -1981,15 +2193,19 @@
       <x:c r="P49" s="18"/>
       <x:c r="Q49" s="18"/>
       <x:c r="R49" s="18"/>
-      <x:c r="S49" s="18"/>
-      <x:c r="T49" s="18"/>
+      <x:c r="S49" s="21"/>
+      <x:c r="T49" s="21"/>
       <x:c r="U49" s="21"/>
       <x:c r="V49" s="21"/>
-      <x:c r="W49" s="18"/>
-      <x:c r="X49" s="18"/>
-      <x:c r="Y49" s="18"/>
-      <x:c r="Z49" s="18"/>
+      <x:c r="W49" s="21"/>
+      <x:c r="X49" s="21"/>
+      <x:c r="Y49" s="21"/>
+      <x:c r="Z49" s="21"/>
       <x:c r="AA49" s="18"/>
+      <x:c r="AB49" s="18"/>
+      <x:c r="AC49" s="18"/>
+      <x:c r="AD49" s="18"/>
+      <x:c r="AE49" s="18"/>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="18"/>
@@ -2010,15 +2226,19 @@
       <x:c r="P50" s="18"/>
       <x:c r="Q50" s="18"/>
       <x:c r="R50" s="18"/>
-      <x:c r="S50" s="18"/>
-      <x:c r="T50" s="18"/>
+      <x:c r="S50" s="21"/>
+      <x:c r="T50" s="21"/>
       <x:c r="U50" s="21"/>
       <x:c r="V50" s="21"/>
-      <x:c r="W50" s="18"/>
-      <x:c r="X50" s="18"/>
-      <x:c r="Y50" s="18"/>
-      <x:c r="Z50" s="18"/>
+      <x:c r="W50" s="21"/>
+      <x:c r="X50" s="21"/>
+      <x:c r="Y50" s="21"/>
+      <x:c r="Z50" s="21"/>
       <x:c r="AA50" s="18"/>
+      <x:c r="AB50" s="18"/>
+      <x:c r="AC50" s="18"/>
+      <x:c r="AD50" s="18"/>
+      <x:c r="AE50" s="18"/>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="18"/>
@@ -2039,15 +2259,19 @@
       <x:c r="P51" s="18"/>
       <x:c r="Q51" s="18"/>
       <x:c r="R51" s="18"/>
-      <x:c r="S51" s="18"/>
-      <x:c r="T51" s="18"/>
+      <x:c r="S51" s="21"/>
+      <x:c r="T51" s="21"/>
       <x:c r="U51" s="21"/>
       <x:c r="V51" s="21"/>
-      <x:c r="W51" s="18"/>
-      <x:c r="X51" s="18"/>
-      <x:c r="Y51" s="18"/>
-      <x:c r="Z51" s="18"/>
+      <x:c r="W51" s="21"/>
+      <x:c r="X51" s="21"/>
+      <x:c r="Y51" s="21"/>
+      <x:c r="Z51" s="21"/>
       <x:c r="AA51" s="18"/>
+      <x:c r="AB51" s="18"/>
+      <x:c r="AC51" s="18"/>
+      <x:c r="AD51" s="18"/>
+      <x:c r="AE51" s="18"/>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="18"/>
@@ -2068,15 +2292,19 @@
       <x:c r="P52" s="18"/>
       <x:c r="Q52" s="18"/>
       <x:c r="R52" s="18"/>
-      <x:c r="S52" s="18"/>
-      <x:c r="T52" s="18"/>
+      <x:c r="S52" s="21"/>
+      <x:c r="T52" s="21"/>
       <x:c r="U52" s="21"/>
       <x:c r="V52" s="21"/>
-      <x:c r="W52" s="18"/>
-      <x:c r="X52" s="18"/>
-      <x:c r="Y52" s="18"/>
-      <x:c r="Z52" s="18"/>
+      <x:c r="W52" s="21"/>
+      <x:c r="X52" s="21"/>
+      <x:c r="Y52" s="21"/>
+      <x:c r="Z52" s="21"/>
       <x:c r="AA52" s="18"/>
+      <x:c r="AB52" s="18"/>
+      <x:c r="AC52" s="18"/>
+      <x:c r="AD52" s="18"/>
+      <x:c r="AE52" s="18"/>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="18"/>
@@ -2097,15 +2325,19 @@
       <x:c r="P53" s="18"/>
       <x:c r="Q53" s="18"/>
       <x:c r="R53" s="18"/>
-      <x:c r="S53" s="18"/>
-      <x:c r="T53" s="18"/>
+      <x:c r="S53" s="21"/>
+      <x:c r="T53" s="21"/>
       <x:c r="U53" s="21"/>
       <x:c r="V53" s="21"/>
-      <x:c r="W53" s="18"/>
-      <x:c r="X53" s="18"/>
-      <x:c r="Y53" s="18"/>
-      <x:c r="Z53" s="18"/>
+      <x:c r="W53" s="21"/>
+      <x:c r="X53" s="21"/>
+      <x:c r="Y53" s="21"/>
+      <x:c r="Z53" s="21"/>
       <x:c r="AA53" s="18"/>
+      <x:c r="AB53" s="18"/>
+      <x:c r="AC53" s="18"/>
+      <x:c r="AD53" s="18"/>
+      <x:c r="AE53" s="18"/>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="18"/>
@@ -2126,15 +2358,19 @@
       <x:c r="P54" s="18"/>
       <x:c r="Q54" s="18"/>
       <x:c r="R54" s="18"/>
-      <x:c r="S54" s="18"/>
-      <x:c r="T54" s="18"/>
+      <x:c r="S54" s="21"/>
+      <x:c r="T54" s="21"/>
       <x:c r="U54" s="21"/>
       <x:c r="V54" s="21"/>
-      <x:c r="W54" s="18"/>
-      <x:c r="X54" s="18"/>
-      <x:c r="Y54" s="18"/>
-      <x:c r="Z54" s="18"/>
+      <x:c r="W54" s="21"/>
+      <x:c r="X54" s="21"/>
+      <x:c r="Y54" s="21"/>
+      <x:c r="Z54" s="21"/>
       <x:c r="AA54" s="18"/>
+      <x:c r="AB54" s="18"/>
+      <x:c r="AC54" s="18"/>
+      <x:c r="AD54" s="18"/>
+      <x:c r="AE54" s="18"/>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="18"/>
@@ -2155,15 +2391,19 @@
       <x:c r="P55" s="18"/>
       <x:c r="Q55" s="18"/>
       <x:c r="R55" s="18"/>
-      <x:c r="S55" s="18"/>
-      <x:c r="T55" s="18"/>
+      <x:c r="S55" s="21"/>
+      <x:c r="T55" s="21"/>
       <x:c r="U55" s="21"/>
       <x:c r="V55" s="21"/>
-      <x:c r="W55" s="18"/>
-      <x:c r="X55" s="18"/>
-      <x:c r="Y55" s="18"/>
-      <x:c r="Z55" s="18"/>
+      <x:c r="W55" s="21"/>
+      <x:c r="X55" s="21"/>
+      <x:c r="Y55" s="21"/>
+      <x:c r="Z55" s="21"/>
       <x:c r="AA55" s="18"/>
+      <x:c r="AB55" s="18"/>
+      <x:c r="AC55" s="18"/>
+      <x:c r="AD55" s="18"/>
+      <x:c r="AE55" s="18"/>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="18"/>
@@ -2184,15 +2424,19 @@
       <x:c r="P56" s="18"/>
       <x:c r="Q56" s="18"/>
       <x:c r="R56" s="18"/>
-      <x:c r="S56" s="18"/>
-      <x:c r="T56" s="18"/>
+      <x:c r="S56" s="21"/>
+      <x:c r="T56" s="21"/>
       <x:c r="U56" s="21"/>
       <x:c r="V56" s="21"/>
-      <x:c r="W56" s="18"/>
-      <x:c r="X56" s="18"/>
-      <x:c r="Y56" s="18"/>
-      <x:c r="Z56" s="18"/>
+      <x:c r="W56" s="21"/>
+      <x:c r="X56" s="21"/>
+      <x:c r="Y56" s="21"/>
+      <x:c r="Z56" s="21"/>
       <x:c r="AA56" s="18"/>
+      <x:c r="AB56" s="18"/>
+      <x:c r="AC56" s="18"/>
+      <x:c r="AD56" s="18"/>
+      <x:c r="AE56" s="18"/>
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="18"/>
@@ -2213,15 +2457,19 @@
       <x:c r="P57" s="18"/>
       <x:c r="Q57" s="18"/>
       <x:c r="R57" s="18"/>
-      <x:c r="S57" s="18"/>
-      <x:c r="T57" s="18"/>
+      <x:c r="S57" s="21"/>
+      <x:c r="T57" s="21"/>
       <x:c r="U57" s="21"/>
       <x:c r="V57" s="21"/>
-      <x:c r="W57" s="18"/>
-      <x:c r="X57" s="18"/>
-      <x:c r="Y57" s="18"/>
-      <x:c r="Z57" s="18"/>
+      <x:c r="W57" s="21"/>
+      <x:c r="X57" s="21"/>
+      <x:c r="Y57" s="21"/>
+      <x:c r="Z57" s="21"/>
       <x:c r="AA57" s="18"/>
+      <x:c r="AB57" s="18"/>
+      <x:c r="AC57" s="18"/>
+      <x:c r="AD57" s="18"/>
+      <x:c r="AE57" s="18"/>
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="18"/>
@@ -2242,15 +2490,19 @@
       <x:c r="P58" s="18"/>
       <x:c r="Q58" s="18"/>
       <x:c r="R58" s="18"/>
-      <x:c r="S58" s="18"/>
-      <x:c r="T58" s="18"/>
+      <x:c r="S58" s="21"/>
+      <x:c r="T58" s="21"/>
       <x:c r="U58" s="21"/>
       <x:c r="V58" s="21"/>
-      <x:c r="W58" s="18"/>
-      <x:c r="X58" s="18"/>
-      <x:c r="Y58" s="18"/>
-      <x:c r="Z58" s="18"/>
+      <x:c r="W58" s="21"/>
+      <x:c r="X58" s="21"/>
+      <x:c r="Y58" s="21"/>
+      <x:c r="Z58" s="21"/>
       <x:c r="AA58" s="18"/>
+      <x:c r="AB58" s="18"/>
+      <x:c r="AC58" s="18"/>
+      <x:c r="AD58" s="18"/>
+      <x:c r="AE58" s="18"/>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="18"/>
@@ -2271,15 +2523,19 @@
       <x:c r="P59" s="18"/>
       <x:c r="Q59" s="18"/>
       <x:c r="R59" s="18"/>
-      <x:c r="S59" s="18"/>
-      <x:c r="T59" s="18"/>
+      <x:c r="S59" s="21"/>
+      <x:c r="T59" s="21"/>
       <x:c r="U59" s="21"/>
       <x:c r="V59" s="21"/>
-      <x:c r="W59" s="18"/>
-      <x:c r="X59" s="18"/>
-      <x:c r="Y59" s="18"/>
-      <x:c r="Z59" s="18"/>
+      <x:c r="W59" s="21"/>
+      <x:c r="X59" s="21"/>
+      <x:c r="Y59" s="21"/>
+      <x:c r="Z59" s="21"/>
       <x:c r="AA59" s="18"/>
+      <x:c r="AB59" s="18"/>
+      <x:c r="AC59" s="18"/>
+      <x:c r="AD59" s="18"/>
+      <x:c r="AE59" s="18"/>
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="18"/>
@@ -2300,15 +2556,19 @@
       <x:c r="P60" s="18"/>
       <x:c r="Q60" s="18"/>
       <x:c r="R60" s="18"/>
-      <x:c r="S60" s="18"/>
-      <x:c r="T60" s="18"/>
+      <x:c r="S60" s="21"/>
+      <x:c r="T60" s="21"/>
       <x:c r="U60" s="21"/>
       <x:c r="V60" s="21"/>
-      <x:c r="W60" s="18"/>
-      <x:c r="X60" s="18"/>
-      <x:c r="Y60" s="18"/>
-      <x:c r="Z60" s="18"/>
+      <x:c r="W60" s="21"/>
+      <x:c r="X60" s="21"/>
+      <x:c r="Y60" s="21"/>
+      <x:c r="Z60" s="21"/>
       <x:c r="AA60" s="18"/>
+      <x:c r="AB60" s="18"/>
+      <x:c r="AC60" s="18"/>
+      <x:c r="AD60" s="18"/>
+      <x:c r="AE60" s="18"/>
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="18"/>
@@ -2329,15 +2589,19 @@
       <x:c r="P61" s="18"/>
       <x:c r="Q61" s="18"/>
       <x:c r="R61" s="18"/>
-      <x:c r="S61" s="18"/>
-      <x:c r="T61" s="18"/>
+      <x:c r="S61" s="21"/>
+      <x:c r="T61" s="21"/>
       <x:c r="U61" s="21"/>
       <x:c r="V61" s="21"/>
-      <x:c r="W61" s="18"/>
-      <x:c r="X61" s="18"/>
-      <x:c r="Y61" s="18"/>
-      <x:c r="Z61" s="18"/>
+      <x:c r="W61" s="21"/>
+      <x:c r="X61" s="21"/>
+      <x:c r="Y61" s="21"/>
+      <x:c r="Z61" s="21"/>
       <x:c r="AA61" s="18"/>
+      <x:c r="AB61" s="18"/>
+      <x:c r="AC61" s="18"/>
+      <x:c r="AD61" s="18"/>
+      <x:c r="AE61" s="18"/>
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="18"/>
@@ -2358,15 +2622,19 @@
       <x:c r="P62" s="18"/>
       <x:c r="Q62" s="18"/>
       <x:c r="R62" s="18"/>
-      <x:c r="S62" s="18"/>
-      <x:c r="T62" s="18"/>
+      <x:c r="S62" s="21"/>
+      <x:c r="T62" s="21"/>
       <x:c r="U62" s="21"/>
       <x:c r="V62" s="21"/>
-      <x:c r="W62" s="18"/>
-      <x:c r="X62" s="18"/>
-      <x:c r="Y62" s="18"/>
-      <x:c r="Z62" s="18"/>
+      <x:c r="W62" s="21"/>
+      <x:c r="X62" s="21"/>
+      <x:c r="Y62" s="21"/>
+      <x:c r="Z62" s="21"/>
       <x:c r="AA62" s="18"/>
+      <x:c r="AB62" s="18"/>
+      <x:c r="AC62" s="18"/>
+      <x:c r="AD62" s="18"/>
+      <x:c r="AE62" s="18"/>
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="18"/>
@@ -2387,15 +2655,19 @@
       <x:c r="P63" s="18"/>
       <x:c r="Q63" s="18"/>
       <x:c r="R63" s="18"/>
-      <x:c r="S63" s="18"/>
-      <x:c r="T63" s="18"/>
+      <x:c r="S63" s="21"/>
+      <x:c r="T63" s="21"/>
       <x:c r="U63" s="21"/>
       <x:c r="V63" s="21"/>
-      <x:c r="W63" s="18"/>
-      <x:c r="X63" s="18"/>
-      <x:c r="Y63" s="18"/>
-      <x:c r="Z63" s="18"/>
+      <x:c r="W63" s="21"/>
+      <x:c r="X63" s="21"/>
+      <x:c r="Y63" s="21"/>
+      <x:c r="Z63" s="21"/>
       <x:c r="AA63" s="18"/>
+      <x:c r="AB63" s="18"/>
+      <x:c r="AC63" s="18"/>
+      <x:c r="AD63" s="18"/>
+      <x:c r="AE63" s="18"/>
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="18"/>
@@ -2416,15 +2688,19 @@
       <x:c r="P64" s="18"/>
       <x:c r="Q64" s="18"/>
       <x:c r="R64" s="18"/>
-      <x:c r="S64" s="18"/>
-      <x:c r="T64" s="18"/>
+      <x:c r="S64" s="21"/>
+      <x:c r="T64" s="21"/>
       <x:c r="U64" s="21"/>
       <x:c r="V64" s="21"/>
-      <x:c r="W64" s="18"/>
-      <x:c r="X64" s="18"/>
-      <x:c r="Y64" s="18"/>
-      <x:c r="Z64" s="18"/>
+      <x:c r="W64" s="21"/>
+      <x:c r="X64" s="21"/>
+      <x:c r="Y64" s="21"/>
+      <x:c r="Z64" s="21"/>
       <x:c r="AA64" s="18"/>
+      <x:c r="AB64" s="18"/>
+      <x:c r="AC64" s="18"/>
+      <x:c r="AD64" s="18"/>
+      <x:c r="AE64" s="18"/>
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="18"/>
@@ -2445,15 +2721,19 @@
       <x:c r="P65" s="18"/>
       <x:c r="Q65" s="18"/>
       <x:c r="R65" s="18"/>
-      <x:c r="S65" s="18"/>
-      <x:c r="T65" s="18"/>
+      <x:c r="S65" s="21"/>
+      <x:c r="T65" s="21"/>
       <x:c r="U65" s="21"/>
       <x:c r="V65" s="21"/>
-      <x:c r="W65" s="18"/>
-      <x:c r="X65" s="18"/>
-      <x:c r="Y65" s="18"/>
-      <x:c r="Z65" s="18"/>
+      <x:c r="W65" s="21"/>
+      <x:c r="X65" s="21"/>
+      <x:c r="Y65" s="21"/>
+      <x:c r="Z65" s="21"/>
       <x:c r="AA65" s="18"/>
+      <x:c r="AB65" s="18"/>
+      <x:c r="AC65" s="18"/>
+      <x:c r="AD65" s="18"/>
+      <x:c r="AE65" s="18"/>
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="18"/>
@@ -2474,15 +2754,19 @@
       <x:c r="P66" s="18"/>
       <x:c r="Q66" s="18"/>
       <x:c r="R66" s="18"/>
-      <x:c r="S66" s="18"/>
-      <x:c r="T66" s="18"/>
+      <x:c r="S66" s="21"/>
+      <x:c r="T66" s="21"/>
       <x:c r="U66" s="21"/>
       <x:c r="V66" s="21"/>
-      <x:c r="W66" s="18"/>
-      <x:c r="X66" s="18"/>
-      <x:c r="Y66" s="18"/>
-      <x:c r="Z66" s="18"/>
+      <x:c r="W66" s="21"/>
+      <x:c r="X66" s="21"/>
+      <x:c r="Y66" s="21"/>
+      <x:c r="Z66" s="21"/>
       <x:c r="AA66" s="18"/>
+      <x:c r="AB66" s="18"/>
+      <x:c r="AC66" s="18"/>
+      <x:c r="AD66" s="18"/>
+      <x:c r="AE66" s="18"/>
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="18"/>
@@ -2503,15 +2787,19 @@
       <x:c r="P67" s="18"/>
       <x:c r="Q67" s="18"/>
       <x:c r="R67" s="18"/>
-      <x:c r="S67" s="18"/>
-      <x:c r="T67" s="18"/>
+      <x:c r="S67" s="21"/>
+      <x:c r="T67" s="21"/>
       <x:c r="U67" s="21"/>
       <x:c r="V67" s="21"/>
-      <x:c r="W67" s="18"/>
-      <x:c r="X67" s="18"/>
-      <x:c r="Y67" s="18"/>
-      <x:c r="Z67" s="18"/>
+      <x:c r="W67" s="21"/>
+      <x:c r="X67" s="21"/>
+      <x:c r="Y67" s="21"/>
+      <x:c r="Z67" s="21"/>
       <x:c r="AA67" s="18"/>
+      <x:c r="AB67" s="18"/>
+      <x:c r="AC67" s="18"/>
+      <x:c r="AD67" s="18"/>
+      <x:c r="AE67" s="18"/>
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="18"/>
@@ -2532,15 +2820,19 @@
       <x:c r="P68" s="18"/>
       <x:c r="Q68" s="18"/>
       <x:c r="R68" s="18"/>
-      <x:c r="S68" s="18"/>
-      <x:c r="T68" s="18"/>
+      <x:c r="S68" s="21"/>
+      <x:c r="T68" s="21"/>
       <x:c r="U68" s="21"/>
       <x:c r="V68" s="21"/>
-      <x:c r="W68" s="18"/>
-      <x:c r="X68" s="18"/>
-      <x:c r="Y68" s="18"/>
-      <x:c r="Z68" s="18"/>
+      <x:c r="W68" s="21"/>
+      <x:c r="X68" s="21"/>
+      <x:c r="Y68" s="21"/>
+      <x:c r="Z68" s="21"/>
       <x:c r="AA68" s="18"/>
+      <x:c r="AB68" s="18"/>
+      <x:c r="AC68" s="18"/>
+      <x:c r="AD68" s="18"/>
+      <x:c r="AE68" s="18"/>
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="18"/>
@@ -2561,15 +2853,19 @@
       <x:c r="P69" s="18"/>
       <x:c r="Q69" s="18"/>
       <x:c r="R69" s="18"/>
-      <x:c r="S69" s="18"/>
-      <x:c r="T69" s="18"/>
+      <x:c r="S69" s="21"/>
+      <x:c r="T69" s="21"/>
       <x:c r="U69" s="21"/>
       <x:c r="V69" s="21"/>
-      <x:c r="W69" s="18"/>
-      <x:c r="X69" s="18"/>
-      <x:c r="Y69" s="18"/>
-      <x:c r="Z69" s="18"/>
+      <x:c r="W69" s="21"/>
+      <x:c r="X69" s="21"/>
+      <x:c r="Y69" s="21"/>
+      <x:c r="Z69" s="21"/>
       <x:c r="AA69" s="18"/>
+      <x:c r="AB69" s="18"/>
+      <x:c r="AC69" s="18"/>
+      <x:c r="AD69" s="18"/>
+      <x:c r="AE69" s="18"/>
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="18"/>
@@ -2590,15 +2886,19 @@
       <x:c r="P70" s="18"/>
       <x:c r="Q70" s="18"/>
       <x:c r="R70" s="18"/>
-      <x:c r="S70" s="18"/>
-      <x:c r="T70" s="18"/>
+      <x:c r="S70" s="21"/>
+      <x:c r="T70" s="21"/>
       <x:c r="U70" s="21"/>
       <x:c r="V70" s="21"/>
-      <x:c r="W70" s="18"/>
-      <x:c r="X70" s="18"/>
-      <x:c r="Y70" s="18"/>
-      <x:c r="Z70" s="18"/>
+      <x:c r="W70" s="21"/>
+      <x:c r="X70" s="21"/>
+      <x:c r="Y70" s="21"/>
+      <x:c r="Z70" s="21"/>
       <x:c r="AA70" s="18"/>
+      <x:c r="AB70" s="18"/>
+      <x:c r="AC70" s="18"/>
+      <x:c r="AD70" s="18"/>
+      <x:c r="AE70" s="18"/>
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="18"/>
@@ -2619,15 +2919,19 @@
       <x:c r="P71" s="18"/>
       <x:c r="Q71" s="18"/>
       <x:c r="R71" s="18"/>
-      <x:c r="S71" s="18"/>
-      <x:c r="T71" s="18"/>
+      <x:c r="S71" s="21"/>
+      <x:c r="T71" s="21"/>
       <x:c r="U71" s="21"/>
       <x:c r="V71" s="21"/>
-      <x:c r="W71" s="18"/>
-      <x:c r="X71" s="18"/>
-      <x:c r="Y71" s="18"/>
-      <x:c r="Z71" s="18"/>
+      <x:c r="W71" s="21"/>
+      <x:c r="X71" s="21"/>
+      <x:c r="Y71" s="21"/>
+      <x:c r="Z71" s="21"/>
       <x:c r="AA71" s="18"/>
+      <x:c r="AB71" s="18"/>
+      <x:c r="AC71" s="18"/>
+      <x:c r="AD71" s="18"/>
+      <x:c r="AE71" s="18"/>
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="18"/>
@@ -2648,15 +2952,19 @@
       <x:c r="P72" s="18"/>
       <x:c r="Q72" s="18"/>
       <x:c r="R72" s="18"/>
-      <x:c r="S72" s="18"/>
-      <x:c r="T72" s="18"/>
+      <x:c r="S72" s="21"/>
+      <x:c r="T72" s="21"/>
       <x:c r="U72" s="21"/>
       <x:c r="V72" s="21"/>
-      <x:c r="W72" s="18"/>
-      <x:c r="X72" s="18"/>
-      <x:c r="Y72" s="18"/>
-      <x:c r="Z72" s="18"/>
+      <x:c r="W72" s="21"/>
+      <x:c r="X72" s="21"/>
+      <x:c r="Y72" s="21"/>
+      <x:c r="Z72" s="21"/>
       <x:c r="AA72" s="18"/>
+      <x:c r="AB72" s="18"/>
+      <x:c r="AC72" s="18"/>
+      <x:c r="AD72" s="18"/>
+      <x:c r="AE72" s="18"/>
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="18"/>
@@ -2677,15 +2985,19 @@
       <x:c r="P73" s="18"/>
       <x:c r="Q73" s="18"/>
       <x:c r="R73" s="18"/>
-      <x:c r="S73" s="18"/>
-      <x:c r="T73" s="18"/>
+      <x:c r="S73" s="21"/>
+      <x:c r="T73" s="21"/>
       <x:c r="U73" s="21"/>
       <x:c r="V73" s="21"/>
-      <x:c r="W73" s="18"/>
-      <x:c r="X73" s="18"/>
-      <x:c r="Y73" s="18"/>
-      <x:c r="Z73" s="18"/>
+      <x:c r="W73" s="21"/>
+      <x:c r="X73" s="21"/>
+      <x:c r="Y73" s="21"/>
+      <x:c r="Z73" s="21"/>
       <x:c r="AA73" s="18"/>
+      <x:c r="AB73" s="18"/>
+      <x:c r="AC73" s="18"/>
+      <x:c r="AD73" s="18"/>
+      <x:c r="AE73" s="18"/>
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="18"/>
@@ -2706,15 +3018,19 @@
       <x:c r="P74" s="18"/>
       <x:c r="Q74" s="18"/>
       <x:c r="R74" s="18"/>
-      <x:c r="S74" s="18"/>
-      <x:c r="T74" s="18"/>
+      <x:c r="S74" s="21"/>
+      <x:c r="T74" s="21"/>
       <x:c r="U74" s="21"/>
       <x:c r="V74" s="21"/>
-      <x:c r="W74" s="18"/>
-      <x:c r="X74" s="18"/>
-      <x:c r="Y74" s="18"/>
-      <x:c r="Z74" s="18"/>
+      <x:c r="W74" s="21"/>
+      <x:c r="X74" s="21"/>
+      <x:c r="Y74" s="21"/>
+      <x:c r="Z74" s="21"/>
       <x:c r="AA74" s="18"/>
+      <x:c r="AB74" s="18"/>
+      <x:c r="AC74" s="18"/>
+      <x:c r="AD74" s="18"/>
+      <x:c r="AE74" s="18"/>
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="18"/>
@@ -2735,15 +3051,19 @@
       <x:c r="P75" s="18"/>
       <x:c r="Q75" s="18"/>
       <x:c r="R75" s="18"/>
-      <x:c r="S75" s="18"/>
-      <x:c r="T75" s="18"/>
+      <x:c r="S75" s="21"/>
+      <x:c r="T75" s="21"/>
       <x:c r="U75" s="21"/>
       <x:c r="V75" s="21"/>
-      <x:c r="W75" s="18"/>
-      <x:c r="X75" s="18"/>
-      <x:c r="Y75" s="18"/>
-      <x:c r="Z75" s="18"/>
+      <x:c r="W75" s="21"/>
+      <x:c r="X75" s="21"/>
+      <x:c r="Y75" s="21"/>
+      <x:c r="Z75" s="21"/>
       <x:c r="AA75" s="18"/>
+      <x:c r="AB75" s="18"/>
+      <x:c r="AC75" s="18"/>
+      <x:c r="AD75" s="18"/>
+      <x:c r="AE75" s="18"/>
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="18"/>
@@ -2764,15 +3084,19 @@
       <x:c r="P76" s="18"/>
       <x:c r="Q76" s="18"/>
       <x:c r="R76" s="18"/>
-      <x:c r="S76" s="18"/>
-      <x:c r="T76" s="18"/>
+      <x:c r="S76" s="21"/>
+      <x:c r="T76" s="21"/>
       <x:c r="U76" s="21"/>
       <x:c r="V76" s="21"/>
-      <x:c r="W76" s="18"/>
-      <x:c r="X76" s="18"/>
-      <x:c r="Y76" s="18"/>
-      <x:c r="Z76" s="18"/>
+      <x:c r="W76" s="21"/>
+      <x:c r="X76" s="21"/>
+      <x:c r="Y76" s="21"/>
+      <x:c r="Z76" s="21"/>
       <x:c r="AA76" s="18"/>
+      <x:c r="AB76" s="18"/>
+      <x:c r="AC76" s="18"/>
+      <x:c r="AD76" s="18"/>
+      <x:c r="AE76" s="18"/>
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="18"/>
@@ -2793,15 +3117,19 @@
       <x:c r="P77" s="18"/>
       <x:c r="Q77" s="18"/>
       <x:c r="R77" s="18"/>
-      <x:c r="S77" s="18"/>
-      <x:c r="T77" s="18"/>
+      <x:c r="S77" s="21"/>
+      <x:c r="T77" s="21"/>
       <x:c r="U77" s="21"/>
       <x:c r="V77" s="21"/>
-      <x:c r="W77" s="18"/>
-      <x:c r="X77" s="18"/>
-      <x:c r="Y77" s="18"/>
-      <x:c r="Z77" s="18"/>
+      <x:c r="W77" s="21"/>
+      <x:c r="X77" s="21"/>
+      <x:c r="Y77" s="21"/>
+      <x:c r="Z77" s="21"/>
       <x:c r="AA77" s="18"/>
+      <x:c r="AB77" s="18"/>
+      <x:c r="AC77" s="18"/>
+      <x:c r="AD77" s="18"/>
+      <x:c r="AE77" s="18"/>
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="18"/>
@@ -2822,15 +3150,19 @@
       <x:c r="P78" s="18"/>
       <x:c r="Q78" s="18"/>
       <x:c r="R78" s="18"/>
-      <x:c r="S78" s="18"/>
-      <x:c r="T78" s="18"/>
+      <x:c r="S78" s="21"/>
+      <x:c r="T78" s="21"/>
       <x:c r="U78" s="21"/>
       <x:c r="V78" s="21"/>
-      <x:c r="W78" s="18"/>
-      <x:c r="X78" s="18"/>
-      <x:c r="Y78" s="18"/>
-      <x:c r="Z78" s="18"/>
+      <x:c r="W78" s="21"/>
+      <x:c r="X78" s="21"/>
+      <x:c r="Y78" s="21"/>
+      <x:c r="Z78" s="21"/>
       <x:c r="AA78" s="18"/>
+      <x:c r="AB78" s="18"/>
+      <x:c r="AC78" s="18"/>
+      <x:c r="AD78" s="18"/>
+      <x:c r="AE78" s="18"/>
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="18"/>
@@ -2851,15 +3183,19 @@
       <x:c r="P79" s="18"/>
       <x:c r="Q79" s="18"/>
       <x:c r="R79" s="18"/>
-      <x:c r="S79" s="18"/>
-      <x:c r="T79" s="18"/>
+      <x:c r="S79" s="21"/>
+      <x:c r="T79" s="21"/>
       <x:c r="U79" s="21"/>
       <x:c r="V79" s="21"/>
-      <x:c r="W79" s="18"/>
-      <x:c r="X79" s="18"/>
-      <x:c r="Y79" s="18"/>
-      <x:c r="Z79" s="18"/>
+      <x:c r="W79" s="21"/>
+      <x:c r="X79" s="21"/>
+      <x:c r="Y79" s="21"/>
+      <x:c r="Z79" s="21"/>
       <x:c r="AA79" s="18"/>
+      <x:c r="AB79" s="18"/>
+      <x:c r="AC79" s="18"/>
+      <x:c r="AD79" s="18"/>
+      <x:c r="AE79" s="18"/>
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="18"/>
@@ -2880,15 +3216,19 @@
       <x:c r="P80" s="18"/>
       <x:c r="Q80" s="18"/>
       <x:c r="R80" s="18"/>
-      <x:c r="S80" s="18"/>
-      <x:c r="T80" s="18"/>
+      <x:c r="S80" s="21"/>
+      <x:c r="T80" s="21"/>
       <x:c r="U80" s="21"/>
       <x:c r="V80" s="21"/>
-      <x:c r="W80" s="18"/>
-      <x:c r="X80" s="18"/>
-      <x:c r="Y80" s="18"/>
-      <x:c r="Z80" s="18"/>
+      <x:c r="W80" s="21"/>
+      <x:c r="X80" s="21"/>
+      <x:c r="Y80" s="21"/>
+      <x:c r="Z80" s="21"/>
       <x:c r="AA80" s="18"/>
+      <x:c r="AB80" s="18"/>
+      <x:c r="AC80" s="18"/>
+      <x:c r="AD80" s="18"/>
+      <x:c r="AE80" s="18"/>
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="18"/>
@@ -2909,15 +3249,19 @@
       <x:c r="P81" s="18"/>
       <x:c r="Q81" s="18"/>
       <x:c r="R81" s="18"/>
-      <x:c r="S81" s="18"/>
-      <x:c r="T81" s="18"/>
+      <x:c r="S81" s="21"/>
+      <x:c r="T81" s="21"/>
       <x:c r="U81" s="21"/>
       <x:c r="V81" s="21"/>
-      <x:c r="W81" s="18"/>
-      <x:c r="X81" s="18"/>
-      <x:c r="Y81" s="18"/>
-      <x:c r="Z81" s="18"/>
+      <x:c r="W81" s="21"/>
+      <x:c r="X81" s="21"/>
+      <x:c r="Y81" s="21"/>
+      <x:c r="Z81" s="21"/>
       <x:c r="AA81" s="18"/>
+      <x:c r="AB81" s="18"/>
+      <x:c r="AC81" s="18"/>
+      <x:c r="AD81" s="18"/>
+      <x:c r="AE81" s="18"/>
     </x:row>
     <x:row r="82">
       <x:c r="A82" s="18"/>
@@ -2938,15 +3282,19 @@
       <x:c r="P82" s="18"/>
       <x:c r="Q82" s="18"/>
       <x:c r="R82" s="18"/>
-      <x:c r="S82" s="18"/>
-      <x:c r="T82" s="18"/>
+      <x:c r="S82" s="21"/>
+      <x:c r="T82" s="21"/>
       <x:c r="U82" s="21"/>
       <x:c r="V82" s="21"/>
-      <x:c r="W82" s="18"/>
-      <x:c r="X82" s="18"/>
-      <x:c r="Y82" s="18"/>
-      <x:c r="Z82" s="18"/>
+      <x:c r="W82" s="21"/>
+      <x:c r="X82" s="21"/>
+      <x:c r="Y82" s="21"/>
+      <x:c r="Z82" s="21"/>
       <x:c r="AA82" s="18"/>
+      <x:c r="AB82" s="18"/>
+      <x:c r="AC82" s="18"/>
+      <x:c r="AD82" s="18"/>
+      <x:c r="AE82" s="18"/>
     </x:row>
     <x:row r="83">
       <x:c r="A83" s="18"/>
@@ -2967,15 +3315,19 @@
       <x:c r="P83" s="18"/>
       <x:c r="Q83" s="18"/>
       <x:c r="R83" s="18"/>
-      <x:c r="S83" s="18"/>
-      <x:c r="T83" s="18"/>
+      <x:c r="S83" s="21"/>
+      <x:c r="T83" s="21"/>
       <x:c r="U83" s="21"/>
       <x:c r="V83" s="21"/>
-      <x:c r="W83" s="18"/>
-      <x:c r="X83" s="18"/>
-      <x:c r="Y83" s="18"/>
-      <x:c r="Z83" s="18"/>
+      <x:c r="W83" s="21"/>
+      <x:c r="X83" s="21"/>
+      <x:c r="Y83" s="21"/>
+      <x:c r="Z83" s="21"/>
       <x:c r="AA83" s="18"/>
+      <x:c r="AB83" s="18"/>
+      <x:c r="AC83" s="18"/>
+      <x:c r="AD83" s="18"/>
+      <x:c r="AE83" s="18"/>
     </x:row>
     <x:row r="84">
       <x:c r="A84" s="18"/>
@@ -2996,15 +3348,19 @@
       <x:c r="P84" s="18"/>
       <x:c r="Q84" s="18"/>
       <x:c r="R84" s="18"/>
-      <x:c r="S84" s="18"/>
-      <x:c r="T84" s="18"/>
+      <x:c r="S84" s="21"/>
+      <x:c r="T84" s="21"/>
       <x:c r="U84" s="21"/>
       <x:c r="V84" s="21"/>
-      <x:c r="W84" s="18"/>
-      <x:c r="X84" s="18"/>
-      <x:c r="Y84" s="18"/>
-      <x:c r="Z84" s="18"/>
+      <x:c r="W84" s="21"/>
+      <x:c r="X84" s="21"/>
+      <x:c r="Y84" s="21"/>
+      <x:c r="Z84" s="21"/>
       <x:c r="AA84" s="18"/>
+      <x:c r="AB84" s="18"/>
+      <x:c r="AC84" s="18"/>
+      <x:c r="AD84" s="18"/>
+      <x:c r="AE84" s="18"/>
     </x:row>
     <x:row r="85">
       <x:c r="A85" s="18"/>
@@ -3025,15 +3381,19 @@
       <x:c r="P85" s="18"/>
       <x:c r="Q85" s="18"/>
       <x:c r="R85" s="18"/>
-      <x:c r="S85" s="18"/>
-      <x:c r="T85" s="18"/>
+      <x:c r="S85" s="21"/>
+      <x:c r="T85" s="21"/>
       <x:c r="U85" s="21"/>
       <x:c r="V85" s="21"/>
-      <x:c r="W85" s="18"/>
-      <x:c r="X85" s="18"/>
-      <x:c r="Y85" s="18"/>
-      <x:c r="Z85" s="18"/>
+      <x:c r="W85" s="21"/>
+      <x:c r="X85" s="21"/>
+      <x:c r="Y85" s="21"/>
+      <x:c r="Z85" s="21"/>
       <x:c r="AA85" s="18"/>
+      <x:c r="AB85" s="18"/>
+      <x:c r="AC85" s="18"/>
+      <x:c r="AD85" s="18"/>
+      <x:c r="AE85" s="18"/>
     </x:row>
     <x:row r="86">
       <x:c r="A86" s="18"/>
@@ -3054,15 +3414,19 @@
       <x:c r="P86" s="18"/>
       <x:c r="Q86" s="18"/>
       <x:c r="R86" s="18"/>
-      <x:c r="S86" s="18"/>
-      <x:c r="T86" s="18"/>
+      <x:c r="S86" s="21"/>
+      <x:c r="T86" s="21"/>
       <x:c r="U86" s="21"/>
       <x:c r="V86" s="21"/>
-      <x:c r="W86" s="18"/>
-      <x:c r="X86" s="18"/>
-      <x:c r="Y86" s="18"/>
-      <x:c r="Z86" s="18"/>
+      <x:c r="W86" s="21"/>
+      <x:c r="X86" s="21"/>
+      <x:c r="Y86" s="21"/>
+      <x:c r="Z86" s="21"/>
       <x:c r="AA86" s="18"/>
+      <x:c r="AB86" s="18"/>
+      <x:c r="AC86" s="18"/>
+      <x:c r="AD86" s="18"/>
+      <x:c r="AE86" s="18"/>
     </x:row>
     <x:row r="87">
       <x:c r="A87" s="18"/>
@@ -3083,15 +3447,19 @@
       <x:c r="P87" s="18"/>
       <x:c r="Q87" s="18"/>
       <x:c r="R87" s="18"/>
-      <x:c r="S87" s="18"/>
-      <x:c r="T87" s="18"/>
+      <x:c r="S87" s="21"/>
+      <x:c r="T87" s="21"/>
       <x:c r="U87" s="21"/>
       <x:c r="V87" s="21"/>
-      <x:c r="W87" s="18"/>
-      <x:c r="X87" s="18"/>
-      <x:c r="Y87" s="18"/>
-      <x:c r="Z87" s="18"/>
+      <x:c r="W87" s="21"/>
+      <x:c r="X87" s="21"/>
+      <x:c r="Y87" s="21"/>
+      <x:c r="Z87" s="21"/>
       <x:c r="AA87" s="18"/>
+      <x:c r="AB87" s="18"/>
+      <x:c r="AC87" s="18"/>
+      <x:c r="AD87" s="18"/>
+      <x:c r="AE87" s="18"/>
     </x:row>
     <x:row r="88">
       <x:c r="A88" s="18"/>
@@ -3112,15 +3480,19 @@
       <x:c r="P88" s="18"/>
       <x:c r="Q88" s="18"/>
       <x:c r="R88" s="18"/>
-      <x:c r="S88" s="18"/>
-      <x:c r="T88" s="18"/>
+      <x:c r="S88" s="21"/>
+      <x:c r="T88" s="21"/>
       <x:c r="U88" s="21"/>
       <x:c r="V88" s="21"/>
-      <x:c r="W88" s="18"/>
-      <x:c r="X88" s="18"/>
-      <x:c r="Y88" s="18"/>
-      <x:c r="Z88" s="18"/>
+      <x:c r="W88" s="21"/>
+      <x:c r="X88" s="21"/>
+      <x:c r="Y88" s="21"/>
+      <x:c r="Z88" s="21"/>
       <x:c r="AA88" s="18"/>
+      <x:c r="AB88" s="18"/>
+      <x:c r="AC88" s="18"/>
+      <x:c r="AD88" s="18"/>
+      <x:c r="AE88" s="18"/>
     </x:row>
     <x:row r="89">
       <x:c r="A89" s="18"/>
@@ -3141,15 +3513,19 @@
       <x:c r="P89" s="18"/>
       <x:c r="Q89" s="18"/>
       <x:c r="R89" s="18"/>
-      <x:c r="S89" s="18"/>
-      <x:c r="T89" s="18"/>
+      <x:c r="S89" s="21"/>
+      <x:c r="T89" s="21"/>
       <x:c r="U89" s="21"/>
       <x:c r="V89" s="21"/>
-      <x:c r="W89" s="18"/>
-      <x:c r="X89" s="18"/>
-      <x:c r="Y89" s="18"/>
-      <x:c r="Z89" s="18"/>
+      <x:c r="W89" s="21"/>
+      <x:c r="X89" s="21"/>
+      <x:c r="Y89" s="21"/>
+      <x:c r="Z89" s="21"/>
       <x:c r="AA89" s="18"/>
+      <x:c r="AB89" s="18"/>
+      <x:c r="AC89" s="18"/>
+      <x:c r="AD89" s="18"/>
+      <x:c r="AE89" s="18"/>
     </x:row>
     <x:row r="90">
       <x:c r="A90" s="18"/>
@@ -3170,15 +3546,19 @@
       <x:c r="P90" s="18"/>
       <x:c r="Q90" s="18"/>
       <x:c r="R90" s="18"/>
-      <x:c r="S90" s="18"/>
-      <x:c r="T90" s="18"/>
+      <x:c r="S90" s="21"/>
+      <x:c r="T90" s="21"/>
       <x:c r="U90" s="21"/>
       <x:c r="V90" s="21"/>
-      <x:c r="W90" s="18"/>
-      <x:c r="X90" s="18"/>
-      <x:c r="Y90" s="18"/>
-      <x:c r="Z90" s="18"/>
+      <x:c r="W90" s="21"/>
+      <x:c r="X90" s="21"/>
+      <x:c r="Y90" s="21"/>
+      <x:c r="Z90" s="21"/>
       <x:c r="AA90" s="18"/>
+      <x:c r="AB90" s="18"/>
+      <x:c r="AC90" s="18"/>
+      <x:c r="AD90" s="18"/>
+      <x:c r="AE90" s="18"/>
     </x:row>
     <x:row r="91">
       <x:c r="A91" s="18"/>
@@ -3199,15 +3579,19 @@
       <x:c r="P91" s="18"/>
       <x:c r="Q91" s="18"/>
       <x:c r="R91" s="18"/>
-      <x:c r="S91" s="18"/>
-      <x:c r="T91" s="18"/>
+      <x:c r="S91" s="21"/>
+      <x:c r="T91" s="21"/>
       <x:c r="U91" s="21"/>
       <x:c r="V91" s="21"/>
-      <x:c r="W91" s="18"/>
-      <x:c r="X91" s="18"/>
-      <x:c r="Y91" s="18"/>
-      <x:c r="Z91" s="18"/>
+      <x:c r="W91" s="21"/>
+      <x:c r="X91" s="21"/>
+      <x:c r="Y91" s="21"/>
+      <x:c r="Z91" s="21"/>
       <x:c r="AA91" s="18"/>
+      <x:c r="AB91" s="18"/>
+      <x:c r="AC91" s="18"/>
+      <x:c r="AD91" s="18"/>
+      <x:c r="AE91" s="18"/>
     </x:row>
     <x:row r="92">
       <x:c r="A92" s="18"/>
@@ -3228,15 +3612,19 @@
       <x:c r="P92" s="18"/>
       <x:c r="Q92" s="18"/>
       <x:c r="R92" s="18"/>
-      <x:c r="S92" s="18"/>
-      <x:c r="T92" s="18"/>
+      <x:c r="S92" s="21"/>
+      <x:c r="T92" s="21"/>
       <x:c r="U92" s="21"/>
       <x:c r="V92" s="21"/>
-      <x:c r="W92" s="18"/>
-      <x:c r="X92" s="18"/>
-      <x:c r="Y92" s="18"/>
-      <x:c r="Z92" s="18"/>
+      <x:c r="W92" s="21"/>
+      <x:c r="X92" s="21"/>
+      <x:c r="Y92" s="21"/>
+      <x:c r="Z92" s="21"/>
       <x:c r="AA92" s="18"/>
+      <x:c r="AB92" s="18"/>
+      <x:c r="AC92" s="18"/>
+      <x:c r="AD92" s="18"/>
+      <x:c r="AE92" s="18"/>
     </x:row>
     <x:row r="93">
       <x:c r="A93" s="18"/>
@@ -3257,15 +3645,19 @@
       <x:c r="P93" s="18"/>
       <x:c r="Q93" s="18"/>
       <x:c r="R93" s="18"/>
-      <x:c r="S93" s="18"/>
-      <x:c r="T93" s="18"/>
+      <x:c r="S93" s="21"/>
+      <x:c r="T93" s="21"/>
       <x:c r="U93" s="21"/>
       <x:c r="V93" s="21"/>
-      <x:c r="W93" s="18"/>
-      <x:c r="X93" s="18"/>
-      <x:c r="Y93" s="18"/>
-      <x:c r="Z93" s="18"/>
+      <x:c r="W93" s="21"/>
+      <x:c r="X93" s="21"/>
+      <x:c r="Y93" s="21"/>
+      <x:c r="Z93" s="21"/>
       <x:c r="AA93" s="18"/>
+      <x:c r="AB93" s="18"/>
+      <x:c r="AC93" s="18"/>
+      <x:c r="AD93" s="18"/>
+      <x:c r="AE93" s="18"/>
     </x:row>
     <x:row r="94">
       <x:c r="A94" s="18"/>
@@ -3286,15 +3678,19 @@
       <x:c r="P94" s="18"/>
       <x:c r="Q94" s="18"/>
       <x:c r="R94" s="18"/>
-      <x:c r="S94" s="18"/>
-      <x:c r="T94" s="18"/>
+      <x:c r="S94" s="21"/>
+      <x:c r="T94" s="21"/>
       <x:c r="U94" s="21"/>
       <x:c r="V94" s="21"/>
-      <x:c r="W94" s="18"/>
-      <x:c r="X94" s="18"/>
-      <x:c r="Y94" s="18"/>
-      <x:c r="Z94" s="18"/>
+      <x:c r="W94" s="21"/>
+      <x:c r="X94" s="21"/>
+      <x:c r="Y94" s="21"/>
+      <x:c r="Z94" s="21"/>
       <x:c r="AA94" s="18"/>
+      <x:c r="AB94" s="18"/>
+      <x:c r="AC94" s="18"/>
+      <x:c r="AD94" s="18"/>
+      <x:c r="AE94" s="18"/>
     </x:row>
     <x:row r="95">
       <x:c r="A95" s="18"/>
@@ -3315,15 +3711,19 @@
       <x:c r="P95" s="18"/>
       <x:c r="Q95" s="18"/>
       <x:c r="R95" s="18"/>
-      <x:c r="S95" s="18"/>
-      <x:c r="T95" s="18"/>
+      <x:c r="S95" s="21"/>
+      <x:c r="T95" s="21"/>
       <x:c r="U95" s="21"/>
       <x:c r="V95" s="21"/>
-      <x:c r="W95" s="18"/>
-      <x:c r="X95" s="18"/>
-      <x:c r="Y95" s="18"/>
-      <x:c r="Z95" s="18"/>
+      <x:c r="W95" s="21"/>
+      <x:c r="X95" s="21"/>
+      <x:c r="Y95" s="21"/>
+      <x:c r="Z95" s="21"/>
       <x:c r="AA95" s="18"/>
+      <x:c r="AB95" s="18"/>
+      <x:c r="AC95" s="18"/>
+      <x:c r="AD95" s="18"/>
+      <x:c r="AE95" s="18"/>
     </x:row>
     <x:row r="96">
       <x:c r="A96" s="18"/>
@@ -3344,15 +3744,19 @@
       <x:c r="P96" s="18"/>
       <x:c r="Q96" s="18"/>
       <x:c r="R96" s="18"/>
-      <x:c r="S96" s="18"/>
-      <x:c r="T96" s="18"/>
+      <x:c r="S96" s="21"/>
+      <x:c r="T96" s="21"/>
       <x:c r="U96" s="21"/>
       <x:c r="V96" s="21"/>
-      <x:c r="W96" s="18"/>
-      <x:c r="X96" s="18"/>
-      <x:c r="Y96" s="18"/>
-      <x:c r="Z96" s="18"/>
+      <x:c r="W96" s="21"/>
+      <x:c r="X96" s="21"/>
+      <x:c r="Y96" s="21"/>
+      <x:c r="Z96" s="21"/>
       <x:c r="AA96" s="18"/>
+      <x:c r="AB96" s="18"/>
+      <x:c r="AC96" s="18"/>
+      <x:c r="AD96" s="18"/>
+      <x:c r="AE96" s="18"/>
     </x:row>
     <x:row r="97">
       <x:c r="A97" s="18"/>
@@ -3373,15 +3777,19 @@
       <x:c r="P97" s="18"/>
       <x:c r="Q97" s="18"/>
       <x:c r="R97" s="18"/>
-      <x:c r="S97" s="18"/>
-      <x:c r="T97" s="18"/>
+      <x:c r="S97" s="21"/>
+      <x:c r="T97" s="21"/>
       <x:c r="U97" s="21"/>
       <x:c r="V97" s="21"/>
-      <x:c r="W97" s="18"/>
-      <x:c r="X97" s="18"/>
-      <x:c r="Y97" s="18"/>
-      <x:c r="Z97" s="18"/>
+      <x:c r="W97" s="21"/>
+      <x:c r="X97" s="21"/>
+      <x:c r="Y97" s="21"/>
+      <x:c r="Z97" s="21"/>
       <x:c r="AA97" s="18"/>
+      <x:c r="AB97" s="18"/>
+      <x:c r="AC97" s="18"/>
+      <x:c r="AD97" s="18"/>
+      <x:c r="AE97" s="18"/>
     </x:row>
     <x:row r="98">
       <x:c r="A98" s="18"/>
@@ -3402,15 +3810,19 @@
       <x:c r="P98" s="18"/>
       <x:c r="Q98" s="18"/>
       <x:c r="R98" s="18"/>
-      <x:c r="S98" s="18"/>
-      <x:c r="T98" s="18"/>
+      <x:c r="S98" s="21"/>
+      <x:c r="T98" s="21"/>
       <x:c r="U98" s="21"/>
       <x:c r="V98" s="21"/>
-      <x:c r="W98" s="18"/>
-      <x:c r="X98" s="18"/>
-      <x:c r="Y98" s="18"/>
-      <x:c r="Z98" s="18"/>
+      <x:c r="W98" s="21"/>
+      <x:c r="X98" s="21"/>
+      <x:c r="Y98" s="21"/>
+      <x:c r="Z98" s="21"/>
       <x:c r="AA98" s="18"/>
+      <x:c r="AB98" s="18"/>
+      <x:c r="AC98" s="18"/>
+      <x:c r="AD98" s="18"/>
+      <x:c r="AE98" s="18"/>
     </x:row>
     <x:row r="99">
       <x:c r="A99" s="18"/>
@@ -3431,15 +3843,19 @@
       <x:c r="P99" s="18"/>
       <x:c r="Q99" s="18"/>
       <x:c r="R99" s="18"/>
-      <x:c r="S99" s="18"/>
-      <x:c r="T99" s="18"/>
+      <x:c r="S99" s="21"/>
+      <x:c r="T99" s="21"/>
       <x:c r="U99" s="21"/>
       <x:c r="V99" s="21"/>
-      <x:c r="W99" s="18"/>
-      <x:c r="X99" s="18"/>
-      <x:c r="Y99" s="18"/>
-      <x:c r="Z99" s="18"/>
+      <x:c r="W99" s="21"/>
+      <x:c r="X99" s="21"/>
+      <x:c r="Y99" s="21"/>
+      <x:c r="Z99" s="21"/>
       <x:c r="AA99" s="18"/>
+      <x:c r="AB99" s="18"/>
+      <x:c r="AC99" s="18"/>
+      <x:c r="AD99" s="18"/>
+      <x:c r="AE99" s="18"/>
     </x:row>
     <x:row r="100">
       <x:c r="A100" s="18"/>
@@ -3460,15 +3876,19 @@
       <x:c r="P100" s="18"/>
       <x:c r="Q100" s="18"/>
       <x:c r="R100" s="18"/>
-      <x:c r="S100" s="18"/>
-      <x:c r="T100" s="18"/>
+      <x:c r="S100" s="21"/>
+      <x:c r="T100" s="21"/>
       <x:c r="U100" s="21"/>
       <x:c r="V100" s="21"/>
-      <x:c r="W100" s="18"/>
-      <x:c r="X100" s="18"/>
-      <x:c r="Y100" s="18"/>
-      <x:c r="Z100" s="18"/>
+      <x:c r="W100" s="21"/>
+      <x:c r="X100" s="21"/>
+      <x:c r="Y100" s="21"/>
+      <x:c r="Z100" s="21"/>
       <x:c r="AA100" s="18"/>
+      <x:c r="AB100" s="18"/>
+      <x:c r="AC100" s="18"/>
+      <x:c r="AD100" s="18"/>
+      <x:c r="AE100" s="18"/>
     </x:row>
     <x:row r="101">
       <x:c r="A101" s="22"/>
@@ -3489,15 +3909,19 @@
       <x:c r="P101" s="22"/>
       <x:c r="Q101" s="22"/>
       <x:c r="R101" s="22"/>
-      <x:c r="S101" s="22"/>
-      <x:c r="T101" s="22"/>
+      <x:c r="S101" s="25"/>
+      <x:c r="T101" s="25"/>
       <x:c r="U101" s="25"/>
       <x:c r="V101" s="25"/>
-      <x:c r="W101" s="22"/>
-      <x:c r="X101" s="22"/>
-      <x:c r="Y101" s="22"/>
-      <x:c r="Z101" s="22"/>
+      <x:c r="W101" s="25"/>
+      <x:c r="X101" s="25"/>
+      <x:c r="Y101" s="25"/>
+      <x:c r="Z101" s="25"/>
       <x:c r="AA101" s="22"/>
+      <x:c r="AB101" s="22"/>
+      <x:c r="AC101" s="22"/>
+      <x:c r="AD101" s="22"/>
+      <x:c r="AE101" s="22"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="3">
@@ -3507,7 +3931,7 @@
     <x:dataValidation type="list" sqref="L2:L101">
       <x:formula1>"in_stock,out_of_stock,pre_order"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="AA2:AA101">
+    <x:dataValidation type="list" sqref="AE2:AE101">
       <x:formula1>"draft"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -3660,7 +4084,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B9" s="37" t="str">
-        <x:v>Use Product Dimensions and Package Dimensions as readable text, including units.</x:v>
+        <x:v>Enter all length, width and height values as numbers in cm; enter net and gross weight as numbers in kg.</x:v>
       </x:c>
     </x:row>
     <x:row r="10">

</xml_diff>

<commit_message>
Connect product dimensions to shipping quotes (#32)
</commit_message>
<xml_diff>
--- a/public/templates/reach-projector-product-import.xlsx
+++ b/public/templates/reach-projector-product-import.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R4fb2e531aad949a5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Specifications" sheetId="2" r:id="R0c68aa6d18a04313"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="3" r:id="R33faa2e2ceb14b6b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R4db6ecbf6ad04fb2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Specifications" sheetId="2" r:id="R8d33d1b4d36d4ea3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="3" r:id="R88b8b34c0c2d495a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -455,11 +455,15 @@
     <x:col min="20" max="20" width="18" hidden="0" customWidth="1"/>
     <x:col min="21" max="21" width="18" hidden="0" customWidth="1"/>
     <x:col min="22" max="22" width="18" hidden="0" customWidth="1"/>
-    <x:col min="23" max="23" width="42" hidden="0" customWidth="1"/>
-    <x:col min="24" max="24" width="42" hidden="0" customWidth="1"/>
-    <x:col min="25" max="25" width="36" hidden="0" customWidth="1"/>
-    <x:col min="26" max="26" width="36" hidden="0" customWidth="1"/>
-    <x:col min="27" max="27" width="18" hidden="0" customWidth="1"/>
+    <x:col min="23" max="23" width="18" hidden="0" customWidth="1"/>
+    <x:col min="24" max="24" width="18" hidden="0" customWidth="1"/>
+    <x:col min="25" max="25" width="18" hidden="0" customWidth="1"/>
+    <x:col min="26" max="26" width="18" hidden="0" customWidth="1"/>
+    <x:col min="27" max="27" width="42" hidden="0" customWidth="1"/>
+    <x:col min="28" max="28" width="42" hidden="0" customWidth="1"/>
+    <x:col min="29" max="29" width="36" hidden="0" customWidth="1"/>
+    <x:col min="30" max="30" width="36" hidden="0" customWidth="1"/>
+    <x:col min="31" max="31" width="18" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
@@ -518,30 +522,42 @@
         <x:v>Country of Origin</x:v>
       </x:c>
       <x:c r="S1" s="13" t="str">
-        <x:v>Product Dimensions</x:v>
+        <x:v>Product Length (cm)</x:v>
       </x:c>
       <x:c r="T1" s="13" t="str">
-        <x:v>Package Dimensions</x:v>
+        <x:v>Product Width (cm)</x:v>
       </x:c>
       <x:c r="U1" s="13" t="str">
+        <x:v>Product Height (cm)</x:v>
+      </x:c>
+      <x:c r="V1" s="13" t="str">
+        <x:v>Package Length (cm)</x:v>
+      </x:c>
+      <x:c r="W1" s="13" t="str">
+        <x:v>Package Width (cm)</x:v>
+      </x:c>
+      <x:c r="X1" s="13" t="str">
+        <x:v>Package Height (cm)</x:v>
+      </x:c>
+      <x:c r="Y1" s="13" t="str">
         <x:v>Net Weight (kg)</x:v>
       </x:c>
-      <x:c r="V1" s="13" t="str">
+      <x:c r="Z1" s="13" t="str">
         <x:v>Gross Weight (kg)</x:v>
       </x:c>
-      <x:c r="W1" s="13" t="str">
+      <x:c r="AA1" s="13" t="str">
         <x:v>Short Description</x:v>
       </x:c>
-      <x:c r="X1" s="13" t="str">
+      <x:c r="AB1" s="13" t="str">
         <x:v>Full Description</x:v>
       </x:c>
-      <x:c r="Y1" s="13" t="str">
+      <x:c r="AC1" s="13" t="str">
         <x:v>SEO Title</x:v>
       </x:c>
-      <x:c r="Z1" s="13" t="str">
+      <x:c r="AD1" s="13" t="str">
         <x:v>Meta Description</x:v>
       </x:c>
-      <x:c r="AA1" s="13" t="str">
+      <x:c r="AE1" s="13" t="str">
         <x:v>Product Status</x:v>
       </x:c>
     </x:row>
@@ -600,31 +616,43 @@
       <x:c r="R2" s="14" t="str">
         <x:v>China</x:v>
       </x:c>
-      <x:c r="S2" s="14" t="str">
-        <x:v>250 x 200 x 100 mm</x:v>
-      </x:c>
-      <x:c r="T2" s="14" t="str">
-        <x:v>350 x 300 x 200 mm</x:v>
+      <x:c r="S2" s="17" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="T2" s="17" t="n">
+        <x:v>20</x:v>
       </x:c>
       <x:c r="U2" s="17" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="V2" s="17" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="W2" s="17" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="X2" s="17" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="Y2" s="17" t="n">
         <x:v>3.2</x:v>
       </x:c>
-      <x:c r="V2" s="17" t="n">
+      <x:c r="Z2" s="17" t="n">
         <x:v>4.5</x:v>
       </x:c>
-      <x:c r="W2" s="14" t="str">
+      <x:c r="AA2" s="14" t="str">
         <x:v>Replace this example with verified product facts.</x:v>
       </x:c>
-      <x:c r="X2" s="14" t="str">
+      <x:c r="AB2" s="14" t="str">
         <x:v>Delete this row before importing.</x:v>
       </x:c>
-      <x:c r="Y2" s="14" t="str">
+      <x:c r="AC2" s="14" t="str">
         <x:v>Example Projector | Reach Projector</x:v>
       </x:c>
-      <x:c r="Z2" s="14" t="str">
+      <x:c r="AD2" s="14" t="str">
         <x:v>Replace with a factual product description.</x:v>
       </x:c>
-      <x:c r="AA2" s="14" t="str">
+      <x:c r="AE2" s="14" t="str">
         <x:v>draft</x:v>
       </x:c>
     </x:row>
@@ -647,15 +675,19 @@
       <x:c r="P3" s="18"/>
       <x:c r="Q3" s="18"/>
       <x:c r="R3" s="18"/>
-      <x:c r="S3" s="18"/>
-      <x:c r="T3" s="18"/>
+      <x:c r="S3" s="21"/>
+      <x:c r="T3" s="21"/>
       <x:c r="U3" s="21"/>
       <x:c r="V3" s="21"/>
-      <x:c r="W3" s="18"/>
-      <x:c r="X3" s="18"/>
-      <x:c r="Y3" s="18"/>
-      <x:c r="Z3" s="18"/>
+      <x:c r="W3" s="21"/>
+      <x:c r="X3" s="21"/>
+      <x:c r="Y3" s="21"/>
+      <x:c r="Z3" s="21"/>
       <x:c r="AA3" s="18"/>
+      <x:c r="AB3" s="18"/>
+      <x:c r="AC3" s="18"/>
+      <x:c r="AD3" s="18"/>
+      <x:c r="AE3" s="18"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="18"/>
@@ -676,15 +708,19 @@
       <x:c r="P4" s="18"/>
       <x:c r="Q4" s="18"/>
       <x:c r="R4" s="18"/>
-      <x:c r="S4" s="18"/>
-      <x:c r="T4" s="18"/>
+      <x:c r="S4" s="21"/>
+      <x:c r="T4" s="21"/>
       <x:c r="U4" s="21"/>
       <x:c r="V4" s="21"/>
-      <x:c r="W4" s="18"/>
-      <x:c r="X4" s="18"/>
-      <x:c r="Y4" s="18"/>
-      <x:c r="Z4" s="18"/>
+      <x:c r="W4" s="21"/>
+      <x:c r="X4" s="21"/>
+      <x:c r="Y4" s="21"/>
+      <x:c r="Z4" s="21"/>
       <x:c r="AA4" s="18"/>
+      <x:c r="AB4" s="18"/>
+      <x:c r="AC4" s="18"/>
+      <x:c r="AD4" s="18"/>
+      <x:c r="AE4" s="18"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="18"/>
@@ -705,15 +741,19 @@
       <x:c r="P5" s="18"/>
       <x:c r="Q5" s="18"/>
       <x:c r="R5" s="18"/>
-      <x:c r="S5" s="18"/>
-      <x:c r="T5" s="18"/>
+      <x:c r="S5" s="21"/>
+      <x:c r="T5" s="21"/>
       <x:c r="U5" s="21"/>
       <x:c r="V5" s="21"/>
-      <x:c r="W5" s="18"/>
-      <x:c r="X5" s="18"/>
-      <x:c r="Y5" s="18"/>
-      <x:c r="Z5" s="18"/>
+      <x:c r="W5" s="21"/>
+      <x:c r="X5" s="21"/>
+      <x:c r="Y5" s="21"/>
+      <x:c r="Z5" s="21"/>
       <x:c r="AA5" s="18"/>
+      <x:c r="AB5" s="18"/>
+      <x:c r="AC5" s="18"/>
+      <x:c r="AD5" s="18"/>
+      <x:c r="AE5" s="18"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="18"/>
@@ -734,15 +774,19 @@
       <x:c r="P6" s="18"/>
       <x:c r="Q6" s="18"/>
       <x:c r="R6" s="18"/>
-      <x:c r="S6" s="18"/>
-      <x:c r="T6" s="18"/>
+      <x:c r="S6" s="21"/>
+      <x:c r="T6" s="21"/>
       <x:c r="U6" s="21"/>
       <x:c r="V6" s="21"/>
-      <x:c r="W6" s="18"/>
-      <x:c r="X6" s="18"/>
-      <x:c r="Y6" s="18"/>
-      <x:c r="Z6" s="18"/>
+      <x:c r="W6" s="21"/>
+      <x:c r="X6" s="21"/>
+      <x:c r="Y6" s="21"/>
+      <x:c r="Z6" s="21"/>
       <x:c r="AA6" s="18"/>
+      <x:c r="AB6" s="18"/>
+      <x:c r="AC6" s="18"/>
+      <x:c r="AD6" s="18"/>
+      <x:c r="AE6" s="18"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="18"/>
@@ -763,15 +807,19 @@
       <x:c r="P7" s="18"/>
       <x:c r="Q7" s="18"/>
       <x:c r="R7" s="18"/>
-      <x:c r="S7" s="18"/>
-      <x:c r="T7" s="18"/>
+      <x:c r="S7" s="21"/>
+      <x:c r="T7" s="21"/>
       <x:c r="U7" s="21"/>
       <x:c r="V7" s="21"/>
-      <x:c r="W7" s="18"/>
-      <x:c r="X7" s="18"/>
-      <x:c r="Y7" s="18"/>
-      <x:c r="Z7" s="18"/>
+      <x:c r="W7" s="21"/>
+      <x:c r="X7" s="21"/>
+      <x:c r="Y7" s="21"/>
+      <x:c r="Z7" s="21"/>
       <x:c r="AA7" s="18"/>
+      <x:c r="AB7" s="18"/>
+      <x:c r="AC7" s="18"/>
+      <x:c r="AD7" s="18"/>
+      <x:c r="AE7" s="18"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="18"/>
@@ -792,15 +840,19 @@
       <x:c r="P8" s="18"/>
       <x:c r="Q8" s="18"/>
       <x:c r="R8" s="18"/>
-      <x:c r="S8" s="18"/>
-      <x:c r="T8" s="18"/>
+      <x:c r="S8" s="21"/>
+      <x:c r="T8" s="21"/>
       <x:c r="U8" s="21"/>
       <x:c r="V8" s="21"/>
-      <x:c r="W8" s="18"/>
-      <x:c r="X8" s="18"/>
-      <x:c r="Y8" s="18"/>
-      <x:c r="Z8" s="18"/>
+      <x:c r="W8" s="21"/>
+      <x:c r="X8" s="21"/>
+      <x:c r="Y8" s="21"/>
+      <x:c r="Z8" s="21"/>
       <x:c r="AA8" s="18"/>
+      <x:c r="AB8" s="18"/>
+      <x:c r="AC8" s="18"/>
+      <x:c r="AD8" s="18"/>
+      <x:c r="AE8" s="18"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="18"/>
@@ -821,15 +873,19 @@
       <x:c r="P9" s="18"/>
       <x:c r="Q9" s="18"/>
       <x:c r="R9" s="18"/>
-      <x:c r="S9" s="18"/>
-      <x:c r="T9" s="18"/>
+      <x:c r="S9" s="21"/>
+      <x:c r="T9" s="21"/>
       <x:c r="U9" s="21"/>
       <x:c r="V9" s="21"/>
-      <x:c r="W9" s="18"/>
-      <x:c r="X9" s="18"/>
-      <x:c r="Y9" s="18"/>
-      <x:c r="Z9" s="18"/>
+      <x:c r="W9" s="21"/>
+      <x:c r="X9" s="21"/>
+      <x:c r="Y9" s="21"/>
+      <x:c r="Z9" s="21"/>
       <x:c r="AA9" s="18"/>
+      <x:c r="AB9" s="18"/>
+      <x:c r="AC9" s="18"/>
+      <x:c r="AD9" s="18"/>
+      <x:c r="AE9" s="18"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="18"/>
@@ -850,15 +906,19 @@
       <x:c r="P10" s="18"/>
       <x:c r="Q10" s="18"/>
       <x:c r="R10" s="18"/>
-      <x:c r="S10" s="18"/>
-      <x:c r="T10" s="18"/>
+      <x:c r="S10" s="21"/>
+      <x:c r="T10" s="21"/>
       <x:c r="U10" s="21"/>
       <x:c r="V10" s="21"/>
-      <x:c r="W10" s="18"/>
-      <x:c r="X10" s="18"/>
-      <x:c r="Y10" s="18"/>
-      <x:c r="Z10" s="18"/>
+      <x:c r="W10" s="21"/>
+      <x:c r="X10" s="21"/>
+      <x:c r="Y10" s="21"/>
+      <x:c r="Z10" s="21"/>
       <x:c r="AA10" s="18"/>
+      <x:c r="AB10" s="18"/>
+      <x:c r="AC10" s="18"/>
+      <x:c r="AD10" s="18"/>
+      <x:c r="AE10" s="18"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="18"/>
@@ -879,15 +939,19 @@
       <x:c r="P11" s="18"/>
       <x:c r="Q11" s="18"/>
       <x:c r="R11" s="18"/>
-      <x:c r="S11" s="18"/>
-      <x:c r="T11" s="18"/>
+      <x:c r="S11" s="21"/>
+      <x:c r="T11" s="21"/>
       <x:c r="U11" s="21"/>
       <x:c r="V11" s="21"/>
-      <x:c r="W11" s="18"/>
-      <x:c r="X11" s="18"/>
-      <x:c r="Y11" s="18"/>
-      <x:c r="Z11" s="18"/>
+      <x:c r="W11" s="21"/>
+      <x:c r="X11" s="21"/>
+      <x:c r="Y11" s="21"/>
+      <x:c r="Z11" s="21"/>
       <x:c r="AA11" s="18"/>
+      <x:c r="AB11" s="18"/>
+      <x:c r="AC11" s="18"/>
+      <x:c r="AD11" s="18"/>
+      <x:c r="AE11" s="18"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="18"/>
@@ -908,15 +972,19 @@
       <x:c r="P12" s="18"/>
       <x:c r="Q12" s="18"/>
       <x:c r="R12" s="18"/>
-      <x:c r="S12" s="18"/>
-      <x:c r="T12" s="18"/>
+      <x:c r="S12" s="21"/>
+      <x:c r="T12" s="21"/>
       <x:c r="U12" s="21"/>
       <x:c r="V12" s="21"/>
-      <x:c r="W12" s="18"/>
-      <x:c r="X12" s="18"/>
-      <x:c r="Y12" s="18"/>
-      <x:c r="Z12" s="18"/>
+      <x:c r="W12" s="21"/>
+      <x:c r="X12" s="21"/>
+      <x:c r="Y12" s="21"/>
+      <x:c r="Z12" s="21"/>
       <x:c r="AA12" s="18"/>
+      <x:c r="AB12" s="18"/>
+      <x:c r="AC12" s="18"/>
+      <x:c r="AD12" s="18"/>
+      <x:c r="AE12" s="18"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="18"/>
@@ -937,15 +1005,19 @@
       <x:c r="P13" s="18"/>
       <x:c r="Q13" s="18"/>
       <x:c r="R13" s="18"/>
-      <x:c r="S13" s="18"/>
-      <x:c r="T13" s="18"/>
+      <x:c r="S13" s="21"/>
+      <x:c r="T13" s="21"/>
       <x:c r="U13" s="21"/>
       <x:c r="V13" s="21"/>
-      <x:c r="W13" s="18"/>
-      <x:c r="X13" s="18"/>
-      <x:c r="Y13" s="18"/>
-      <x:c r="Z13" s="18"/>
+      <x:c r="W13" s="21"/>
+      <x:c r="X13" s="21"/>
+      <x:c r="Y13" s="21"/>
+      <x:c r="Z13" s="21"/>
       <x:c r="AA13" s="18"/>
+      <x:c r="AB13" s="18"/>
+      <x:c r="AC13" s="18"/>
+      <x:c r="AD13" s="18"/>
+      <x:c r="AE13" s="18"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="18"/>
@@ -966,15 +1038,19 @@
       <x:c r="P14" s="18"/>
       <x:c r="Q14" s="18"/>
       <x:c r="R14" s="18"/>
-      <x:c r="S14" s="18"/>
-      <x:c r="T14" s="18"/>
+      <x:c r="S14" s="21"/>
+      <x:c r="T14" s="21"/>
       <x:c r="U14" s="21"/>
       <x:c r="V14" s="21"/>
-      <x:c r="W14" s="18"/>
-      <x:c r="X14" s="18"/>
-      <x:c r="Y14" s="18"/>
-      <x:c r="Z14" s="18"/>
+      <x:c r="W14" s="21"/>
+      <x:c r="X14" s="21"/>
+      <x:c r="Y14" s="21"/>
+      <x:c r="Z14" s="21"/>
       <x:c r="AA14" s="18"/>
+      <x:c r="AB14" s="18"/>
+      <x:c r="AC14" s="18"/>
+      <x:c r="AD14" s="18"/>
+      <x:c r="AE14" s="18"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="18"/>
@@ -995,15 +1071,19 @@
       <x:c r="P15" s="18"/>
       <x:c r="Q15" s="18"/>
       <x:c r="R15" s="18"/>
-      <x:c r="S15" s="18"/>
-      <x:c r="T15" s="18"/>
+      <x:c r="S15" s="21"/>
+      <x:c r="T15" s="21"/>
       <x:c r="U15" s="21"/>
       <x:c r="V15" s="21"/>
-      <x:c r="W15" s="18"/>
-      <x:c r="X15" s="18"/>
-      <x:c r="Y15" s="18"/>
-      <x:c r="Z15" s="18"/>
+      <x:c r="W15" s="21"/>
+      <x:c r="X15" s="21"/>
+      <x:c r="Y15" s="21"/>
+      <x:c r="Z15" s="21"/>
       <x:c r="AA15" s="18"/>
+      <x:c r="AB15" s="18"/>
+      <x:c r="AC15" s="18"/>
+      <x:c r="AD15" s="18"/>
+      <x:c r="AE15" s="18"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="18"/>
@@ -1024,15 +1104,19 @@
       <x:c r="P16" s="18"/>
       <x:c r="Q16" s="18"/>
       <x:c r="R16" s="18"/>
-      <x:c r="S16" s="18"/>
-      <x:c r="T16" s="18"/>
+      <x:c r="S16" s="21"/>
+      <x:c r="T16" s="21"/>
       <x:c r="U16" s="21"/>
       <x:c r="V16" s="21"/>
-      <x:c r="W16" s="18"/>
-      <x:c r="X16" s="18"/>
-      <x:c r="Y16" s="18"/>
-      <x:c r="Z16" s="18"/>
+      <x:c r="W16" s="21"/>
+      <x:c r="X16" s="21"/>
+      <x:c r="Y16" s="21"/>
+      <x:c r="Z16" s="21"/>
       <x:c r="AA16" s="18"/>
+      <x:c r="AB16" s="18"/>
+      <x:c r="AC16" s="18"/>
+      <x:c r="AD16" s="18"/>
+      <x:c r="AE16" s="18"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="18"/>
@@ -1053,15 +1137,19 @@
       <x:c r="P17" s="18"/>
       <x:c r="Q17" s="18"/>
       <x:c r="R17" s="18"/>
-      <x:c r="S17" s="18"/>
-      <x:c r="T17" s="18"/>
+      <x:c r="S17" s="21"/>
+      <x:c r="T17" s="21"/>
       <x:c r="U17" s="21"/>
       <x:c r="V17" s="21"/>
-      <x:c r="W17" s="18"/>
-      <x:c r="X17" s="18"/>
-      <x:c r="Y17" s="18"/>
-      <x:c r="Z17" s="18"/>
+      <x:c r="W17" s="21"/>
+      <x:c r="X17" s="21"/>
+      <x:c r="Y17" s="21"/>
+      <x:c r="Z17" s="21"/>
       <x:c r="AA17" s="18"/>
+      <x:c r="AB17" s="18"/>
+      <x:c r="AC17" s="18"/>
+      <x:c r="AD17" s="18"/>
+      <x:c r="AE17" s="18"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="18"/>
@@ -1082,15 +1170,19 @@
       <x:c r="P18" s="18"/>
       <x:c r="Q18" s="18"/>
       <x:c r="R18" s="18"/>
-      <x:c r="S18" s="18"/>
-      <x:c r="T18" s="18"/>
+      <x:c r="S18" s="21"/>
+      <x:c r="T18" s="21"/>
       <x:c r="U18" s="21"/>
       <x:c r="V18" s="21"/>
-      <x:c r="W18" s="18"/>
-      <x:c r="X18" s="18"/>
-      <x:c r="Y18" s="18"/>
-      <x:c r="Z18" s="18"/>
+      <x:c r="W18" s="21"/>
+      <x:c r="X18" s="21"/>
+      <x:c r="Y18" s="21"/>
+      <x:c r="Z18" s="21"/>
       <x:c r="AA18" s="18"/>
+      <x:c r="AB18" s="18"/>
+      <x:c r="AC18" s="18"/>
+      <x:c r="AD18" s="18"/>
+      <x:c r="AE18" s="18"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="18"/>
@@ -1111,15 +1203,19 @@
       <x:c r="P19" s="18"/>
       <x:c r="Q19" s="18"/>
       <x:c r="R19" s="18"/>
-      <x:c r="S19" s="18"/>
-      <x:c r="T19" s="18"/>
+      <x:c r="S19" s="21"/>
+      <x:c r="T19" s="21"/>
       <x:c r="U19" s="21"/>
       <x:c r="V19" s="21"/>
-      <x:c r="W19" s="18"/>
-      <x:c r="X19" s="18"/>
-      <x:c r="Y19" s="18"/>
-      <x:c r="Z19" s="18"/>
+      <x:c r="W19" s="21"/>
+      <x:c r="X19" s="21"/>
+      <x:c r="Y19" s="21"/>
+      <x:c r="Z19" s="21"/>
       <x:c r="AA19" s="18"/>
+      <x:c r="AB19" s="18"/>
+      <x:c r="AC19" s="18"/>
+      <x:c r="AD19" s="18"/>
+      <x:c r="AE19" s="18"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="18"/>
@@ -1140,15 +1236,19 @@
       <x:c r="P20" s="18"/>
       <x:c r="Q20" s="18"/>
       <x:c r="R20" s="18"/>
-      <x:c r="S20" s="18"/>
-      <x:c r="T20" s="18"/>
+      <x:c r="S20" s="21"/>
+      <x:c r="T20" s="21"/>
       <x:c r="U20" s="21"/>
       <x:c r="V20" s="21"/>
-      <x:c r="W20" s="18"/>
-      <x:c r="X20" s="18"/>
-      <x:c r="Y20" s="18"/>
-      <x:c r="Z20" s="18"/>
+      <x:c r="W20" s="21"/>
+      <x:c r="X20" s="21"/>
+      <x:c r="Y20" s="21"/>
+      <x:c r="Z20" s="21"/>
       <x:c r="AA20" s="18"/>
+      <x:c r="AB20" s="18"/>
+      <x:c r="AC20" s="18"/>
+      <x:c r="AD20" s="18"/>
+      <x:c r="AE20" s="18"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="18"/>
@@ -1169,15 +1269,19 @@
       <x:c r="P21" s="18"/>
       <x:c r="Q21" s="18"/>
       <x:c r="R21" s="18"/>
-      <x:c r="S21" s="18"/>
-      <x:c r="T21" s="18"/>
+      <x:c r="S21" s="21"/>
+      <x:c r="T21" s="21"/>
       <x:c r="U21" s="21"/>
       <x:c r="V21" s="21"/>
-      <x:c r="W21" s="18"/>
-      <x:c r="X21" s="18"/>
-      <x:c r="Y21" s="18"/>
-      <x:c r="Z21" s="18"/>
+      <x:c r="W21" s="21"/>
+      <x:c r="X21" s="21"/>
+      <x:c r="Y21" s="21"/>
+      <x:c r="Z21" s="21"/>
       <x:c r="AA21" s="18"/>
+      <x:c r="AB21" s="18"/>
+      <x:c r="AC21" s="18"/>
+      <x:c r="AD21" s="18"/>
+      <x:c r="AE21" s="18"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="18"/>
@@ -1198,15 +1302,19 @@
       <x:c r="P22" s="18"/>
       <x:c r="Q22" s="18"/>
       <x:c r="R22" s="18"/>
-      <x:c r="S22" s="18"/>
-      <x:c r="T22" s="18"/>
+      <x:c r="S22" s="21"/>
+      <x:c r="T22" s="21"/>
       <x:c r="U22" s="21"/>
       <x:c r="V22" s="21"/>
-      <x:c r="W22" s="18"/>
-      <x:c r="X22" s="18"/>
-      <x:c r="Y22" s="18"/>
-      <x:c r="Z22" s="18"/>
+      <x:c r="W22" s="21"/>
+      <x:c r="X22" s="21"/>
+      <x:c r="Y22" s="21"/>
+      <x:c r="Z22" s="21"/>
       <x:c r="AA22" s="18"/>
+      <x:c r="AB22" s="18"/>
+      <x:c r="AC22" s="18"/>
+      <x:c r="AD22" s="18"/>
+      <x:c r="AE22" s="18"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="18"/>
@@ -1227,15 +1335,19 @@
       <x:c r="P23" s="18"/>
       <x:c r="Q23" s="18"/>
       <x:c r="R23" s="18"/>
-      <x:c r="S23" s="18"/>
-      <x:c r="T23" s="18"/>
+      <x:c r="S23" s="21"/>
+      <x:c r="T23" s="21"/>
       <x:c r="U23" s="21"/>
       <x:c r="V23" s="21"/>
-      <x:c r="W23" s="18"/>
-      <x:c r="X23" s="18"/>
-      <x:c r="Y23" s="18"/>
-      <x:c r="Z23" s="18"/>
+      <x:c r="W23" s="21"/>
+      <x:c r="X23" s="21"/>
+      <x:c r="Y23" s="21"/>
+      <x:c r="Z23" s="21"/>
       <x:c r="AA23" s="18"/>
+      <x:c r="AB23" s="18"/>
+      <x:c r="AC23" s="18"/>
+      <x:c r="AD23" s="18"/>
+      <x:c r="AE23" s="18"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="18"/>
@@ -1256,15 +1368,19 @@
       <x:c r="P24" s="18"/>
       <x:c r="Q24" s="18"/>
       <x:c r="R24" s="18"/>
-      <x:c r="S24" s="18"/>
-      <x:c r="T24" s="18"/>
+      <x:c r="S24" s="21"/>
+      <x:c r="T24" s="21"/>
       <x:c r="U24" s="21"/>
       <x:c r="V24" s="21"/>
-      <x:c r="W24" s="18"/>
-      <x:c r="X24" s="18"/>
-      <x:c r="Y24" s="18"/>
-      <x:c r="Z24" s="18"/>
+      <x:c r="W24" s="21"/>
+      <x:c r="X24" s="21"/>
+      <x:c r="Y24" s="21"/>
+      <x:c r="Z24" s="21"/>
       <x:c r="AA24" s="18"/>
+      <x:c r="AB24" s="18"/>
+      <x:c r="AC24" s="18"/>
+      <x:c r="AD24" s="18"/>
+      <x:c r="AE24" s="18"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="18"/>
@@ -1285,15 +1401,19 @@
       <x:c r="P25" s="18"/>
       <x:c r="Q25" s="18"/>
       <x:c r="R25" s="18"/>
-      <x:c r="S25" s="18"/>
-      <x:c r="T25" s="18"/>
+      <x:c r="S25" s="21"/>
+      <x:c r="T25" s="21"/>
       <x:c r="U25" s="21"/>
       <x:c r="V25" s="21"/>
-      <x:c r="W25" s="18"/>
-      <x:c r="X25" s="18"/>
-      <x:c r="Y25" s="18"/>
-      <x:c r="Z25" s="18"/>
+      <x:c r="W25" s="21"/>
+      <x:c r="X25" s="21"/>
+      <x:c r="Y25" s="21"/>
+      <x:c r="Z25" s="21"/>
       <x:c r="AA25" s="18"/>
+      <x:c r="AB25" s="18"/>
+      <x:c r="AC25" s="18"/>
+      <x:c r="AD25" s="18"/>
+      <x:c r="AE25" s="18"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="18"/>
@@ -1314,15 +1434,19 @@
       <x:c r="P26" s="18"/>
       <x:c r="Q26" s="18"/>
       <x:c r="R26" s="18"/>
-      <x:c r="S26" s="18"/>
-      <x:c r="T26" s="18"/>
+      <x:c r="S26" s="21"/>
+      <x:c r="T26" s="21"/>
       <x:c r="U26" s="21"/>
       <x:c r="V26" s="21"/>
-      <x:c r="W26" s="18"/>
-      <x:c r="X26" s="18"/>
-      <x:c r="Y26" s="18"/>
-      <x:c r="Z26" s="18"/>
+      <x:c r="W26" s="21"/>
+      <x:c r="X26" s="21"/>
+      <x:c r="Y26" s="21"/>
+      <x:c r="Z26" s="21"/>
       <x:c r="AA26" s="18"/>
+      <x:c r="AB26" s="18"/>
+      <x:c r="AC26" s="18"/>
+      <x:c r="AD26" s="18"/>
+      <x:c r="AE26" s="18"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="18"/>
@@ -1343,15 +1467,19 @@
       <x:c r="P27" s="18"/>
       <x:c r="Q27" s="18"/>
       <x:c r="R27" s="18"/>
-      <x:c r="S27" s="18"/>
-      <x:c r="T27" s="18"/>
+      <x:c r="S27" s="21"/>
+      <x:c r="T27" s="21"/>
       <x:c r="U27" s="21"/>
       <x:c r="V27" s="21"/>
-      <x:c r="W27" s="18"/>
-      <x:c r="X27" s="18"/>
-      <x:c r="Y27" s="18"/>
-      <x:c r="Z27" s="18"/>
+      <x:c r="W27" s="21"/>
+      <x:c r="X27" s="21"/>
+      <x:c r="Y27" s="21"/>
+      <x:c r="Z27" s="21"/>
       <x:c r="AA27" s="18"/>
+      <x:c r="AB27" s="18"/>
+      <x:c r="AC27" s="18"/>
+      <x:c r="AD27" s="18"/>
+      <x:c r="AE27" s="18"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="18"/>
@@ -1372,15 +1500,19 @@
       <x:c r="P28" s="18"/>
       <x:c r="Q28" s="18"/>
       <x:c r="R28" s="18"/>
-      <x:c r="S28" s="18"/>
-      <x:c r="T28" s="18"/>
+      <x:c r="S28" s="21"/>
+      <x:c r="T28" s="21"/>
       <x:c r="U28" s="21"/>
       <x:c r="V28" s="21"/>
-      <x:c r="W28" s="18"/>
-      <x:c r="X28" s="18"/>
-      <x:c r="Y28" s="18"/>
-      <x:c r="Z28" s="18"/>
+      <x:c r="W28" s="21"/>
+      <x:c r="X28" s="21"/>
+      <x:c r="Y28" s="21"/>
+      <x:c r="Z28" s="21"/>
       <x:c r="AA28" s="18"/>
+      <x:c r="AB28" s="18"/>
+      <x:c r="AC28" s="18"/>
+      <x:c r="AD28" s="18"/>
+      <x:c r="AE28" s="18"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="18"/>
@@ -1401,15 +1533,19 @@
       <x:c r="P29" s="18"/>
       <x:c r="Q29" s="18"/>
       <x:c r="R29" s="18"/>
-      <x:c r="S29" s="18"/>
-      <x:c r="T29" s="18"/>
+      <x:c r="S29" s="21"/>
+      <x:c r="T29" s="21"/>
       <x:c r="U29" s="21"/>
       <x:c r="V29" s="21"/>
-      <x:c r="W29" s="18"/>
-      <x:c r="X29" s="18"/>
-      <x:c r="Y29" s="18"/>
-      <x:c r="Z29" s="18"/>
+      <x:c r="W29" s="21"/>
+      <x:c r="X29" s="21"/>
+      <x:c r="Y29" s="21"/>
+      <x:c r="Z29" s="21"/>
       <x:c r="AA29" s="18"/>
+      <x:c r="AB29" s="18"/>
+      <x:c r="AC29" s="18"/>
+      <x:c r="AD29" s="18"/>
+      <x:c r="AE29" s="18"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="18"/>
@@ -1430,15 +1566,19 @@
       <x:c r="P30" s="18"/>
       <x:c r="Q30" s="18"/>
       <x:c r="R30" s="18"/>
-      <x:c r="S30" s="18"/>
-      <x:c r="T30" s="18"/>
+      <x:c r="S30" s="21"/>
+      <x:c r="T30" s="21"/>
       <x:c r="U30" s="21"/>
       <x:c r="V30" s="21"/>
-      <x:c r="W30" s="18"/>
-      <x:c r="X30" s="18"/>
-      <x:c r="Y30" s="18"/>
-      <x:c r="Z30" s="18"/>
+      <x:c r="W30" s="21"/>
+      <x:c r="X30" s="21"/>
+      <x:c r="Y30" s="21"/>
+      <x:c r="Z30" s="21"/>
       <x:c r="AA30" s="18"/>
+      <x:c r="AB30" s="18"/>
+      <x:c r="AC30" s="18"/>
+      <x:c r="AD30" s="18"/>
+      <x:c r="AE30" s="18"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="18"/>
@@ -1459,15 +1599,19 @@
       <x:c r="P31" s="18"/>
       <x:c r="Q31" s="18"/>
       <x:c r="R31" s="18"/>
-      <x:c r="S31" s="18"/>
-      <x:c r="T31" s="18"/>
+      <x:c r="S31" s="21"/>
+      <x:c r="T31" s="21"/>
       <x:c r="U31" s="21"/>
       <x:c r="V31" s="21"/>
-      <x:c r="W31" s="18"/>
-      <x:c r="X31" s="18"/>
-      <x:c r="Y31" s="18"/>
-      <x:c r="Z31" s="18"/>
+      <x:c r="W31" s="21"/>
+      <x:c r="X31" s="21"/>
+      <x:c r="Y31" s="21"/>
+      <x:c r="Z31" s="21"/>
       <x:c r="AA31" s="18"/>
+      <x:c r="AB31" s="18"/>
+      <x:c r="AC31" s="18"/>
+      <x:c r="AD31" s="18"/>
+      <x:c r="AE31" s="18"/>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="18"/>
@@ -1488,15 +1632,19 @@
       <x:c r="P32" s="18"/>
       <x:c r="Q32" s="18"/>
       <x:c r="R32" s="18"/>
-      <x:c r="S32" s="18"/>
-      <x:c r="T32" s="18"/>
+      <x:c r="S32" s="21"/>
+      <x:c r="T32" s="21"/>
       <x:c r="U32" s="21"/>
       <x:c r="V32" s="21"/>
-      <x:c r="W32" s="18"/>
-      <x:c r="X32" s="18"/>
-      <x:c r="Y32" s="18"/>
-      <x:c r="Z32" s="18"/>
+      <x:c r="W32" s="21"/>
+      <x:c r="X32" s="21"/>
+      <x:c r="Y32" s="21"/>
+      <x:c r="Z32" s="21"/>
       <x:c r="AA32" s="18"/>
+      <x:c r="AB32" s="18"/>
+      <x:c r="AC32" s="18"/>
+      <x:c r="AD32" s="18"/>
+      <x:c r="AE32" s="18"/>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="18"/>
@@ -1517,15 +1665,19 @@
       <x:c r="P33" s="18"/>
       <x:c r="Q33" s="18"/>
       <x:c r="R33" s="18"/>
-      <x:c r="S33" s="18"/>
-      <x:c r="T33" s="18"/>
+      <x:c r="S33" s="21"/>
+      <x:c r="T33" s="21"/>
       <x:c r="U33" s="21"/>
       <x:c r="V33" s="21"/>
-      <x:c r="W33" s="18"/>
-      <x:c r="X33" s="18"/>
-      <x:c r="Y33" s="18"/>
-      <x:c r="Z33" s="18"/>
+      <x:c r="W33" s="21"/>
+      <x:c r="X33" s="21"/>
+      <x:c r="Y33" s="21"/>
+      <x:c r="Z33" s="21"/>
       <x:c r="AA33" s="18"/>
+      <x:c r="AB33" s="18"/>
+      <x:c r="AC33" s="18"/>
+      <x:c r="AD33" s="18"/>
+      <x:c r="AE33" s="18"/>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="18"/>
@@ -1546,15 +1698,19 @@
       <x:c r="P34" s="18"/>
       <x:c r="Q34" s="18"/>
       <x:c r="R34" s="18"/>
-      <x:c r="S34" s="18"/>
-      <x:c r="T34" s="18"/>
+      <x:c r="S34" s="21"/>
+      <x:c r="T34" s="21"/>
       <x:c r="U34" s="21"/>
       <x:c r="V34" s="21"/>
-      <x:c r="W34" s="18"/>
-      <x:c r="X34" s="18"/>
-      <x:c r="Y34" s="18"/>
-      <x:c r="Z34" s="18"/>
+      <x:c r="W34" s="21"/>
+      <x:c r="X34" s="21"/>
+      <x:c r="Y34" s="21"/>
+      <x:c r="Z34" s="21"/>
       <x:c r="AA34" s="18"/>
+      <x:c r="AB34" s="18"/>
+      <x:c r="AC34" s="18"/>
+      <x:c r="AD34" s="18"/>
+      <x:c r="AE34" s="18"/>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="18"/>
@@ -1575,15 +1731,19 @@
       <x:c r="P35" s="18"/>
       <x:c r="Q35" s="18"/>
       <x:c r="R35" s="18"/>
-      <x:c r="S35" s="18"/>
-      <x:c r="T35" s="18"/>
+      <x:c r="S35" s="21"/>
+      <x:c r="T35" s="21"/>
       <x:c r="U35" s="21"/>
       <x:c r="V35" s="21"/>
-      <x:c r="W35" s="18"/>
-      <x:c r="X35" s="18"/>
-      <x:c r="Y35" s="18"/>
-      <x:c r="Z35" s="18"/>
+      <x:c r="W35" s="21"/>
+      <x:c r="X35" s="21"/>
+      <x:c r="Y35" s="21"/>
+      <x:c r="Z35" s="21"/>
       <x:c r="AA35" s="18"/>
+      <x:c r="AB35" s="18"/>
+      <x:c r="AC35" s="18"/>
+      <x:c r="AD35" s="18"/>
+      <x:c r="AE35" s="18"/>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="18"/>
@@ -1604,15 +1764,19 @@
       <x:c r="P36" s="18"/>
       <x:c r="Q36" s="18"/>
       <x:c r="R36" s="18"/>
-      <x:c r="S36" s="18"/>
-      <x:c r="T36" s="18"/>
+      <x:c r="S36" s="21"/>
+      <x:c r="T36" s="21"/>
       <x:c r="U36" s="21"/>
       <x:c r="V36" s="21"/>
-      <x:c r="W36" s="18"/>
-      <x:c r="X36" s="18"/>
-      <x:c r="Y36" s="18"/>
-      <x:c r="Z36" s="18"/>
+      <x:c r="W36" s="21"/>
+      <x:c r="X36" s="21"/>
+      <x:c r="Y36" s="21"/>
+      <x:c r="Z36" s="21"/>
       <x:c r="AA36" s="18"/>
+      <x:c r="AB36" s="18"/>
+      <x:c r="AC36" s="18"/>
+      <x:c r="AD36" s="18"/>
+      <x:c r="AE36" s="18"/>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="18"/>
@@ -1633,15 +1797,19 @@
       <x:c r="P37" s="18"/>
       <x:c r="Q37" s="18"/>
       <x:c r="R37" s="18"/>
-      <x:c r="S37" s="18"/>
-      <x:c r="T37" s="18"/>
+      <x:c r="S37" s="21"/>
+      <x:c r="T37" s="21"/>
       <x:c r="U37" s="21"/>
       <x:c r="V37" s="21"/>
-      <x:c r="W37" s="18"/>
-      <x:c r="X37" s="18"/>
-      <x:c r="Y37" s="18"/>
-      <x:c r="Z37" s="18"/>
+      <x:c r="W37" s="21"/>
+      <x:c r="X37" s="21"/>
+      <x:c r="Y37" s="21"/>
+      <x:c r="Z37" s="21"/>
       <x:c r="AA37" s="18"/>
+      <x:c r="AB37" s="18"/>
+      <x:c r="AC37" s="18"/>
+      <x:c r="AD37" s="18"/>
+      <x:c r="AE37" s="18"/>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="18"/>
@@ -1662,15 +1830,19 @@
       <x:c r="P38" s="18"/>
       <x:c r="Q38" s="18"/>
       <x:c r="R38" s="18"/>
-      <x:c r="S38" s="18"/>
-      <x:c r="T38" s="18"/>
+      <x:c r="S38" s="21"/>
+      <x:c r="T38" s="21"/>
       <x:c r="U38" s="21"/>
       <x:c r="V38" s="21"/>
-      <x:c r="W38" s="18"/>
-      <x:c r="X38" s="18"/>
-      <x:c r="Y38" s="18"/>
-      <x:c r="Z38" s="18"/>
+      <x:c r="W38" s="21"/>
+      <x:c r="X38" s="21"/>
+      <x:c r="Y38" s="21"/>
+      <x:c r="Z38" s="21"/>
       <x:c r="AA38" s="18"/>
+      <x:c r="AB38" s="18"/>
+      <x:c r="AC38" s="18"/>
+      <x:c r="AD38" s="18"/>
+      <x:c r="AE38" s="18"/>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="18"/>
@@ -1691,15 +1863,19 @@
       <x:c r="P39" s="18"/>
       <x:c r="Q39" s="18"/>
       <x:c r="R39" s="18"/>
-      <x:c r="S39" s="18"/>
-      <x:c r="T39" s="18"/>
+      <x:c r="S39" s="21"/>
+      <x:c r="T39" s="21"/>
       <x:c r="U39" s="21"/>
       <x:c r="V39" s="21"/>
-      <x:c r="W39" s="18"/>
-      <x:c r="X39" s="18"/>
-      <x:c r="Y39" s="18"/>
-      <x:c r="Z39" s="18"/>
+      <x:c r="W39" s="21"/>
+      <x:c r="X39" s="21"/>
+      <x:c r="Y39" s="21"/>
+      <x:c r="Z39" s="21"/>
       <x:c r="AA39" s="18"/>
+      <x:c r="AB39" s="18"/>
+      <x:c r="AC39" s="18"/>
+      <x:c r="AD39" s="18"/>
+      <x:c r="AE39" s="18"/>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="18"/>
@@ -1720,15 +1896,19 @@
       <x:c r="P40" s="18"/>
       <x:c r="Q40" s="18"/>
       <x:c r="R40" s="18"/>
-      <x:c r="S40" s="18"/>
-      <x:c r="T40" s="18"/>
+      <x:c r="S40" s="21"/>
+      <x:c r="T40" s="21"/>
       <x:c r="U40" s="21"/>
       <x:c r="V40" s="21"/>
-      <x:c r="W40" s="18"/>
-      <x:c r="X40" s="18"/>
-      <x:c r="Y40" s="18"/>
-      <x:c r="Z40" s="18"/>
+      <x:c r="W40" s="21"/>
+      <x:c r="X40" s="21"/>
+      <x:c r="Y40" s="21"/>
+      <x:c r="Z40" s="21"/>
       <x:c r="AA40" s="18"/>
+      <x:c r="AB40" s="18"/>
+      <x:c r="AC40" s="18"/>
+      <x:c r="AD40" s="18"/>
+      <x:c r="AE40" s="18"/>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="18"/>
@@ -1749,15 +1929,19 @@
       <x:c r="P41" s="18"/>
       <x:c r="Q41" s="18"/>
       <x:c r="R41" s="18"/>
-      <x:c r="S41" s="18"/>
-      <x:c r="T41" s="18"/>
+      <x:c r="S41" s="21"/>
+      <x:c r="T41" s="21"/>
       <x:c r="U41" s="21"/>
       <x:c r="V41" s="21"/>
-      <x:c r="W41" s="18"/>
-      <x:c r="X41" s="18"/>
-      <x:c r="Y41" s="18"/>
-      <x:c r="Z41" s="18"/>
+      <x:c r="W41" s="21"/>
+      <x:c r="X41" s="21"/>
+      <x:c r="Y41" s="21"/>
+      <x:c r="Z41" s="21"/>
       <x:c r="AA41" s="18"/>
+      <x:c r="AB41" s="18"/>
+      <x:c r="AC41" s="18"/>
+      <x:c r="AD41" s="18"/>
+      <x:c r="AE41" s="18"/>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="18"/>
@@ -1778,15 +1962,19 @@
       <x:c r="P42" s="18"/>
       <x:c r="Q42" s="18"/>
       <x:c r="R42" s="18"/>
-      <x:c r="S42" s="18"/>
-      <x:c r="T42" s="18"/>
+      <x:c r="S42" s="21"/>
+      <x:c r="T42" s="21"/>
       <x:c r="U42" s="21"/>
       <x:c r="V42" s="21"/>
-      <x:c r="W42" s="18"/>
-      <x:c r="X42" s="18"/>
-      <x:c r="Y42" s="18"/>
-      <x:c r="Z42" s="18"/>
+      <x:c r="W42" s="21"/>
+      <x:c r="X42" s="21"/>
+      <x:c r="Y42" s="21"/>
+      <x:c r="Z42" s="21"/>
       <x:c r="AA42" s="18"/>
+      <x:c r="AB42" s="18"/>
+      <x:c r="AC42" s="18"/>
+      <x:c r="AD42" s="18"/>
+      <x:c r="AE42" s="18"/>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="18"/>
@@ -1807,15 +1995,19 @@
       <x:c r="P43" s="18"/>
       <x:c r="Q43" s="18"/>
       <x:c r="R43" s="18"/>
-      <x:c r="S43" s="18"/>
-      <x:c r="T43" s="18"/>
+      <x:c r="S43" s="21"/>
+      <x:c r="T43" s="21"/>
       <x:c r="U43" s="21"/>
       <x:c r="V43" s="21"/>
-      <x:c r="W43" s="18"/>
-      <x:c r="X43" s="18"/>
-      <x:c r="Y43" s="18"/>
-      <x:c r="Z43" s="18"/>
+      <x:c r="W43" s="21"/>
+      <x:c r="X43" s="21"/>
+      <x:c r="Y43" s="21"/>
+      <x:c r="Z43" s="21"/>
       <x:c r="AA43" s="18"/>
+      <x:c r="AB43" s="18"/>
+      <x:c r="AC43" s="18"/>
+      <x:c r="AD43" s="18"/>
+      <x:c r="AE43" s="18"/>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="18"/>
@@ -1836,15 +2028,19 @@
       <x:c r="P44" s="18"/>
       <x:c r="Q44" s="18"/>
       <x:c r="R44" s="18"/>
-      <x:c r="S44" s="18"/>
-      <x:c r="T44" s="18"/>
+      <x:c r="S44" s="21"/>
+      <x:c r="T44" s="21"/>
       <x:c r="U44" s="21"/>
       <x:c r="V44" s="21"/>
-      <x:c r="W44" s="18"/>
-      <x:c r="X44" s="18"/>
-      <x:c r="Y44" s="18"/>
-      <x:c r="Z44" s="18"/>
+      <x:c r="W44" s="21"/>
+      <x:c r="X44" s="21"/>
+      <x:c r="Y44" s="21"/>
+      <x:c r="Z44" s="21"/>
       <x:c r="AA44" s="18"/>
+      <x:c r="AB44" s="18"/>
+      <x:c r="AC44" s="18"/>
+      <x:c r="AD44" s="18"/>
+      <x:c r="AE44" s="18"/>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="18"/>
@@ -1865,15 +2061,19 @@
       <x:c r="P45" s="18"/>
       <x:c r="Q45" s="18"/>
       <x:c r="R45" s="18"/>
-      <x:c r="S45" s="18"/>
-      <x:c r="T45" s="18"/>
+      <x:c r="S45" s="21"/>
+      <x:c r="T45" s="21"/>
       <x:c r="U45" s="21"/>
       <x:c r="V45" s="21"/>
-      <x:c r="W45" s="18"/>
-      <x:c r="X45" s="18"/>
-      <x:c r="Y45" s="18"/>
-      <x:c r="Z45" s="18"/>
+      <x:c r="W45" s="21"/>
+      <x:c r="X45" s="21"/>
+      <x:c r="Y45" s="21"/>
+      <x:c r="Z45" s="21"/>
       <x:c r="AA45" s="18"/>
+      <x:c r="AB45" s="18"/>
+      <x:c r="AC45" s="18"/>
+      <x:c r="AD45" s="18"/>
+      <x:c r="AE45" s="18"/>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="18"/>
@@ -1894,15 +2094,19 @@
       <x:c r="P46" s="18"/>
       <x:c r="Q46" s="18"/>
       <x:c r="R46" s="18"/>
-      <x:c r="S46" s="18"/>
-      <x:c r="T46" s="18"/>
+      <x:c r="S46" s="21"/>
+      <x:c r="T46" s="21"/>
       <x:c r="U46" s="21"/>
       <x:c r="V46" s="21"/>
-      <x:c r="W46" s="18"/>
-      <x:c r="X46" s="18"/>
-      <x:c r="Y46" s="18"/>
-      <x:c r="Z46" s="18"/>
+      <x:c r="W46" s="21"/>
+      <x:c r="X46" s="21"/>
+      <x:c r="Y46" s="21"/>
+      <x:c r="Z46" s="21"/>
       <x:c r="AA46" s="18"/>
+      <x:c r="AB46" s="18"/>
+      <x:c r="AC46" s="18"/>
+      <x:c r="AD46" s="18"/>
+      <x:c r="AE46" s="18"/>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="18"/>
@@ -1923,15 +2127,19 @@
       <x:c r="P47" s="18"/>
       <x:c r="Q47" s="18"/>
       <x:c r="R47" s="18"/>
-      <x:c r="S47" s="18"/>
-      <x:c r="T47" s="18"/>
+      <x:c r="S47" s="21"/>
+      <x:c r="T47" s="21"/>
       <x:c r="U47" s="21"/>
       <x:c r="V47" s="21"/>
-      <x:c r="W47" s="18"/>
-      <x:c r="X47" s="18"/>
-      <x:c r="Y47" s="18"/>
-      <x:c r="Z47" s="18"/>
+      <x:c r="W47" s="21"/>
+      <x:c r="X47" s="21"/>
+      <x:c r="Y47" s="21"/>
+      <x:c r="Z47" s="21"/>
       <x:c r="AA47" s="18"/>
+      <x:c r="AB47" s="18"/>
+      <x:c r="AC47" s="18"/>
+      <x:c r="AD47" s="18"/>
+      <x:c r="AE47" s="18"/>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="18"/>
@@ -1952,15 +2160,19 @@
       <x:c r="P48" s="18"/>
       <x:c r="Q48" s="18"/>
       <x:c r="R48" s="18"/>
-      <x:c r="S48" s="18"/>
-      <x:c r="T48" s="18"/>
+      <x:c r="S48" s="21"/>
+      <x:c r="T48" s="21"/>
       <x:c r="U48" s="21"/>
       <x:c r="V48" s="21"/>
-      <x:c r="W48" s="18"/>
-      <x:c r="X48" s="18"/>
-      <x:c r="Y48" s="18"/>
-      <x:c r="Z48" s="18"/>
+      <x:c r="W48" s="21"/>
+      <x:c r="X48" s="21"/>
+      <x:c r="Y48" s="21"/>
+      <x:c r="Z48" s="21"/>
       <x:c r="AA48" s="18"/>
+      <x:c r="AB48" s="18"/>
+      <x:c r="AC48" s="18"/>
+      <x:c r="AD48" s="18"/>
+      <x:c r="AE48" s="18"/>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="18"/>
@@ -1981,15 +2193,19 @@
       <x:c r="P49" s="18"/>
       <x:c r="Q49" s="18"/>
       <x:c r="R49" s="18"/>
-      <x:c r="S49" s="18"/>
-      <x:c r="T49" s="18"/>
+      <x:c r="S49" s="21"/>
+      <x:c r="T49" s="21"/>
       <x:c r="U49" s="21"/>
       <x:c r="V49" s="21"/>
-      <x:c r="W49" s="18"/>
-      <x:c r="X49" s="18"/>
-      <x:c r="Y49" s="18"/>
-      <x:c r="Z49" s="18"/>
+      <x:c r="W49" s="21"/>
+      <x:c r="X49" s="21"/>
+      <x:c r="Y49" s="21"/>
+      <x:c r="Z49" s="21"/>
       <x:c r="AA49" s="18"/>
+      <x:c r="AB49" s="18"/>
+      <x:c r="AC49" s="18"/>
+      <x:c r="AD49" s="18"/>
+      <x:c r="AE49" s="18"/>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="18"/>
@@ -2010,15 +2226,19 @@
       <x:c r="P50" s="18"/>
       <x:c r="Q50" s="18"/>
       <x:c r="R50" s="18"/>
-      <x:c r="S50" s="18"/>
-      <x:c r="T50" s="18"/>
+      <x:c r="S50" s="21"/>
+      <x:c r="T50" s="21"/>
       <x:c r="U50" s="21"/>
       <x:c r="V50" s="21"/>
-      <x:c r="W50" s="18"/>
-      <x:c r="X50" s="18"/>
-      <x:c r="Y50" s="18"/>
-      <x:c r="Z50" s="18"/>
+      <x:c r="W50" s="21"/>
+      <x:c r="X50" s="21"/>
+      <x:c r="Y50" s="21"/>
+      <x:c r="Z50" s="21"/>
       <x:c r="AA50" s="18"/>
+      <x:c r="AB50" s="18"/>
+      <x:c r="AC50" s="18"/>
+      <x:c r="AD50" s="18"/>
+      <x:c r="AE50" s="18"/>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="18"/>
@@ -2039,15 +2259,19 @@
       <x:c r="P51" s="18"/>
       <x:c r="Q51" s="18"/>
       <x:c r="R51" s="18"/>
-      <x:c r="S51" s="18"/>
-      <x:c r="T51" s="18"/>
+      <x:c r="S51" s="21"/>
+      <x:c r="T51" s="21"/>
       <x:c r="U51" s="21"/>
       <x:c r="V51" s="21"/>
-      <x:c r="W51" s="18"/>
-      <x:c r="X51" s="18"/>
-      <x:c r="Y51" s="18"/>
-      <x:c r="Z51" s="18"/>
+      <x:c r="W51" s="21"/>
+      <x:c r="X51" s="21"/>
+      <x:c r="Y51" s="21"/>
+      <x:c r="Z51" s="21"/>
       <x:c r="AA51" s="18"/>
+      <x:c r="AB51" s="18"/>
+      <x:c r="AC51" s="18"/>
+      <x:c r="AD51" s="18"/>
+      <x:c r="AE51" s="18"/>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="18"/>
@@ -2068,15 +2292,19 @@
       <x:c r="P52" s="18"/>
       <x:c r="Q52" s="18"/>
       <x:c r="R52" s="18"/>
-      <x:c r="S52" s="18"/>
-      <x:c r="T52" s="18"/>
+      <x:c r="S52" s="21"/>
+      <x:c r="T52" s="21"/>
       <x:c r="U52" s="21"/>
       <x:c r="V52" s="21"/>
-      <x:c r="W52" s="18"/>
-      <x:c r="X52" s="18"/>
-      <x:c r="Y52" s="18"/>
-      <x:c r="Z52" s="18"/>
+      <x:c r="W52" s="21"/>
+      <x:c r="X52" s="21"/>
+      <x:c r="Y52" s="21"/>
+      <x:c r="Z52" s="21"/>
       <x:c r="AA52" s="18"/>
+      <x:c r="AB52" s="18"/>
+      <x:c r="AC52" s="18"/>
+      <x:c r="AD52" s="18"/>
+      <x:c r="AE52" s="18"/>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="18"/>
@@ -2097,15 +2325,19 @@
       <x:c r="P53" s="18"/>
       <x:c r="Q53" s="18"/>
       <x:c r="R53" s="18"/>
-      <x:c r="S53" s="18"/>
-      <x:c r="T53" s="18"/>
+      <x:c r="S53" s="21"/>
+      <x:c r="T53" s="21"/>
       <x:c r="U53" s="21"/>
       <x:c r="V53" s="21"/>
-      <x:c r="W53" s="18"/>
-      <x:c r="X53" s="18"/>
-      <x:c r="Y53" s="18"/>
-      <x:c r="Z53" s="18"/>
+      <x:c r="W53" s="21"/>
+      <x:c r="X53" s="21"/>
+      <x:c r="Y53" s="21"/>
+      <x:c r="Z53" s="21"/>
       <x:c r="AA53" s="18"/>
+      <x:c r="AB53" s="18"/>
+      <x:c r="AC53" s="18"/>
+      <x:c r="AD53" s="18"/>
+      <x:c r="AE53" s="18"/>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="18"/>
@@ -2126,15 +2358,19 @@
       <x:c r="P54" s="18"/>
       <x:c r="Q54" s="18"/>
       <x:c r="R54" s="18"/>
-      <x:c r="S54" s="18"/>
-      <x:c r="T54" s="18"/>
+      <x:c r="S54" s="21"/>
+      <x:c r="T54" s="21"/>
       <x:c r="U54" s="21"/>
       <x:c r="V54" s="21"/>
-      <x:c r="W54" s="18"/>
-      <x:c r="X54" s="18"/>
-      <x:c r="Y54" s="18"/>
-      <x:c r="Z54" s="18"/>
+      <x:c r="W54" s="21"/>
+      <x:c r="X54" s="21"/>
+      <x:c r="Y54" s="21"/>
+      <x:c r="Z54" s="21"/>
       <x:c r="AA54" s="18"/>
+      <x:c r="AB54" s="18"/>
+      <x:c r="AC54" s="18"/>
+      <x:c r="AD54" s="18"/>
+      <x:c r="AE54" s="18"/>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="18"/>
@@ -2155,15 +2391,19 @@
       <x:c r="P55" s="18"/>
       <x:c r="Q55" s="18"/>
       <x:c r="R55" s="18"/>
-      <x:c r="S55" s="18"/>
-      <x:c r="T55" s="18"/>
+      <x:c r="S55" s="21"/>
+      <x:c r="T55" s="21"/>
       <x:c r="U55" s="21"/>
       <x:c r="V55" s="21"/>
-      <x:c r="W55" s="18"/>
-      <x:c r="X55" s="18"/>
-      <x:c r="Y55" s="18"/>
-      <x:c r="Z55" s="18"/>
+      <x:c r="W55" s="21"/>
+      <x:c r="X55" s="21"/>
+      <x:c r="Y55" s="21"/>
+      <x:c r="Z55" s="21"/>
       <x:c r="AA55" s="18"/>
+      <x:c r="AB55" s="18"/>
+      <x:c r="AC55" s="18"/>
+      <x:c r="AD55" s="18"/>
+      <x:c r="AE55" s="18"/>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="18"/>
@@ -2184,15 +2424,19 @@
       <x:c r="P56" s="18"/>
       <x:c r="Q56" s="18"/>
       <x:c r="R56" s="18"/>
-      <x:c r="S56" s="18"/>
-      <x:c r="T56" s="18"/>
+      <x:c r="S56" s="21"/>
+      <x:c r="T56" s="21"/>
       <x:c r="U56" s="21"/>
       <x:c r="V56" s="21"/>
-      <x:c r="W56" s="18"/>
-      <x:c r="X56" s="18"/>
-      <x:c r="Y56" s="18"/>
-      <x:c r="Z56" s="18"/>
+      <x:c r="W56" s="21"/>
+      <x:c r="X56" s="21"/>
+      <x:c r="Y56" s="21"/>
+      <x:c r="Z56" s="21"/>
       <x:c r="AA56" s="18"/>
+      <x:c r="AB56" s="18"/>
+      <x:c r="AC56" s="18"/>
+      <x:c r="AD56" s="18"/>
+      <x:c r="AE56" s="18"/>
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="18"/>
@@ -2213,15 +2457,19 @@
       <x:c r="P57" s="18"/>
       <x:c r="Q57" s="18"/>
       <x:c r="R57" s="18"/>
-      <x:c r="S57" s="18"/>
-      <x:c r="T57" s="18"/>
+      <x:c r="S57" s="21"/>
+      <x:c r="T57" s="21"/>
       <x:c r="U57" s="21"/>
       <x:c r="V57" s="21"/>
-      <x:c r="W57" s="18"/>
-      <x:c r="X57" s="18"/>
-      <x:c r="Y57" s="18"/>
-      <x:c r="Z57" s="18"/>
+      <x:c r="W57" s="21"/>
+      <x:c r="X57" s="21"/>
+      <x:c r="Y57" s="21"/>
+      <x:c r="Z57" s="21"/>
       <x:c r="AA57" s="18"/>
+      <x:c r="AB57" s="18"/>
+      <x:c r="AC57" s="18"/>
+      <x:c r="AD57" s="18"/>
+      <x:c r="AE57" s="18"/>
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="18"/>
@@ -2242,15 +2490,19 @@
       <x:c r="P58" s="18"/>
       <x:c r="Q58" s="18"/>
       <x:c r="R58" s="18"/>
-      <x:c r="S58" s="18"/>
-      <x:c r="T58" s="18"/>
+      <x:c r="S58" s="21"/>
+      <x:c r="T58" s="21"/>
       <x:c r="U58" s="21"/>
       <x:c r="V58" s="21"/>
-      <x:c r="W58" s="18"/>
-      <x:c r="X58" s="18"/>
-      <x:c r="Y58" s="18"/>
-      <x:c r="Z58" s="18"/>
+      <x:c r="W58" s="21"/>
+      <x:c r="X58" s="21"/>
+      <x:c r="Y58" s="21"/>
+      <x:c r="Z58" s="21"/>
       <x:c r="AA58" s="18"/>
+      <x:c r="AB58" s="18"/>
+      <x:c r="AC58" s="18"/>
+      <x:c r="AD58" s="18"/>
+      <x:c r="AE58" s="18"/>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="18"/>
@@ -2271,15 +2523,19 @@
       <x:c r="P59" s="18"/>
       <x:c r="Q59" s="18"/>
       <x:c r="R59" s="18"/>
-      <x:c r="S59" s="18"/>
-      <x:c r="T59" s="18"/>
+      <x:c r="S59" s="21"/>
+      <x:c r="T59" s="21"/>
       <x:c r="U59" s="21"/>
       <x:c r="V59" s="21"/>
-      <x:c r="W59" s="18"/>
-      <x:c r="X59" s="18"/>
-      <x:c r="Y59" s="18"/>
-      <x:c r="Z59" s="18"/>
+      <x:c r="W59" s="21"/>
+      <x:c r="X59" s="21"/>
+      <x:c r="Y59" s="21"/>
+      <x:c r="Z59" s="21"/>
       <x:c r="AA59" s="18"/>
+      <x:c r="AB59" s="18"/>
+      <x:c r="AC59" s="18"/>
+      <x:c r="AD59" s="18"/>
+      <x:c r="AE59" s="18"/>
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="18"/>
@@ -2300,15 +2556,19 @@
       <x:c r="P60" s="18"/>
       <x:c r="Q60" s="18"/>
       <x:c r="R60" s="18"/>
-      <x:c r="S60" s="18"/>
-      <x:c r="T60" s="18"/>
+      <x:c r="S60" s="21"/>
+      <x:c r="T60" s="21"/>
       <x:c r="U60" s="21"/>
       <x:c r="V60" s="21"/>
-      <x:c r="W60" s="18"/>
-      <x:c r="X60" s="18"/>
-      <x:c r="Y60" s="18"/>
-      <x:c r="Z60" s="18"/>
+      <x:c r="W60" s="21"/>
+      <x:c r="X60" s="21"/>
+      <x:c r="Y60" s="21"/>
+      <x:c r="Z60" s="21"/>
       <x:c r="AA60" s="18"/>
+      <x:c r="AB60" s="18"/>
+      <x:c r="AC60" s="18"/>
+      <x:c r="AD60" s="18"/>
+      <x:c r="AE60" s="18"/>
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="18"/>
@@ -2329,15 +2589,19 @@
       <x:c r="P61" s="18"/>
       <x:c r="Q61" s="18"/>
       <x:c r="R61" s="18"/>
-      <x:c r="S61" s="18"/>
-      <x:c r="T61" s="18"/>
+      <x:c r="S61" s="21"/>
+      <x:c r="T61" s="21"/>
       <x:c r="U61" s="21"/>
       <x:c r="V61" s="21"/>
-      <x:c r="W61" s="18"/>
-      <x:c r="X61" s="18"/>
-      <x:c r="Y61" s="18"/>
-      <x:c r="Z61" s="18"/>
+      <x:c r="W61" s="21"/>
+      <x:c r="X61" s="21"/>
+      <x:c r="Y61" s="21"/>
+      <x:c r="Z61" s="21"/>
       <x:c r="AA61" s="18"/>
+      <x:c r="AB61" s="18"/>
+      <x:c r="AC61" s="18"/>
+      <x:c r="AD61" s="18"/>
+      <x:c r="AE61" s="18"/>
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="18"/>
@@ -2358,15 +2622,19 @@
       <x:c r="P62" s="18"/>
       <x:c r="Q62" s="18"/>
       <x:c r="R62" s="18"/>
-      <x:c r="S62" s="18"/>
-      <x:c r="T62" s="18"/>
+      <x:c r="S62" s="21"/>
+      <x:c r="T62" s="21"/>
       <x:c r="U62" s="21"/>
       <x:c r="V62" s="21"/>
-      <x:c r="W62" s="18"/>
-      <x:c r="X62" s="18"/>
-      <x:c r="Y62" s="18"/>
-      <x:c r="Z62" s="18"/>
+      <x:c r="W62" s="21"/>
+      <x:c r="X62" s="21"/>
+      <x:c r="Y62" s="21"/>
+      <x:c r="Z62" s="21"/>
       <x:c r="AA62" s="18"/>
+      <x:c r="AB62" s="18"/>
+      <x:c r="AC62" s="18"/>
+      <x:c r="AD62" s="18"/>
+      <x:c r="AE62" s="18"/>
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="18"/>
@@ -2387,15 +2655,19 @@
       <x:c r="P63" s="18"/>
       <x:c r="Q63" s="18"/>
       <x:c r="R63" s="18"/>
-      <x:c r="S63" s="18"/>
-      <x:c r="T63" s="18"/>
+      <x:c r="S63" s="21"/>
+      <x:c r="T63" s="21"/>
       <x:c r="U63" s="21"/>
       <x:c r="V63" s="21"/>
-      <x:c r="W63" s="18"/>
-      <x:c r="X63" s="18"/>
-      <x:c r="Y63" s="18"/>
-      <x:c r="Z63" s="18"/>
+      <x:c r="W63" s="21"/>
+      <x:c r="X63" s="21"/>
+      <x:c r="Y63" s="21"/>
+      <x:c r="Z63" s="21"/>
       <x:c r="AA63" s="18"/>
+      <x:c r="AB63" s="18"/>
+      <x:c r="AC63" s="18"/>
+      <x:c r="AD63" s="18"/>
+      <x:c r="AE63" s="18"/>
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="18"/>
@@ -2416,15 +2688,19 @@
       <x:c r="P64" s="18"/>
       <x:c r="Q64" s="18"/>
       <x:c r="R64" s="18"/>
-      <x:c r="S64" s="18"/>
-      <x:c r="T64" s="18"/>
+      <x:c r="S64" s="21"/>
+      <x:c r="T64" s="21"/>
       <x:c r="U64" s="21"/>
       <x:c r="V64" s="21"/>
-      <x:c r="W64" s="18"/>
-      <x:c r="X64" s="18"/>
-      <x:c r="Y64" s="18"/>
-      <x:c r="Z64" s="18"/>
+      <x:c r="W64" s="21"/>
+      <x:c r="X64" s="21"/>
+      <x:c r="Y64" s="21"/>
+      <x:c r="Z64" s="21"/>
       <x:c r="AA64" s="18"/>
+      <x:c r="AB64" s="18"/>
+      <x:c r="AC64" s="18"/>
+      <x:c r="AD64" s="18"/>
+      <x:c r="AE64" s="18"/>
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="18"/>
@@ -2445,15 +2721,19 @@
       <x:c r="P65" s="18"/>
       <x:c r="Q65" s="18"/>
       <x:c r="R65" s="18"/>
-      <x:c r="S65" s="18"/>
-      <x:c r="T65" s="18"/>
+      <x:c r="S65" s="21"/>
+      <x:c r="T65" s="21"/>
       <x:c r="U65" s="21"/>
       <x:c r="V65" s="21"/>
-      <x:c r="W65" s="18"/>
-      <x:c r="X65" s="18"/>
-      <x:c r="Y65" s="18"/>
-      <x:c r="Z65" s="18"/>
+      <x:c r="W65" s="21"/>
+      <x:c r="X65" s="21"/>
+      <x:c r="Y65" s="21"/>
+      <x:c r="Z65" s="21"/>
       <x:c r="AA65" s="18"/>
+      <x:c r="AB65" s="18"/>
+      <x:c r="AC65" s="18"/>
+      <x:c r="AD65" s="18"/>
+      <x:c r="AE65" s="18"/>
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="18"/>
@@ -2474,15 +2754,19 @@
       <x:c r="P66" s="18"/>
       <x:c r="Q66" s="18"/>
       <x:c r="R66" s="18"/>
-      <x:c r="S66" s="18"/>
-      <x:c r="T66" s="18"/>
+      <x:c r="S66" s="21"/>
+      <x:c r="T66" s="21"/>
       <x:c r="U66" s="21"/>
       <x:c r="V66" s="21"/>
-      <x:c r="W66" s="18"/>
-      <x:c r="X66" s="18"/>
-      <x:c r="Y66" s="18"/>
-      <x:c r="Z66" s="18"/>
+      <x:c r="W66" s="21"/>
+      <x:c r="X66" s="21"/>
+      <x:c r="Y66" s="21"/>
+      <x:c r="Z66" s="21"/>
       <x:c r="AA66" s="18"/>
+      <x:c r="AB66" s="18"/>
+      <x:c r="AC66" s="18"/>
+      <x:c r="AD66" s="18"/>
+      <x:c r="AE66" s="18"/>
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="18"/>
@@ -2503,15 +2787,19 @@
       <x:c r="P67" s="18"/>
       <x:c r="Q67" s="18"/>
       <x:c r="R67" s="18"/>
-      <x:c r="S67" s="18"/>
-      <x:c r="T67" s="18"/>
+      <x:c r="S67" s="21"/>
+      <x:c r="T67" s="21"/>
       <x:c r="U67" s="21"/>
       <x:c r="V67" s="21"/>
-      <x:c r="W67" s="18"/>
-      <x:c r="X67" s="18"/>
-      <x:c r="Y67" s="18"/>
-      <x:c r="Z67" s="18"/>
+      <x:c r="W67" s="21"/>
+      <x:c r="X67" s="21"/>
+      <x:c r="Y67" s="21"/>
+      <x:c r="Z67" s="21"/>
       <x:c r="AA67" s="18"/>
+      <x:c r="AB67" s="18"/>
+      <x:c r="AC67" s="18"/>
+      <x:c r="AD67" s="18"/>
+      <x:c r="AE67" s="18"/>
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="18"/>
@@ -2532,15 +2820,19 @@
       <x:c r="P68" s="18"/>
       <x:c r="Q68" s="18"/>
       <x:c r="R68" s="18"/>
-      <x:c r="S68" s="18"/>
-      <x:c r="T68" s="18"/>
+      <x:c r="S68" s="21"/>
+      <x:c r="T68" s="21"/>
       <x:c r="U68" s="21"/>
       <x:c r="V68" s="21"/>
-      <x:c r="W68" s="18"/>
-      <x:c r="X68" s="18"/>
-      <x:c r="Y68" s="18"/>
-      <x:c r="Z68" s="18"/>
+      <x:c r="W68" s="21"/>
+      <x:c r="X68" s="21"/>
+      <x:c r="Y68" s="21"/>
+      <x:c r="Z68" s="21"/>
       <x:c r="AA68" s="18"/>
+      <x:c r="AB68" s="18"/>
+      <x:c r="AC68" s="18"/>
+      <x:c r="AD68" s="18"/>
+      <x:c r="AE68" s="18"/>
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="18"/>
@@ -2561,15 +2853,19 @@
       <x:c r="P69" s="18"/>
       <x:c r="Q69" s="18"/>
       <x:c r="R69" s="18"/>
-      <x:c r="S69" s="18"/>
-      <x:c r="T69" s="18"/>
+      <x:c r="S69" s="21"/>
+      <x:c r="T69" s="21"/>
       <x:c r="U69" s="21"/>
       <x:c r="V69" s="21"/>
-      <x:c r="W69" s="18"/>
-      <x:c r="X69" s="18"/>
-      <x:c r="Y69" s="18"/>
-      <x:c r="Z69" s="18"/>
+      <x:c r="W69" s="21"/>
+      <x:c r="X69" s="21"/>
+      <x:c r="Y69" s="21"/>
+      <x:c r="Z69" s="21"/>
       <x:c r="AA69" s="18"/>
+      <x:c r="AB69" s="18"/>
+      <x:c r="AC69" s="18"/>
+      <x:c r="AD69" s="18"/>
+      <x:c r="AE69" s="18"/>
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="18"/>
@@ -2590,15 +2886,19 @@
       <x:c r="P70" s="18"/>
       <x:c r="Q70" s="18"/>
       <x:c r="R70" s="18"/>
-      <x:c r="S70" s="18"/>
-      <x:c r="T70" s="18"/>
+      <x:c r="S70" s="21"/>
+      <x:c r="T70" s="21"/>
       <x:c r="U70" s="21"/>
       <x:c r="V70" s="21"/>
-      <x:c r="W70" s="18"/>
-      <x:c r="X70" s="18"/>
-      <x:c r="Y70" s="18"/>
-      <x:c r="Z70" s="18"/>
+      <x:c r="W70" s="21"/>
+      <x:c r="X70" s="21"/>
+      <x:c r="Y70" s="21"/>
+      <x:c r="Z70" s="21"/>
       <x:c r="AA70" s="18"/>
+      <x:c r="AB70" s="18"/>
+      <x:c r="AC70" s="18"/>
+      <x:c r="AD70" s="18"/>
+      <x:c r="AE70" s="18"/>
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="18"/>
@@ -2619,15 +2919,19 @@
       <x:c r="P71" s="18"/>
       <x:c r="Q71" s="18"/>
       <x:c r="R71" s="18"/>
-      <x:c r="S71" s="18"/>
-      <x:c r="T71" s="18"/>
+      <x:c r="S71" s="21"/>
+      <x:c r="T71" s="21"/>
       <x:c r="U71" s="21"/>
       <x:c r="V71" s="21"/>
-      <x:c r="W71" s="18"/>
-      <x:c r="X71" s="18"/>
-      <x:c r="Y71" s="18"/>
-      <x:c r="Z71" s="18"/>
+      <x:c r="W71" s="21"/>
+      <x:c r="X71" s="21"/>
+      <x:c r="Y71" s="21"/>
+      <x:c r="Z71" s="21"/>
       <x:c r="AA71" s="18"/>
+      <x:c r="AB71" s="18"/>
+      <x:c r="AC71" s="18"/>
+      <x:c r="AD71" s="18"/>
+      <x:c r="AE71" s="18"/>
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="18"/>
@@ -2648,15 +2952,19 @@
       <x:c r="P72" s="18"/>
       <x:c r="Q72" s="18"/>
       <x:c r="R72" s="18"/>
-      <x:c r="S72" s="18"/>
-      <x:c r="T72" s="18"/>
+      <x:c r="S72" s="21"/>
+      <x:c r="T72" s="21"/>
       <x:c r="U72" s="21"/>
       <x:c r="V72" s="21"/>
-      <x:c r="W72" s="18"/>
-      <x:c r="X72" s="18"/>
-      <x:c r="Y72" s="18"/>
-      <x:c r="Z72" s="18"/>
+      <x:c r="W72" s="21"/>
+      <x:c r="X72" s="21"/>
+      <x:c r="Y72" s="21"/>
+      <x:c r="Z72" s="21"/>
       <x:c r="AA72" s="18"/>
+      <x:c r="AB72" s="18"/>
+      <x:c r="AC72" s="18"/>
+      <x:c r="AD72" s="18"/>
+      <x:c r="AE72" s="18"/>
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="18"/>
@@ -2677,15 +2985,19 @@
       <x:c r="P73" s="18"/>
       <x:c r="Q73" s="18"/>
       <x:c r="R73" s="18"/>
-      <x:c r="S73" s="18"/>
-      <x:c r="T73" s="18"/>
+      <x:c r="S73" s="21"/>
+      <x:c r="T73" s="21"/>
       <x:c r="U73" s="21"/>
       <x:c r="V73" s="21"/>
-      <x:c r="W73" s="18"/>
-      <x:c r="X73" s="18"/>
-      <x:c r="Y73" s="18"/>
-      <x:c r="Z73" s="18"/>
+      <x:c r="W73" s="21"/>
+      <x:c r="X73" s="21"/>
+      <x:c r="Y73" s="21"/>
+      <x:c r="Z73" s="21"/>
       <x:c r="AA73" s="18"/>
+      <x:c r="AB73" s="18"/>
+      <x:c r="AC73" s="18"/>
+      <x:c r="AD73" s="18"/>
+      <x:c r="AE73" s="18"/>
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="18"/>
@@ -2706,15 +3018,19 @@
       <x:c r="P74" s="18"/>
       <x:c r="Q74" s="18"/>
       <x:c r="R74" s="18"/>
-      <x:c r="S74" s="18"/>
-      <x:c r="T74" s="18"/>
+      <x:c r="S74" s="21"/>
+      <x:c r="T74" s="21"/>
       <x:c r="U74" s="21"/>
       <x:c r="V74" s="21"/>
-      <x:c r="W74" s="18"/>
-      <x:c r="X74" s="18"/>
-      <x:c r="Y74" s="18"/>
-      <x:c r="Z74" s="18"/>
+      <x:c r="W74" s="21"/>
+      <x:c r="X74" s="21"/>
+      <x:c r="Y74" s="21"/>
+      <x:c r="Z74" s="21"/>
       <x:c r="AA74" s="18"/>
+      <x:c r="AB74" s="18"/>
+      <x:c r="AC74" s="18"/>
+      <x:c r="AD74" s="18"/>
+      <x:c r="AE74" s="18"/>
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="18"/>
@@ -2735,15 +3051,19 @@
       <x:c r="P75" s="18"/>
       <x:c r="Q75" s="18"/>
       <x:c r="R75" s="18"/>
-      <x:c r="S75" s="18"/>
-      <x:c r="T75" s="18"/>
+      <x:c r="S75" s="21"/>
+      <x:c r="T75" s="21"/>
       <x:c r="U75" s="21"/>
       <x:c r="V75" s="21"/>
-      <x:c r="W75" s="18"/>
-      <x:c r="X75" s="18"/>
-      <x:c r="Y75" s="18"/>
-      <x:c r="Z75" s="18"/>
+      <x:c r="W75" s="21"/>
+      <x:c r="X75" s="21"/>
+      <x:c r="Y75" s="21"/>
+      <x:c r="Z75" s="21"/>
       <x:c r="AA75" s="18"/>
+      <x:c r="AB75" s="18"/>
+      <x:c r="AC75" s="18"/>
+      <x:c r="AD75" s="18"/>
+      <x:c r="AE75" s="18"/>
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="18"/>
@@ -2764,15 +3084,19 @@
       <x:c r="P76" s="18"/>
       <x:c r="Q76" s="18"/>
       <x:c r="R76" s="18"/>
-      <x:c r="S76" s="18"/>
-      <x:c r="T76" s="18"/>
+      <x:c r="S76" s="21"/>
+      <x:c r="T76" s="21"/>
       <x:c r="U76" s="21"/>
       <x:c r="V76" s="21"/>
-      <x:c r="W76" s="18"/>
-      <x:c r="X76" s="18"/>
-      <x:c r="Y76" s="18"/>
-      <x:c r="Z76" s="18"/>
+      <x:c r="W76" s="21"/>
+      <x:c r="X76" s="21"/>
+      <x:c r="Y76" s="21"/>
+      <x:c r="Z76" s="21"/>
       <x:c r="AA76" s="18"/>
+      <x:c r="AB76" s="18"/>
+      <x:c r="AC76" s="18"/>
+      <x:c r="AD76" s="18"/>
+      <x:c r="AE76" s="18"/>
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="18"/>
@@ -2793,15 +3117,19 @@
       <x:c r="P77" s="18"/>
       <x:c r="Q77" s="18"/>
       <x:c r="R77" s="18"/>
-      <x:c r="S77" s="18"/>
-      <x:c r="T77" s="18"/>
+      <x:c r="S77" s="21"/>
+      <x:c r="T77" s="21"/>
       <x:c r="U77" s="21"/>
       <x:c r="V77" s="21"/>
-      <x:c r="W77" s="18"/>
-      <x:c r="X77" s="18"/>
-      <x:c r="Y77" s="18"/>
-      <x:c r="Z77" s="18"/>
+      <x:c r="W77" s="21"/>
+      <x:c r="X77" s="21"/>
+      <x:c r="Y77" s="21"/>
+      <x:c r="Z77" s="21"/>
       <x:c r="AA77" s="18"/>
+      <x:c r="AB77" s="18"/>
+      <x:c r="AC77" s="18"/>
+      <x:c r="AD77" s="18"/>
+      <x:c r="AE77" s="18"/>
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="18"/>
@@ -2822,15 +3150,19 @@
       <x:c r="P78" s="18"/>
       <x:c r="Q78" s="18"/>
       <x:c r="R78" s="18"/>
-      <x:c r="S78" s="18"/>
-      <x:c r="T78" s="18"/>
+      <x:c r="S78" s="21"/>
+      <x:c r="T78" s="21"/>
       <x:c r="U78" s="21"/>
       <x:c r="V78" s="21"/>
-      <x:c r="W78" s="18"/>
-      <x:c r="X78" s="18"/>
-      <x:c r="Y78" s="18"/>
-      <x:c r="Z78" s="18"/>
+      <x:c r="W78" s="21"/>
+      <x:c r="X78" s="21"/>
+      <x:c r="Y78" s="21"/>
+      <x:c r="Z78" s="21"/>
       <x:c r="AA78" s="18"/>
+      <x:c r="AB78" s="18"/>
+      <x:c r="AC78" s="18"/>
+      <x:c r="AD78" s="18"/>
+      <x:c r="AE78" s="18"/>
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="18"/>
@@ -2851,15 +3183,19 @@
       <x:c r="P79" s="18"/>
       <x:c r="Q79" s="18"/>
       <x:c r="R79" s="18"/>
-      <x:c r="S79" s="18"/>
-      <x:c r="T79" s="18"/>
+      <x:c r="S79" s="21"/>
+      <x:c r="T79" s="21"/>
       <x:c r="U79" s="21"/>
       <x:c r="V79" s="21"/>
-      <x:c r="W79" s="18"/>
-      <x:c r="X79" s="18"/>
-      <x:c r="Y79" s="18"/>
-      <x:c r="Z79" s="18"/>
+      <x:c r="W79" s="21"/>
+      <x:c r="X79" s="21"/>
+      <x:c r="Y79" s="21"/>
+      <x:c r="Z79" s="21"/>
       <x:c r="AA79" s="18"/>
+      <x:c r="AB79" s="18"/>
+      <x:c r="AC79" s="18"/>
+      <x:c r="AD79" s="18"/>
+      <x:c r="AE79" s="18"/>
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="18"/>
@@ -2880,15 +3216,19 @@
       <x:c r="P80" s="18"/>
       <x:c r="Q80" s="18"/>
       <x:c r="R80" s="18"/>
-      <x:c r="S80" s="18"/>
-      <x:c r="T80" s="18"/>
+      <x:c r="S80" s="21"/>
+      <x:c r="T80" s="21"/>
       <x:c r="U80" s="21"/>
       <x:c r="V80" s="21"/>
-      <x:c r="W80" s="18"/>
-      <x:c r="X80" s="18"/>
-      <x:c r="Y80" s="18"/>
-      <x:c r="Z80" s="18"/>
+      <x:c r="W80" s="21"/>
+      <x:c r="X80" s="21"/>
+      <x:c r="Y80" s="21"/>
+      <x:c r="Z80" s="21"/>
       <x:c r="AA80" s="18"/>
+      <x:c r="AB80" s="18"/>
+      <x:c r="AC80" s="18"/>
+      <x:c r="AD80" s="18"/>
+      <x:c r="AE80" s="18"/>
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="18"/>
@@ -2909,15 +3249,19 @@
       <x:c r="P81" s="18"/>
       <x:c r="Q81" s="18"/>
       <x:c r="R81" s="18"/>
-      <x:c r="S81" s="18"/>
-      <x:c r="T81" s="18"/>
+      <x:c r="S81" s="21"/>
+      <x:c r="T81" s="21"/>
       <x:c r="U81" s="21"/>
       <x:c r="V81" s="21"/>
-      <x:c r="W81" s="18"/>
-      <x:c r="X81" s="18"/>
-      <x:c r="Y81" s="18"/>
-      <x:c r="Z81" s="18"/>
+      <x:c r="W81" s="21"/>
+      <x:c r="X81" s="21"/>
+      <x:c r="Y81" s="21"/>
+      <x:c r="Z81" s="21"/>
       <x:c r="AA81" s="18"/>
+      <x:c r="AB81" s="18"/>
+      <x:c r="AC81" s="18"/>
+      <x:c r="AD81" s="18"/>
+      <x:c r="AE81" s="18"/>
     </x:row>
     <x:row r="82">
       <x:c r="A82" s="18"/>
@@ -2938,15 +3282,19 @@
       <x:c r="P82" s="18"/>
       <x:c r="Q82" s="18"/>
       <x:c r="R82" s="18"/>
-      <x:c r="S82" s="18"/>
-      <x:c r="T82" s="18"/>
+      <x:c r="S82" s="21"/>
+      <x:c r="T82" s="21"/>
       <x:c r="U82" s="21"/>
       <x:c r="V82" s="21"/>
-      <x:c r="W82" s="18"/>
-      <x:c r="X82" s="18"/>
-      <x:c r="Y82" s="18"/>
-      <x:c r="Z82" s="18"/>
+      <x:c r="W82" s="21"/>
+      <x:c r="X82" s="21"/>
+      <x:c r="Y82" s="21"/>
+      <x:c r="Z82" s="21"/>
       <x:c r="AA82" s="18"/>
+      <x:c r="AB82" s="18"/>
+      <x:c r="AC82" s="18"/>
+      <x:c r="AD82" s="18"/>
+      <x:c r="AE82" s="18"/>
     </x:row>
     <x:row r="83">
       <x:c r="A83" s="18"/>
@@ -2967,15 +3315,19 @@
       <x:c r="P83" s="18"/>
       <x:c r="Q83" s="18"/>
       <x:c r="R83" s="18"/>
-      <x:c r="S83" s="18"/>
-      <x:c r="T83" s="18"/>
+      <x:c r="S83" s="21"/>
+      <x:c r="T83" s="21"/>
       <x:c r="U83" s="21"/>
       <x:c r="V83" s="21"/>
-      <x:c r="W83" s="18"/>
-      <x:c r="X83" s="18"/>
-      <x:c r="Y83" s="18"/>
-      <x:c r="Z83" s="18"/>
+      <x:c r="W83" s="21"/>
+      <x:c r="X83" s="21"/>
+      <x:c r="Y83" s="21"/>
+      <x:c r="Z83" s="21"/>
       <x:c r="AA83" s="18"/>
+      <x:c r="AB83" s="18"/>
+      <x:c r="AC83" s="18"/>
+      <x:c r="AD83" s="18"/>
+      <x:c r="AE83" s="18"/>
     </x:row>
     <x:row r="84">
       <x:c r="A84" s="18"/>
@@ -2996,15 +3348,19 @@
       <x:c r="P84" s="18"/>
       <x:c r="Q84" s="18"/>
       <x:c r="R84" s="18"/>
-      <x:c r="S84" s="18"/>
-      <x:c r="T84" s="18"/>
+      <x:c r="S84" s="21"/>
+      <x:c r="T84" s="21"/>
       <x:c r="U84" s="21"/>
       <x:c r="V84" s="21"/>
-      <x:c r="W84" s="18"/>
-      <x:c r="X84" s="18"/>
-      <x:c r="Y84" s="18"/>
-      <x:c r="Z84" s="18"/>
+      <x:c r="W84" s="21"/>
+      <x:c r="X84" s="21"/>
+      <x:c r="Y84" s="21"/>
+      <x:c r="Z84" s="21"/>
       <x:c r="AA84" s="18"/>
+      <x:c r="AB84" s="18"/>
+      <x:c r="AC84" s="18"/>
+      <x:c r="AD84" s="18"/>
+      <x:c r="AE84" s="18"/>
     </x:row>
     <x:row r="85">
       <x:c r="A85" s="18"/>
@@ -3025,15 +3381,19 @@
       <x:c r="P85" s="18"/>
       <x:c r="Q85" s="18"/>
       <x:c r="R85" s="18"/>
-      <x:c r="S85" s="18"/>
-      <x:c r="T85" s="18"/>
+      <x:c r="S85" s="21"/>
+      <x:c r="T85" s="21"/>
       <x:c r="U85" s="21"/>
       <x:c r="V85" s="21"/>
-      <x:c r="W85" s="18"/>
-      <x:c r="X85" s="18"/>
-      <x:c r="Y85" s="18"/>
-      <x:c r="Z85" s="18"/>
+      <x:c r="W85" s="21"/>
+      <x:c r="X85" s="21"/>
+      <x:c r="Y85" s="21"/>
+      <x:c r="Z85" s="21"/>
       <x:c r="AA85" s="18"/>
+      <x:c r="AB85" s="18"/>
+      <x:c r="AC85" s="18"/>
+      <x:c r="AD85" s="18"/>
+      <x:c r="AE85" s="18"/>
     </x:row>
     <x:row r="86">
       <x:c r="A86" s="18"/>
@@ -3054,15 +3414,19 @@
       <x:c r="P86" s="18"/>
       <x:c r="Q86" s="18"/>
       <x:c r="R86" s="18"/>
-      <x:c r="S86" s="18"/>
-      <x:c r="T86" s="18"/>
+      <x:c r="S86" s="21"/>
+      <x:c r="T86" s="21"/>
       <x:c r="U86" s="21"/>
       <x:c r="V86" s="21"/>
-      <x:c r="W86" s="18"/>
-      <x:c r="X86" s="18"/>
-      <x:c r="Y86" s="18"/>
-      <x:c r="Z86" s="18"/>
+      <x:c r="W86" s="21"/>
+      <x:c r="X86" s="21"/>
+      <x:c r="Y86" s="21"/>
+      <x:c r="Z86" s="21"/>
       <x:c r="AA86" s="18"/>
+      <x:c r="AB86" s="18"/>
+      <x:c r="AC86" s="18"/>
+      <x:c r="AD86" s="18"/>
+      <x:c r="AE86" s="18"/>
     </x:row>
     <x:row r="87">
       <x:c r="A87" s="18"/>
@@ -3083,15 +3447,19 @@
       <x:c r="P87" s="18"/>
       <x:c r="Q87" s="18"/>
       <x:c r="R87" s="18"/>
-      <x:c r="S87" s="18"/>
-      <x:c r="T87" s="18"/>
+      <x:c r="S87" s="21"/>
+      <x:c r="T87" s="21"/>
       <x:c r="U87" s="21"/>
       <x:c r="V87" s="21"/>
-      <x:c r="W87" s="18"/>
-      <x:c r="X87" s="18"/>
-      <x:c r="Y87" s="18"/>
-      <x:c r="Z87" s="18"/>
+      <x:c r="W87" s="21"/>
+      <x:c r="X87" s="21"/>
+      <x:c r="Y87" s="21"/>
+      <x:c r="Z87" s="21"/>
       <x:c r="AA87" s="18"/>
+      <x:c r="AB87" s="18"/>
+      <x:c r="AC87" s="18"/>
+      <x:c r="AD87" s="18"/>
+      <x:c r="AE87" s="18"/>
     </x:row>
     <x:row r="88">
       <x:c r="A88" s="18"/>
@@ -3112,15 +3480,19 @@
       <x:c r="P88" s="18"/>
       <x:c r="Q88" s="18"/>
       <x:c r="R88" s="18"/>
-      <x:c r="S88" s="18"/>
-      <x:c r="T88" s="18"/>
+      <x:c r="S88" s="21"/>
+      <x:c r="T88" s="21"/>
       <x:c r="U88" s="21"/>
       <x:c r="V88" s="21"/>
-      <x:c r="W88" s="18"/>
-      <x:c r="X88" s="18"/>
-      <x:c r="Y88" s="18"/>
-      <x:c r="Z88" s="18"/>
+      <x:c r="W88" s="21"/>
+      <x:c r="X88" s="21"/>
+      <x:c r="Y88" s="21"/>
+      <x:c r="Z88" s="21"/>
       <x:c r="AA88" s="18"/>
+      <x:c r="AB88" s="18"/>
+      <x:c r="AC88" s="18"/>
+      <x:c r="AD88" s="18"/>
+      <x:c r="AE88" s="18"/>
     </x:row>
     <x:row r="89">
       <x:c r="A89" s="18"/>
@@ -3141,15 +3513,19 @@
       <x:c r="P89" s="18"/>
       <x:c r="Q89" s="18"/>
       <x:c r="R89" s="18"/>
-      <x:c r="S89" s="18"/>
-      <x:c r="T89" s="18"/>
+      <x:c r="S89" s="21"/>
+      <x:c r="T89" s="21"/>
       <x:c r="U89" s="21"/>
       <x:c r="V89" s="21"/>
-      <x:c r="W89" s="18"/>
-      <x:c r="X89" s="18"/>
-      <x:c r="Y89" s="18"/>
-      <x:c r="Z89" s="18"/>
+      <x:c r="W89" s="21"/>
+      <x:c r="X89" s="21"/>
+      <x:c r="Y89" s="21"/>
+      <x:c r="Z89" s="21"/>
       <x:c r="AA89" s="18"/>
+      <x:c r="AB89" s="18"/>
+      <x:c r="AC89" s="18"/>
+      <x:c r="AD89" s="18"/>
+      <x:c r="AE89" s="18"/>
     </x:row>
     <x:row r="90">
       <x:c r="A90" s="18"/>
@@ -3170,15 +3546,19 @@
       <x:c r="P90" s="18"/>
       <x:c r="Q90" s="18"/>
       <x:c r="R90" s="18"/>
-      <x:c r="S90" s="18"/>
-      <x:c r="T90" s="18"/>
+      <x:c r="S90" s="21"/>
+      <x:c r="T90" s="21"/>
       <x:c r="U90" s="21"/>
       <x:c r="V90" s="21"/>
-      <x:c r="W90" s="18"/>
-      <x:c r="X90" s="18"/>
-      <x:c r="Y90" s="18"/>
-      <x:c r="Z90" s="18"/>
+      <x:c r="W90" s="21"/>
+      <x:c r="X90" s="21"/>
+      <x:c r="Y90" s="21"/>
+      <x:c r="Z90" s="21"/>
       <x:c r="AA90" s="18"/>
+      <x:c r="AB90" s="18"/>
+      <x:c r="AC90" s="18"/>
+      <x:c r="AD90" s="18"/>
+      <x:c r="AE90" s="18"/>
     </x:row>
     <x:row r="91">
       <x:c r="A91" s="18"/>
@@ -3199,15 +3579,19 @@
       <x:c r="P91" s="18"/>
       <x:c r="Q91" s="18"/>
       <x:c r="R91" s="18"/>
-      <x:c r="S91" s="18"/>
-      <x:c r="T91" s="18"/>
+      <x:c r="S91" s="21"/>
+      <x:c r="T91" s="21"/>
       <x:c r="U91" s="21"/>
       <x:c r="V91" s="21"/>
-      <x:c r="W91" s="18"/>
-      <x:c r="X91" s="18"/>
-      <x:c r="Y91" s="18"/>
-      <x:c r="Z91" s="18"/>
+      <x:c r="W91" s="21"/>
+      <x:c r="X91" s="21"/>
+      <x:c r="Y91" s="21"/>
+      <x:c r="Z91" s="21"/>
       <x:c r="AA91" s="18"/>
+      <x:c r="AB91" s="18"/>
+      <x:c r="AC91" s="18"/>
+      <x:c r="AD91" s="18"/>
+      <x:c r="AE91" s="18"/>
     </x:row>
     <x:row r="92">
       <x:c r="A92" s="18"/>
@@ -3228,15 +3612,19 @@
       <x:c r="P92" s="18"/>
       <x:c r="Q92" s="18"/>
       <x:c r="R92" s="18"/>
-      <x:c r="S92" s="18"/>
-      <x:c r="T92" s="18"/>
+      <x:c r="S92" s="21"/>
+      <x:c r="T92" s="21"/>
       <x:c r="U92" s="21"/>
       <x:c r="V92" s="21"/>
-      <x:c r="W92" s="18"/>
-      <x:c r="X92" s="18"/>
-      <x:c r="Y92" s="18"/>
-      <x:c r="Z92" s="18"/>
+      <x:c r="W92" s="21"/>
+      <x:c r="X92" s="21"/>
+      <x:c r="Y92" s="21"/>
+      <x:c r="Z92" s="21"/>
       <x:c r="AA92" s="18"/>
+      <x:c r="AB92" s="18"/>
+      <x:c r="AC92" s="18"/>
+      <x:c r="AD92" s="18"/>
+      <x:c r="AE92" s="18"/>
     </x:row>
     <x:row r="93">
       <x:c r="A93" s="18"/>
@@ -3257,15 +3645,19 @@
       <x:c r="P93" s="18"/>
       <x:c r="Q93" s="18"/>
       <x:c r="R93" s="18"/>
-      <x:c r="S93" s="18"/>
-      <x:c r="T93" s="18"/>
+      <x:c r="S93" s="21"/>
+      <x:c r="T93" s="21"/>
       <x:c r="U93" s="21"/>
       <x:c r="V93" s="21"/>
-      <x:c r="W93" s="18"/>
-      <x:c r="X93" s="18"/>
-      <x:c r="Y93" s="18"/>
-      <x:c r="Z93" s="18"/>
+      <x:c r="W93" s="21"/>
+      <x:c r="X93" s="21"/>
+      <x:c r="Y93" s="21"/>
+      <x:c r="Z93" s="21"/>
       <x:c r="AA93" s="18"/>
+      <x:c r="AB93" s="18"/>
+      <x:c r="AC93" s="18"/>
+      <x:c r="AD93" s="18"/>
+      <x:c r="AE93" s="18"/>
     </x:row>
     <x:row r="94">
       <x:c r="A94" s="18"/>
@@ -3286,15 +3678,19 @@
       <x:c r="P94" s="18"/>
       <x:c r="Q94" s="18"/>
       <x:c r="R94" s="18"/>
-      <x:c r="S94" s="18"/>
-      <x:c r="T94" s="18"/>
+      <x:c r="S94" s="21"/>
+      <x:c r="T94" s="21"/>
       <x:c r="U94" s="21"/>
       <x:c r="V94" s="21"/>
-      <x:c r="W94" s="18"/>
-      <x:c r="X94" s="18"/>
-      <x:c r="Y94" s="18"/>
-      <x:c r="Z94" s="18"/>
+      <x:c r="W94" s="21"/>
+      <x:c r="X94" s="21"/>
+      <x:c r="Y94" s="21"/>
+      <x:c r="Z94" s="21"/>
       <x:c r="AA94" s="18"/>
+      <x:c r="AB94" s="18"/>
+      <x:c r="AC94" s="18"/>
+      <x:c r="AD94" s="18"/>
+      <x:c r="AE94" s="18"/>
     </x:row>
     <x:row r="95">
       <x:c r="A95" s="18"/>
@@ -3315,15 +3711,19 @@
       <x:c r="P95" s="18"/>
       <x:c r="Q95" s="18"/>
       <x:c r="R95" s="18"/>
-      <x:c r="S95" s="18"/>
-      <x:c r="T95" s="18"/>
+      <x:c r="S95" s="21"/>
+      <x:c r="T95" s="21"/>
       <x:c r="U95" s="21"/>
       <x:c r="V95" s="21"/>
-      <x:c r="W95" s="18"/>
-      <x:c r="X95" s="18"/>
-      <x:c r="Y95" s="18"/>
-      <x:c r="Z95" s="18"/>
+      <x:c r="W95" s="21"/>
+      <x:c r="X95" s="21"/>
+      <x:c r="Y95" s="21"/>
+      <x:c r="Z95" s="21"/>
       <x:c r="AA95" s="18"/>
+      <x:c r="AB95" s="18"/>
+      <x:c r="AC95" s="18"/>
+      <x:c r="AD95" s="18"/>
+      <x:c r="AE95" s="18"/>
     </x:row>
     <x:row r="96">
       <x:c r="A96" s="18"/>
@@ -3344,15 +3744,19 @@
       <x:c r="P96" s="18"/>
       <x:c r="Q96" s="18"/>
       <x:c r="R96" s="18"/>
-      <x:c r="S96" s="18"/>
-      <x:c r="T96" s="18"/>
+      <x:c r="S96" s="21"/>
+      <x:c r="T96" s="21"/>
       <x:c r="U96" s="21"/>
       <x:c r="V96" s="21"/>
-      <x:c r="W96" s="18"/>
-      <x:c r="X96" s="18"/>
-      <x:c r="Y96" s="18"/>
-      <x:c r="Z96" s="18"/>
+      <x:c r="W96" s="21"/>
+      <x:c r="X96" s="21"/>
+      <x:c r="Y96" s="21"/>
+      <x:c r="Z96" s="21"/>
       <x:c r="AA96" s="18"/>
+      <x:c r="AB96" s="18"/>
+      <x:c r="AC96" s="18"/>
+      <x:c r="AD96" s="18"/>
+      <x:c r="AE96" s="18"/>
     </x:row>
     <x:row r="97">
       <x:c r="A97" s="18"/>
@@ -3373,15 +3777,19 @@
       <x:c r="P97" s="18"/>
       <x:c r="Q97" s="18"/>
       <x:c r="R97" s="18"/>
-      <x:c r="S97" s="18"/>
-      <x:c r="T97" s="18"/>
+      <x:c r="S97" s="21"/>
+      <x:c r="T97" s="21"/>
       <x:c r="U97" s="21"/>
       <x:c r="V97" s="21"/>
-      <x:c r="W97" s="18"/>
-      <x:c r="X97" s="18"/>
-      <x:c r="Y97" s="18"/>
-      <x:c r="Z97" s="18"/>
+      <x:c r="W97" s="21"/>
+      <x:c r="X97" s="21"/>
+      <x:c r="Y97" s="21"/>
+      <x:c r="Z97" s="21"/>
       <x:c r="AA97" s="18"/>
+      <x:c r="AB97" s="18"/>
+      <x:c r="AC97" s="18"/>
+      <x:c r="AD97" s="18"/>
+      <x:c r="AE97" s="18"/>
     </x:row>
     <x:row r="98">
       <x:c r="A98" s="18"/>
@@ -3402,15 +3810,19 @@
       <x:c r="P98" s="18"/>
       <x:c r="Q98" s="18"/>
       <x:c r="R98" s="18"/>
-      <x:c r="S98" s="18"/>
-      <x:c r="T98" s="18"/>
+      <x:c r="S98" s="21"/>
+      <x:c r="T98" s="21"/>
       <x:c r="U98" s="21"/>
       <x:c r="V98" s="21"/>
-      <x:c r="W98" s="18"/>
-      <x:c r="X98" s="18"/>
-      <x:c r="Y98" s="18"/>
-      <x:c r="Z98" s="18"/>
+      <x:c r="W98" s="21"/>
+      <x:c r="X98" s="21"/>
+      <x:c r="Y98" s="21"/>
+      <x:c r="Z98" s="21"/>
       <x:c r="AA98" s="18"/>
+      <x:c r="AB98" s="18"/>
+      <x:c r="AC98" s="18"/>
+      <x:c r="AD98" s="18"/>
+      <x:c r="AE98" s="18"/>
     </x:row>
     <x:row r="99">
       <x:c r="A99" s="18"/>
@@ -3431,15 +3843,19 @@
       <x:c r="P99" s="18"/>
       <x:c r="Q99" s="18"/>
       <x:c r="R99" s="18"/>
-      <x:c r="S99" s="18"/>
-      <x:c r="T99" s="18"/>
+      <x:c r="S99" s="21"/>
+      <x:c r="T99" s="21"/>
       <x:c r="U99" s="21"/>
       <x:c r="V99" s="21"/>
-      <x:c r="W99" s="18"/>
-      <x:c r="X99" s="18"/>
-      <x:c r="Y99" s="18"/>
-      <x:c r="Z99" s="18"/>
+      <x:c r="W99" s="21"/>
+      <x:c r="X99" s="21"/>
+      <x:c r="Y99" s="21"/>
+      <x:c r="Z99" s="21"/>
       <x:c r="AA99" s="18"/>
+      <x:c r="AB99" s="18"/>
+      <x:c r="AC99" s="18"/>
+      <x:c r="AD99" s="18"/>
+      <x:c r="AE99" s="18"/>
     </x:row>
     <x:row r="100">
       <x:c r="A100" s="18"/>
@@ -3460,15 +3876,19 @@
       <x:c r="P100" s="18"/>
       <x:c r="Q100" s="18"/>
       <x:c r="R100" s="18"/>
-      <x:c r="S100" s="18"/>
-      <x:c r="T100" s="18"/>
+      <x:c r="S100" s="21"/>
+      <x:c r="T100" s="21"/>
       <x:c r="U100" s="21"/>
       <x:c r="V100" s="21"/>
-      <x:c r="W100" s="18"/>
-      <x:c r="X100" s="18"/>
-      <x:c r="Y100" s="18"/>
-      <x:c r="Z100" s="18"/>
+      <x:c r="W100" s="21"/>
+      <x:c r="X100" s="21"/>
+      <x:c r="Y100" s="21"/>
+      <x:c r="Z100" s="21"/>
       <x:c r="AA100" s="18"/>
+      <x:c r="AB100" s="18"/>
+      <x:c r="AC100" s="18"/>
+      <x:c r="AD100" s="18"/>
+      <x:c r="AE100" s="18"/>
     </x:row>
     <x:row r="101">
       <x:c r="A101" s="22"/>
@@ -3489,15 +3909,19 @@
       <x:c r="P101" s="22"/>
       <x:c r="Q101" s="22"/>
       <x:c r="R101" s="22"/>
-      <x:c r="S101" s="22"/>
-      <x:c r="T101" s="22"/>
+      <x:c r="S101" s="25"/>
+      <x:c r="T101" s="25"/>
       <x:c r="U101" s="25"/>
       <x:c r="V101" s="25"/>
-      <x:c r="W101" s="22"/>
-      <x:c r="X101" s="22"/>
-      <x:c r="Y101" s="22"/>
-      <x:c r="Z101" s="22"/>
+      <x:c r="W101" s="25"/>
+      <x:c r="X101" s="25"/>
+      <x:c r="Y101" s="25"/>
+      <x:c r="Z101" s="25"/>
       <x:c r="AA101" s="22"/>
+      <x:c r="AB101" s="22"/>
+      <x:c r="AC101" s="22"/>
+      <x:c r="AD101" s="22"/>
+      <x:c r="AE101" s="22"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="3">
@@ -3507,7 +3931,7 @@
     <x:dataValidation type="list" sqref="L2:L101">
       <x:formula1>"in_stock,out_of_stock,pre_order"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="AA2:AA101">
+    <x:dataValidation type="list" sqref="AE2:AE101">
       <x:formula1>"draft"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -3660,7 +4084,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B9" s="37" t="str">
-        <x:v>Use Product Dimensions and Package Dimensions as readable text, including units.</x:v>
+        <x:v>Enter all length, width and height values as numbers in cm; enter net and gross weight as numbers in kg.</x:v>
       </x:c>
     </x:row>
     <x:row r="10">

</xml_diff>